<commit_message>
Update berita 2026-08-09 18:26 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -762,8 +762,431 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pramusim: Arsenal tunduk 2-3 dari Borussia Dortmund di Emirates Cup</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 01:08:30 +0700</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Arsenal ditundukkan Borussia Dortmund 2-3 dalam laga pramusim bertajuk Emirates Cup di Stadion Emirates, ...</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686948/pramusim-arsenal-tunduk-2-3-dari-borussia-dortmund-di-emirates-cup</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000043587.jpg</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sambut HUT RI, PB Jatma Aswaja gelar zikir kebangsaan di Istiqlal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 01:06:37 +0700</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ANTARA - Pengurus Besar Jam'iyah Ahlith Thariqah Al Mutabaroh Ahlussunnah wal Jama'ah (PB Jatma Aswaja) menggelar Zikir ...</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686945/sambut-hut-ri-pb-jatma-aswaja-gelar-zikir-kebangsaan-di-istiqlal</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_SAMBUT-HUT-RI-PB-JATMA-ASWAJA-GELAR-ZIKIR-KEBANGSAAN-DI-ISTIQLAL.jpg</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pramusim: Liverpool takluk 2-3 dari AS Monaco di Anfield</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 00:44:41 +0700</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Liverpool menelan kekalahan 2-3 dari AS Monaco dalam laga pramusim 2026 di Stadion Anfield, Inggris pada Minggu malam ...</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686944/pramusim-liverpool-takluk-2-3-dari-as-monaco-di-anfield</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000043577.jpg</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PSSI minta publik tak hujat pemain terkait Piala AFF</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 00:25:02 +0700</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sekretaris Jendral Persatuan Sepak Bola Seluruh Indonesia (PSSI), Yunus Nusi meminta publik tidak menempatkan pemain ...</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686941/pssi-minta-publik-tak-hujat-pemain-terkait-piala-aff</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/10/IMG_8030.jpeg</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Yayasan Sekolah di Jaksel Ungkap Eks Pemilik Utang ke Bank Buat Lapangan Padel</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 00:59:01 +0700</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Mantan pemilik yayasan IWD, diduga menggunakan yayasan untuk kepentingan pribadi dan menyimpan senjata. Salah satunya membuat lapangan padel.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611448/yayasan-sekolah-di-jaksel-ungkap-eks-pemilik-utang-ke-bank-buat-lapangan-padel</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kuasa-hukum-yayasan-sekolah-swasta-di-jaksel-hermawanto-menjelaskan-soal-temuan-ratusan-senjata-1786150520216_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pasutri di Mojokerto Syok Tiba-tiba di Rumahnya Ada Kuburan Bayi</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 00:28:22 +0700</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Enggran Eko Budianto</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Pasangan di Mojokerto temukan kuburan bayi di pekarangan rumah. Penemuan ini terjadi setelah pulang dari Gresik.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611416/pasutri-di-mojokerto-syok-tiba-tiba-di-rumahnya-ada-kuburan-bayi</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/bayi-dikubur-di-sebelah-sumur-rumah-warga-mojokerto-1786280765341_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Buntut Putusan MA soal Kasus Timah, Pakar Minta Pengadilan Konsisten Gunakan Audit BPK</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 00:55:21 +0700</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Huda menjelaskan kewenangan BPK menghitung kerugian keuangan negara sesuai dengan amanat Peraturan Mahkamah Agung , putusan MK hingga UU</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866111/buntut-putusan-ma-soal-kasus-timah-pakar-minta-pengadilan-konsisten-gunakan-audit-bpk</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8HGoys_ssFVqS7iCYXN7nF8pZQU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sidang-korupsi-PT-Timah-dengan-terdakwa-Harvey-Moeis-dkk-di-Pengadilan-Tipikor-Jakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tingkatkan Mutu Dokter Indonesia, Kampus Swasta Gandeng UI, Dosen Pakar Bisa Ikut Mengajar</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 00:47:33 +0700</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Kerja sama ini juga mencakup pendampingan dalam pengembangan kurikulum, sistem pembelajaran hingga peningkatan mutu pendidikan</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866110/tingkatkan-mutu-dokter-indonesia-kampus-swasta-gandeng-ui-dosen-pakar-bisa-ikut-mengajar</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/KOteNA0RNnet3qmGm8GTnWBegtY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kampus-Universitas-Indonesia-di-Depok-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Detik-detik Mencekam Pegawai Tutup Lapak di Tengah Kebakaran Mal Nipah Makassar</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 00:29:40 +0700</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Beredar di media sosial dan menjadi perbincangan warga setelah video memperihatkan kondisi mencekam saat kebakaran di Mal Nipah, Makassar</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866109/detik-detik-mencekam-pegawai-tutup-lapak-di-tengah-kebakaran-mal-nipah-makassar</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/agcpkJPhibG2HYwEc7hsXBKRlyg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Seorang-pria-menjadi-sorotan-di-tengah-kebakaran-di-Mal-Nipah-Makassar.jpg</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I7"/>
+  <autoFilter ref="A1:I16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 19:27 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1185,8 +1185,243 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Menko Pangan minta doa agar semua program pemerintah berjalan optimal</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 01:42:58 +0700</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Pangan Zulkifli Hasan meminta doa dan dukungan masyarakat, utamanya dari warga Jatma Aswaja, ...</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686952/menko-pangan-minta-doa-agar-semua-program-pemerintah-berjalan-optimal</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000177340.jpg</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>20 Bulan Pemerintahan, Zulhas Akui Tak Semua Program Pemerintah Berhasil: Ada yang Belum</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 02:01:49 +0700</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Zulkifli Hasan atau Zulhas menyebut hampir 2 tahun ada program yang berhasil dan belum, salah satunya MBG</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866114/20-bulan-pemerintahan-zulhas-akui-tak-semua-program-pemerintah-berhasil-ada-yang-belum</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/BNe0CId_2a99tvpmY4ZZwt1N04U=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/rgizi-gratis-MBG-di-Gedung-Gra.jpg</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Prabowo Minta Pertamina Pangkas Layer dan Anak Cucu Perusahaan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 01:47:06 +0700</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Prabowo dalam pertemuan di Kediaman Hambalang meminta Simon untuk memangkas anak perusahaan Pertamina</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866113/prabowo-minta-pertamina-pangkas-layer-dan-anak-cucu-perusahaan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/MackvCUZGbNLLnq3IkwyNkR7jhE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Presiden-Prabowo-Subianto-menerima-Direktur-Utama-Pertamina-Simon-Mantiri.jpg</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Zulhas Ungkap Penyebab Prabowo Tak Hadiri Zikir Kebangsaan, Titip Salam dan Permintaan Maaf</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 01:33:31 +0700</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Zulkifli Hasan menyampaikan salam dari Presiden Prabowo kepada para peserta Zikir Kebangsaan di Masjid Istiqlal</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866112/zulhas-ungkap-penyebab-prabowo-tak-hadiri-zikir-kebangsaan-titip-salam-dan-permintaan-maaf</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/c0QGsg2O8JT9_f3rBKREvX_aY4k=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ZULKIFLI-HASAN-89097.jpg</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Hype</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Denny Sumargo Sebut Anak dan Istrinya Ikut Dirundung karena Podcast Bareng Sarwendah dan Ruben Onsu</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 02:27:25 +0700</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Denny Sumargo akui dampak podcast Sarwendah-Ruben Onsu menyerang keluarga, bahkan istri &amp; anaknya dibully netizen. Densu berharap semua pihak bisa tenang.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/hype/read/2026/08/09/235845166/denny-sumargo-sebut-anak-dan-istrinya-ikut-dirundung-karena-podcast-bareng</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/D6w0YmIxiwP9_2Y51yV5iJn24mM=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c8191ee571.png,0,-0,1)/data/photo/2026/08/09/6a7873c4d8031.jpg</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I16"/>
+  <autoFilter ref="A1:I21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 20:21 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1420,8 +1420,102 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Menhut: Pemadaman kebakaran Bromo andalkan "water bombing"</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 02:39:38 +0700</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ANTARA - ‎Menteri Kehutanan Raja Juli Antoni meninjau langsung penanganan kebakaran hutan dan lahan di kawasan ...</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686937/menhut-pemadaman-kebakaran-bromo-andalkan-water-bombing</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_MENHUT-PEMADAMAN-KEBAKARAN-BROMO-ANDALKAN-22WATER-BOMBING-22.jpg</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Prabowo Panggil Dirut Pertamina ke Hambalang, Ini yang Dibahas</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 02:27:47 +0700</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Kadek Melda Luxiana</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo memanggil Dirut Pertamina ke Hambalang. Apa saja yang dibahas?</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611458/prabowo-panggil-dirut-pertamina-ke-hambalang-ini-yang-dibahas</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/prabowo-panggil-dirut-pertamina-ke-hambalang-dok-instagram-1786303642467_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I21"/>
+  <autoFilter ref="A1:I23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 21:24 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1514,8 +1514,102 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Menhut Tinjau Penanganan Kebakaran Bromo, Maksimalkan Penggunaan Water Bombing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 03:39:38 +0700</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>M rofiq</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Menteri Kehutanan Raja Juli Antoni meninjau penanganan kebakaran hutan di Gunung Bromo. Helikopter water bombing digunakan maksimal untuk padamkan api.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611464/menhut-tinjau-penanganan-kebakaran-bromo-maksimalkan-penggunaan-water-bombing</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/menteri-kehutanan-ri-raja-juli-antoni-1786272285884_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>MTQ XXXIV Kalbar di Kayong Utara Resmi Berakhir, Kubu Raya Raih Juara Umum</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 03:11:09 +0700</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MTQ XXXIV Tingkat Provinsi Kalbar Tahun 2026 di Sukadana, Kabupaten Kayong Utara resmi ditutup, Kubu Raya juara umum</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866115/mtq-xxxiv-kalbar-di-kayong-utara-resmi-berakhir-kubu-raya-raih-juara-umum</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/-7mLvM1yZQMwrBzZ6WIrr0Lwydw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Penyelenggaraan-MTQ-XXXIV-Kalbar-resmi-ditutup.jpg</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I23"/>
+  <autoFilter ref="A1:I25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 23:24 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -2266,8 +2266,1136 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Humaniora kemarin, kirab Merah Putih hingga zikir akbar di Istiqlal</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 06:04:16 +0700</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Terdapat sejumlah berita humaniora menarik yang terjadi pada Minggu (9/8) dan bisa dibaca kembali pada pagi ini untuk ...</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686983/humaniora-kemarin-kirab-merah-putih-hingga-zikir-akbar-di-istiqlal</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/12/26/foto-terbaik-2025-2696548.jpg</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Satgas PRR Kemendagri tinjau proyek PSN di Nagan Raya Aceh</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 06:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ANTARA - Tim Satgas Percepatan Rehabilitasi dan Rekonstruksi (PRR) Kementerian Dalam Negeri meninjau perkembangan ...</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686929/satgas-prr-kemendagri-tinjau-proyek-psn-di-nagan-raya-aceh</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_SATGAS-PRR-KEMENDAGRI-TINJAU-PROYEK-PSN-DI-NAGAN-RAYA-ACEH.jpg</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Satelit Lampung-1 untuk kembangkan pertanian</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 06:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Satelit Lampung-1 diluncurkan ke orbit menggunakan roket pengangkut Smart Dragon-3 dari Shandong, China, Rabu (5/8). ...</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5686864/satelit-lampung-1-untuk-kembangkan-pertanian</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/20260809-Satelit-Lampung-1-untuk-kembangkan-pertanian.jpg</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain datangkan Lucas Digne dari Aston Villa</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:57:17 +0700</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain (PSG) resmi mendatangkan bek kiri timnas Prancis, Lucas Digne dari Aston Villa pada bursa transfer ...</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686981/paris-saint-germain-datangkan-lucas-digne-dari-aston-villa</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2022/01/22/2022-01-22T131523Z_577296983_UP1EI1M10TKFY_RTRMADP_3_SOCCER-ENGLAND-EVE-AVA-REPORT.jpg</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Senin, BMKG: Mayoritas wilayah RI berawan hingga hujan ringan</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:56:55 +0700</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) memprakirakan cuaca di mayoritas wilayah Indonesia didominasi ...</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686977/senin-bmkg-mayoritas-wilayah-ri-berawan-hingga-hujan-ringan</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/04/23/IMG_20241219_140043.jpg</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>DKI kemarin, JIS jadi kandang Persija hingga Tj rute Senayan-Ancol</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:52:47 +0700</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Sejumlah berita di DKI Jakarta pada Minggu (9/8) masih menarik untuk disimak hari ini mulai dari Transjakarta buka rute ...</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686975/dki-kemarin-jis-jadi-kandang-persija-hingga-tj-rute-senayan-ancol</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/22/RESIZED-WhatsApp-Image-2026-06-22-at-18.42.28.jpg</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Kriminal kemarin, temuan senjata hingga perusak kabel optik ditangkap</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:50:27 +0700</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Sejumlah berita kriminal di wilayah Jakarta pada Minggu (9/8) yang masih layak dibaca hari ini antara lain polisi ...</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686971/kriminal-kemarin-temuan-senjata-hingga-perusak-kabel-optik-ditangkap</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001016025.jpg</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Como 1907 boyong Trevoh Chalobah dari Chelsea</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:49:12 +0700</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Klub Liga Italia, Como 1907 resmi memboyong bek timnas Inggris, Trevoh Chalobah dari Chelsea pada bursa transfer musim ...</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686969/como-1907-boyong-trevoh-chalobah-dari-chelsea</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000043632.jpg</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Cuaca Jakarta diprakirakan akan cerah berawan pada Senin</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:45:30 +0700</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) memprakirakan cuaca di seluruh wilayah DKI jakarta akan cerah ...</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686967/cuaca-jakarta-diprakirakan-akan-cerah-berawan-pada-senin</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/19/IMG_20260719_000858.jpg</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>PD soal Isu Reshuffle: Siapa dan Dari Mana Menterinya, Sepenuhnya Presiden</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:19:12 +0700</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Azhar Bagas Ramadhan</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Partai Demokrat menegaskan reshuffle kabinet adalah hak prerogatif Presiden. Mereka mendukung pemilihan menteri berdasarkan kemampuan, bukan asal partai.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611470/pd-soal-isu-reshuffle-siapa-dan-dari-mana-menterinya-sepenuhnya-presiden</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/09/16/sekjen-dpp-partai-demokrat-herman-khaeron-usai-menghadiri-rakerda-dpd-demokrat-bali-di-denpasar-selasa-1692025-1758033321170_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Sengketa Ahli Waris Lina Jubaedah Masuk Kasasi, Teddy Pardiyana Pilih Tenang</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 06:03:38 +0700</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Sengketa ahli waris Lina Jubaedah berlanjut ke tahap kasasi di Mahkamah Agung. Teddy Pardiyana tetap tenang dan terbuka untuk mediasi dengan Rizky Febian.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8611447/sengketa-ahli-waris-lina-jubaedah-masuk-kasasi-teddy-pardiyana-pilih-tenang</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/30/rizky-febian-1785413128625_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Netanyahu Tolak 15 Poin Rencana Damai Gaza Usulan Board of Peace Trump</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 06:05:37 +0700</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Tolak usulan Board of Peace, Netanyahu ogah tarik militernya dari Jalur Gaza sebelum Hamas serahkan senjata secara penuh.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810055257-120-1390397/netanyahu-tolak-15-poin-rencana-damai-gaza-usulan-board-of-peace-trump</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/10/12/pm-israel-benjamin-netanyahu-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Kanada Usir 3 Ribu Warga India hingga Israel Mau Serang Iran Tanpa AS</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:45:50 +0700</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Lebih dari tiga ribu WN India dipulangkan dari Kanada sampai Israel mau serang Iran sepihak jika perang AS-Teheran berakhir.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810053224-134-1390395/kanada-usir-3-ribu-warga-india-hingga-israel-mau-serang-iran-tanpa-as</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/04/19/ilustrasi-konflik-israel-iran_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Tragedi Maut Ajang Balap Drag Race Kotamobagu: Mobil Pembalap Tabrak Penonton, 7 Tewas, 9 Luka-luka</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 06:04:31 +0700</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Mobil peserta balap di Kotamobagu Sulut tabrak penonton akibatkan 7 korban tewas dan 9 luka-luka pada Minggu (9/8/2026).</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866125/tragedi-maut-ajang-balap-drag-race-kotamobagu-mobil-pembalap-tabrak-penonton-7-tewas-9-luka-luka</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/sdtdONAMpybx_mtcJWcZYFFaWCI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/drage-race-kotamogaku-kecelakaan-tabrak-penonton.jpg</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Daftar Penghargaan Individu SEA V Cup 2026 Putri Leg 2: Indah Guretno Best Libero, Thailand Dominan</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:47:05 +0700</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Indah Guretno menjadi satu-satunya wakil Indonesia yang menyabet penghargaan SEA V Cup 2026 putri leg 2 sebagai best libero.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866124/daftar-penghargaan-individu-sea-v-cup-2026-putri-leg-2-indah-guretno-best-libero-thailand-dominan</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ji5jh_awPmeoo7bKdWFIChFnymU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pemain-Timnas-Voli-Putri-Indonesia-melakukan-perayaan-setelah-mencetak-poin-saat.jpg</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Ramai Warga Minta Refund Tiket Kunjungan Bromo di Komentar Unggahan Menhut Raja Juli</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:37:38 +0700</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Penutupan Bromo akibat karhutla membuat calon wisatawan ramai menanyakan mekanisme refund tiket di unggahan Menhut Raja Juli.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866123/ramai-warga-minta-refund-tiket-kunjungan-bromo-di-komentar-unggahan-menhut-raja-juli</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/L5V5p-yUMV9CORbJGZWh8Kcyvtc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Raja-Juli-Antoni-mengunjungi-Kawasan-Hutan-Dengan-Tujuan-Khusus-KHDTK-Tabo-Tabo.jpg</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Hasil MotoGP Inggris 2026 Tak Memuaskan, Marc Marquez Pilih Kritik Diri Sendiri</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:33:59 +0700</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Marc Marquez gagal menunjukkan performa terbaiknya di MotoGP Inggris 2026 dan menyebut motor bukan menjadi faktor masalah</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866122/hasil-motogp-inggris-2026-tak-memuaskan-marc-marquez-pilih-kritik-diri-sendiri</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/_zd0Xjtfz40QQD41FEpzeehTLvQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Marc-Marquez-dan-Alex-Marquez-MotoGP-Inggris-2025.jpg</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Denny Sumargo Sebut Keluarga Kena Hujat Netizen usai Podcast Bareng Sarwendah</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:24:39 +0700</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Denny Sumargo menyebut keluarganya, terutama sang istri, Olivia Allan dan anaknya menjadi sasaran hujatan netizen buntut podcast bersama Sarwendah.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866121/denny-sumargo-sebut-keluarga-kena-hujat-netizen-usai-podcast-bareng-sarwendah</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ik23waLzTdDpWPovuqWu3mZdce4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Denny-Sumargo-1-03082026.jpg</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Sejak Kapan Bayi Boleh Pakai Skincare? Ini Penjelasan Dokter</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:12:23 +0700</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>dr. HANS menjelaskan bahwa bayi boleh memakai skincare sejak bayi baru lahir jika formula produknya memang untuk kulit sensitif.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866120/sejak-kapan-bayi-boleh-pakai-skincare-ini-penjelasan-dokter</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/umKVBJF65IbfXBVjy48cT4Yds4Q=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/teknik-pijat-lembut-pada-bayi-untuk-meredakan-gejala-batuk-dan-pilek.jpg</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Alasan Maarten Paes Cadangan dalam Kemenangan Ajax atas PEC Zwolle, Bukan Gegara Michel Tak Suka</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:07:47 +0700</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Pelatih Ajax, Michel, mengungkapkan alasan di balik keputusannya mainkan Ter Stegen dan mencadangkan Maarten Paes dalam kemenangan atas PEC Zwolle.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866119/alasan-maarten-paes-cadangan-dalam-kemenangan-ajax-atas-pec-zwolle-bukan-gegara-michel-tak-suka</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/2OWvW2i5iEbzDBtJC2ErtaNIvaY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Eskpresi-Maarten-Paes-setelah-menepis-penendang-penalti-FC-Utrecht.jpg</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>BMKG Ungkap Prakiraan Cuaca Jakarta Senin, Ada Wilayah Berawan Tebal</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 06:15:51 +0700</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>BMKG memprakirakan cuaca Jakarta didominasi cerah berawan pada Senin, dengan sejumlah wilayah berawan tebal.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265899/bmkg-ungkap-prakiraan-cuaca-jakarta-senin-ada-wilayah-berawan-tebal</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/3-F2plV7Pg7xWbP2yDN5g6R05rM=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/3453943/original/049969200_1620650232-Jakarta_Cerah.jpg</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Yayasan Bongkar Dugaan Kredit Eks Pemilik Sekolah untuk Lapangan Padel</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 06:15:14 +0700</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Kuasa hukum Yayasan Harapan Ibu Pondok Pinang membantah sejumlah pernyataan pihak mantan ketua yayasan dan mengungkap dugaan penyalahgunaan kewenangan.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265891/yayasan-bongkar-dugaan-kredit-eks-pemilik-sekolah-untuk-lapangan-padel</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/YAVOExu6fnI0Yew1ROoX836YmpQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319668/original/013460500_1786264819-71184.jpg</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Sehari Bersama Caregiver: Nyaris Tak Pernah Pulang dari Rumah Sakit</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 06:00:15 +0700</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Pengalaman merawat sang ibu yang menderita gagal ginjal selama sembilan tahun membentuk Angie menjadi sosok yang terbiasa mendampingi orang sakit.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265029/sehari-bersama-caregiver-nyaris-tak-pernah-pulang-dari-rumah-sakit</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/gG-_zkFKY72s5JWNdtPSRArZzog=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318946/original/065932000_1786172831-DSC00542.jpg</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Beton Drainase Roboh, Dua Pekerja Sempat Terjebak</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 05:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Proses evakuasi berlangsung lebih dari tiga jam, menyebabkan kepadatan lalu lintas.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265890/beton-drainase-roboh-dua-pekerja-sempat-terjebak</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Tvv251YSKPKSeACTE9mQdjtNuwQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319886/original/063438000_1786314490-2819b90b-dc27-4278-a00e-307bca883b52.jpg</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I39"/>
+  <autoFilter ref="A1:I63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 11:45 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$719</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$794</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I719"/>
+  <dimension ref="A1:I794"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -34232,8 +34232,3533 @@
         </is>
       </c>
     </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Mario Aji syukuri hasil GP Inggris</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:39:31 +0700</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>Pembalap Moto2 Mario Aji mensyukuri hasil GP Inggris 2026, Minggu (9/8), ketika menuntaskan balapan di peringkat ke-22, ...</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687912/mario-aji-syukuri-hasil-gp-inggris</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/21/Latihan-pembalap-nasional-Moto2-dan-Moto3-di-Mandalika-210726-AS-8.jpg</t>
+        </is>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Jerman perketat pemulangan migran</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:36:42 +0700</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>Jerman dilaporkan mempertegas sikapnya terkait pemulangan migran dan ingin melanjutkan kembali transfer migran ke ...</t>
+        </is>
+      </c>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687907/jerman-perketat-pemulangan-migran</t>
+        </is>
+      </c>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/08/06/create-antaranews-logo.jpg</t>
+        </is>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Kementan siapkan kapal pengiriman 200 sapi perah demi swasembada susu</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:35:46 +0700</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>Kementerian Pertanian (Kementan) menyiapkan Kapal Motor (KM) Camara Nusantara I untuk mengangkut 200 sapi perah bunting ...</t>
+        </is>
+      </c>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687903/kementan-siapkan-kapal-pengiriman-200-sapi-perah-demi-swasembada-susu</t>
+        </is>
+      </c>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/7AE4ED87-1327-4F74-A776-1B732F18C9F6.jpeg</t>
+        </is>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Menkopolkam minta Kalteng dan Kalbar hentikan izin pembakaran lahan</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:35:13 +0700</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Politik dan Keamanan (Menkopolkam) Djamari Chaniago meminta pemerintah daerah Kalimantan ...</t>
+        </is>
+      </c>
+      <c r="F723" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G723" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687900/menkopolkam-minta-kalteng-dan-kalbar-hentikan-izin-pembakaran-lahan</t>
+        </is>
+      </c>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/20260810_150224.jpg</t>
+        </is>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>PSSI prihatin kritik negatif terhadap Justin Hubner dan keluarganya</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:34:00 +0700</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>Persatuan Sepak Bola Seluruh Indonesia (PSSI) menyatakan prihatin terhadap munculnya kritik negatif terhadap pemain ...</t>
+        </is>
+      </c>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687899/pssi-prihatin-kritik-negatif-terhadap-justin-hubner-dan-keluarganya</t>
+        </is>
+      </c>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/timnas-indonesia-dikalahkan-vietnam-di-piala-aff-2833631.jpg</t>
+        </is>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Pramono Anung: Pemulung Bantargebang didaftarkan BPJS Ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:32:44 +0700</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>ANTARA - Gubernur Jakarta Pramono Anung Wibowo mengungkapkan sebanyak 4.000 pemulung di Tempat Pengolahan Sampah ...</t>
+        </is>
+      </c>
+      <c r="F725" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5687847/pramono-anung-pemulung-bantargebang-didaftarkan-bpjs-ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AYM_RAMONO-ANUNG-PEMULUNG-BANTARGEBANG.jpg</t>
+        </is>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Karhutla meluas, BMKG ungkap mengapa belum bisa laksanakan OMC</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:29:23 +0700</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mengungkapkan Operasi Modifikasi Cuaca (OMC) untuk membantu ...</t>
+        </is>
+      </c>
+      <c r="F726" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687895/karhutla-meluas-bmkg-ungkap-mengapa-belum-bisa-laksanakan-omc</t>
+        </is>
+      </c>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/patroli-kebakaran-hutan-dan-lahan-melalui-udara-di-kalteng-2834369.jpg</t>
+        </is>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Pemkot Ambon gelar lomba Jukulele, sokong kreativitas generasi muda</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:23:51 +0700</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>ANTARA - Wakil Wali kota Ambon Ely Toisuta membuka lomba Jukulele di Taman Budaya kota Ambon, Maluku, Senin ...</t>
+        </is>
+      </c>
+      <c r="F727" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5687656/pemkot-ambon-gelar-lomba-jukulele-sokong-kreativitas-generasi-muda</t>
+        </is>
+      </c>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PEMKOT-AMBON-GELAR-LOMBA-JUKULELE-SOKONG-KREATIVITAS-GENERASI-MUDA_1.jpg</t>
+        </is>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Dekranasda DKI tegaskan karya Nusantara harus hadir di ruang perkotaan</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:20:19 +0700</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>Ketua Dewan Kerajinan Nasional Daerah (Dekranasda) DKI Jakarta Hani Pramono menegaskan karya tradisional dan produk ...</t>
+        </is>
+      </c>
+      <c r="F728" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687889/dekranasda-dki-tegaskan-karya-nusantara-harus-hadir-di-ruang-perkotaan</t>
+        </is>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000835766.jpg</t>
+        </is>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Kejagung periksa tujuh saksi terkait kasus TPPU Febrie Adriansyah</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:16:55 +0700</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>Tim Penyidik Kejaksaan Agung (Tim 9) memeriksa tujuh saksi dalam proses penyidikan kasus dugaan tindak pidana pencucian ...</t>
+        </is>
+      </c>
+      <c r="F729" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687885/kejagung-periksa-tujuh-saksi-terkait-kasus-tppu-febrie-adriansyah</t>
+        </is>
+      </c>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000087297.jpg</t>
+        </is>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Kasus temuan senjata, KPAI terima aduan dari sekolah dan yayasan</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:16:10 +0700</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>Komisi Perlindungan Anak Indonesia (KPAI) menerima pengaduan resmi dari pihak yayasan dan sekolah terkait,  ...</t>
+        </is>
+      </c>
+      <c r="F730" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687881/kasus-temuan-senjata-kpai-terima-aduan-dari-sekolah-dan-yayasan</t>
+        </is>
+      </c>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/tanggapan-pihak-sekolah-terkait-temuan-senjata-di-sekolah-2837852.jpg</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Danpaspampres pimpin gelar kesiapan pasukan rangkaian HUT Ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:14:06 +0700</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>Komandan Pasukan Pengamanan Presiden (Danpaspampres) Mayjen TNI Edwin Adrian Sumantha memimpin Apel Gelar Kesiapan ...</t>
+        </is>
+      </c>
+      <c r="F731" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G731" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687877/danpaspampres-pimpin-gelar-kesiapan-pasukan-rangkaian-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_4888.jpg</t>
+        </is>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Pemerintah fokus tangani karhutla di enam provinsi rawan</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:13:53 +0700</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>Pemerintah memfokuskan penanganan kebakaran hutan dan lahan (karhutla) di enam provinsi yang paling rawan, yakni Riau, ...</t>
+        </is>
+      </c>
+      <c r="F732" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687873/pemerintah-fokus-tangani-karhutla-di-enam-provinsi-rawan</t>
+        </is>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/rakor-penanganan-kebakaran-hutan-dan-lahan-2838469.jpg</t>
+        </is>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>BEI catat tambahan 9,9 juta investor dalam 7,5 bulan</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:13:38 +0700</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>PT Bursa Efek Indonesia (BEI) mencatat penambahan sekitar 9,9 juta investor pasar modal dalam kurun 7,5 bulan pada 2026 ...</t>
+        </is>
+      </c>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687869/bei-catat-tambahan-99-juta-investor-dalam-75-bulan</t>
+        </is>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000179366.jpg</t>
+        </is>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Polsek Sawah Besar amankan WNA pelaku penganiayaan di Pasar Baru</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:12:30 +0700</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>Polres Metro Jakarta Pusat melalui Polsek Sawah Besar mengamankan seorang warga negara asing (WNA) asal Nigeria ...</t>
+        </is>
+      </c>
+      <c r="F734" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687867/polsek-sawah-besar-amankan-wna-pelaku-penganiayaan-di-pasar-baru</t>
+        </is>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/01/1000000143.jpg</t>
+        </is>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>APBD Perubahan Jatim 2026 prioritaskan pelayanan publik-infrastruktur</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:11:04 +0700</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi Jawa Timur memprioritaskan penguatan sektor pelayanan publik, pendidikan, kesehatan, dan ...</t>
+        </is>
+      </c>
+      <c r="F735" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687864/apbd-perubahan-jatim-2026-prioritaskan-pelayanan-publik-infrastruktur</t>
+        </is>
+      </c>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1343790.jpg</t>
+        </is>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Dorongan transparansi dan independensi BPKH terus menguat</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:10:57 +0700</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>Rancangan Undang-Undang (RUU) tentang Perubahan atas Undang-Undang Nomor 34 Tahun 2014 tentang Pengelolaan Keuangan ...</t>
+        </is>
+      </c>
+      <c r="F736" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687863/dorongan-transparansi-dan-independensi-bpkh-terus-menguat</t>
+        </is>
+      </c>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/21/pembagian-biaya-hidup-kepada-jch-embarkasi-makassar-2775924.jpg</t>
+        </is>
+      </c>
+      <c r="I736" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>ITERA-ITB kolabirasi program fast track S1-S2 jadi Lima tahun</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:10:40 +0700</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>Institut Teknologi Sumatera (ITERA) berkolaborasi dengan Institut Teknologi Bandung (ITB) melalui Jalur Kerja Sama ...</t>
+        </is>
+      </c>
+      <c r="F737" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687860/itera-itb-kolabirasi-program-fast-track-s1-s2-jadi-lima-tahun</t>
+        </is>
+      </c>
+      <c r="H737" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1001143937.jpg</t>
+        </is>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Produsen robot China Unitree buka pemesanan IPO respons minat investor</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:09:19 +0700</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>Produsen robot asal China, Unitree Robotics, pada Senin (10/8) membuka periode pemesanan untuk penawaran umum perdana ...</t>
+        </is>
+      </c>
+      <c r="F738" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687859/produsen-robot-china-unitree-buka-pemesanan-ipo-respons-minat-investor</t>
+        </is>
+      </c>
+      <c r="H738" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/CjkinzN000011_20260810_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Kim Ji Won sumbangkan 100 juta won untuk RS dan ringankan pengobatan</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:08:49 +0700</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>Aktris Korea Selatan Kim Ji Won menyumbangkan 100 juta won atau Rp1,26 miliar rupiah (asumsi kurs Rp12,64) untuk ...</t>
+        </is>
+      </c>
+      <c r="F739" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687857/kim-ji-won-sumbangkan-100-juta-won-untuk-rs-dan-ringankan-pengobatan</t>
+        </is>
+      </c>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/02/17/KimJiwon.jpg</t>
+        </is>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Perluas layanan, PAM Jaya akan bangun 7.000 km jaringan pipa</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:07:33 +0700</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>Perusahaan Air Minum (PAM) Jaya akan membangun sekitar 7.000 kilometer (km) jaringan pipa baru dalam beberapa tahun ke ...</t>
+        </is>
+      </c>
+      <c r="F740" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687856/perluas-layanan-pam-jaya-akan-bangun-7000-km-jaringan-pipa</t>
+        </is>
+      </c>
+      <c r="H740" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_6665.jpeg</t>
+        </is>
+      </c>
+      <c r="I740" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Pegadaian resmi jadi satu-satunya Bullion Bank Underlying Provider ETF Emas di Indonesia</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:06:16 +0700</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>Memasuki babak baru pengembangan ekosistem investasi emas di Indonesia, Exchange Traded Fund (ETF) Emas resmi ...</t>
+        </is>
+      </c>
+      <c r="F741" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G741" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687855/pegadaian-resmi-jadi-satu-satunya-bullion-bank-underlying-provider-etf-emas-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H741" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/Peluncuran-ETF-Emas.jpg</t>
+        </is>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Kebun Raya Bogor kembangkan wisata berbasis pengalaman</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:05:35 +0700</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>Kebun Raya Bogor mengembangkan konsep wisata berbasis pengalaman dengan mengajak pengunjung mengenal dan mempelajari ...</t>
+        </is>
+      </c>
+      <c r="F742" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687851/kebun-raya-bogor-kembangkan-wisata-berbasis-pengalaman</t>
+        </is>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1003328073.jpg</t>
+        </is>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Tim Ekspedisi Patriot latih UMKM di Manokwari olah matoa jadi dodol</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:03:14 +0700</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>Tim Ekspedisi Patriot Universitas Airlangga (Unair) Surabaya melatih pelaku usaha mikro kecil dan menengah (UMKM) ...</t>
+        </is>
+      </c>
+      <c r="F743" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G743" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687843/tim-ekspedisi-patriot-latih-umkm-di-manokwari-olah-matoa-jadi-dodol</t>
+        </is>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/25132.jpg</t>
+        </is>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Kemenhub catat 1,35 juta kendaraan angkutan barang patuhi aturan</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:00:42 +0700</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>Kementerian Perhubungan (Kemenhub) mencatat sekitar 1,3 juta kendaraan angkutan barang telah mematuhi ketentuan dimensi ...</t>
+        </is>
+      </c>
+      <c r="F744" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687841/kemenhub-catat-135-juta-kendaraan-angkutan-barang-patuhi-aturan</t>
+        </is>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/8243E8DC-E87A-4F8A-A69B-8E852D26B953.jpeg</t>
+        </is>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Aksi TNI AL gagalkan penyelundupan 1,3 ton narkoba</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>TNI Angkatan Laut bersama tim gabungan menggagalkan upaya penyelundupan 1,3 ton narkoba jenis ketamin dari kapal asing ...</t>
+        </is>
+      </c>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5687724/aksi-tni-al-gagalkan-penyelundupan-13-ton-narkoba</t>
+        </is>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/20260810-Aksi-cepat-gagalkan-penyelundupan-1-3-ton-narkoba_2.jpg</t>
+        </is>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Kurir SPX kembalikan uang Rp92 juta akibat salah transfer</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:57:30 +0700</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>Seorang kurir SPX Express, Syarif Husein Akbar, mengembalikan uang sebesar Rp92 juta milik pelanggan yang salah ...</t>
+        </is>
+      </c>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687837/kurir-spx-kembalikan-uang-rp92-juta-akibat-salah-transfer</t>
+        </is>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/WhatsApp-Image-2026-08-10-at-5.14.22-PM.jpeg</t>
+        </is>
+      </c>
+      <c r="I746" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Hoaks! Pendaftaran upacara HUT Ke-81 RI di Istana Merdeka berbayar</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:56:45 +0700</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>Jakarta (ANTARA/JACX) – Sebuah unggahan di Facebook menarasikan bahwa masyarakat yang ingin mengikuti ...</t>
+        </is>
+      </c>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687833/hoaks-pendaftaran-upacara-hut-ke-81-ri-di-istana-merdeka-berbayar</t>
+        </is>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/08/19/edit-CBS_7400.jpg</t>
+        </is>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Polinela-Unila terapkan IoT dan PLTS untuk penyiraman kebun terong</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:56:41 +0700</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>Politeknik Negeri Lampung (Polinela) bersama Universitas Lampung (Unila) Polinela menerapkan sistem penyiraman ...</t>
+        </is>
+      </c>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687831/polinela-unila-terapkan-iot-dan-plts-untuk-penyiraman-kebun-terong</t>
+        </is>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_1729.jpeg</t>
+        </is>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Kegiatan otomotif semakin lekat dengan industri kreatif</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:56:33 +0700</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>Budaya kustom atau custome culture sejak beberapa tahun silam, telah menunjukkan fenomena yang bersinggungan dengan ...</t>
+        </is>
+      </c>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5687827/kegiatan-otomotif-semakin-lekat-dengan-industri-kreatif</t>
+        </is>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/WhatsApp-Image-2026-08-10-at-16.44.24.jpeg</t>
+        </is>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Hoaks! Mendes Yandri minta warung desa ditutup agar warga belanja di Kopdes</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:55:18 +0700</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>Jakarta (ANTARA/JACX) – Sebuah unggahan video berdurasi delapan detik di Facebook menampilkan Menteri ...</t>
+        </is>
+      </c>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687823/hoaks-mendes-yandri-minta-warung-desa-ditutup-agar-warga-belanja-di-kopdes</t>
+        </is>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/IMG_20260801_172518.jpg</t>
+        </is>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Keluarga Sutrimo Pertanyakan Formulir Kronologi-Dompet dan HP yang Tak kembali</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:11:33 +0700</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>Anang Firmansyah</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>Kuasa hukum keluarga Sutrimo mengungkap awalnya tidak menaruh kecurigaan apa pun saat menerima jenazah Sutrimo.</t>
+        </is>
+      </c>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612621/keluarga-sutrimo-pertanyakan-formulir-kronologi-dompet-dan-hp-yang-tak-kembali</t>
+        </is>
+      </c>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/kuasa-hukum-keluarga-sutrimo-aan-rohaeni-saat-memberikan-keterangan-kepada-wartawan-usai-melapor-ke-polresta-banyumas-sabtu-88-1786357485293_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I751" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Soekarno Cup 2026 Bentuk Komitmen PDIP Ciptakan Bibit Muda Sepakbola RI</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:08:35 +0700</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>Faiq Azmi</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>Turnamen Soekarno Cup 2026 resmi dimulai, diikuti 16 provinsi. PDIP berkomitmen mencari bibit pesepakbola muda untuk masa depan sepakbola Indonesia.</t>
+        </is>
+      </c>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612618/soekarno-cup-2026-bentuk-komitmen-pdip-ciptakan-bibit-muda-sepakbola-ri</t>
+        </is>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/soekarno-cup-2026-1786211228302.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Satpam Five Stars Bali Sempat Kabur Bawa Ekstasi Saat Hendak Ditangkap Polisi</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:03:07 +0700</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>Direktorat Narkoba Polri menangkap 53 orang di kelab malam Five Stars Bali terkait peredaran narkoba. Penyelidikan melibatkan teknik Under Cover Buy.</t>
+        </is>
+      </c>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612614/satpam-five-stars-bali-sempat-kabur-bawa-ekstasi-saat-hendak-ditangkap-polisi</t>
+        </is>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/bareskrim-polri-mengungkap-peredaran-di-five-stars-denpasar-bali-dan-mengamankan-53-orang-1786079431797_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I753" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Pria di Kuningan Tega Bunuh Ibu gegara Kesal Dibangunkan Salat Subuh</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:51:44 +0700</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>Fahmi Labibnajib</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>Seorang pria di Kuningan tega membunuh ibunya lantaran kesal dibangunkan salat subuh. Pelaku ditangkap polisi setelah melarikan diri ke Brebes.</t>
+        </is>
+      </c>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612591/pria-di-kuningan-tega-bunuh-ibu-gegara-kesal-dibangunkan-salat-subuh</t>
+        </is>
+      </c>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/08/12/ilustrasi-pembunuhan-1754995633409_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Kronologi Duel Maut 2 WNA Asal Afrika Dipicu Utang di Kafe Jakpus</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:50:59 +0700</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Jabbar Ramdhani</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>Dua WNA berduel di salah satu kafe kawasan Jakpus hingga mengakibatkan salah satunya tewas. Polisi telah menangkap WN Nigeria terkait duel maut itu.</t>
+        </is>
+      </c>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612589/kronologi-duel-maut-2-wna-asal-afrika-dipicu-utang-di-kafe-jakpus</t>
+        </is>
+      </c>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/dua-wna-berduel-di-salah-satu-kafe-kawasan-jakpus-hingga-mengakibatkan-salah-satunya-tewas-polisi-telah-menangkap-wn-nigeria-t-1786359032609_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I755" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Inflasi Juli 2026 Capai 2,88 Persen, Mendagri Sebut Masih Rentang Ideal</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:49:39 +0700</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>Fara Difa Alfeni</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>Mendagri Tito Karnavian menyatakan inflasi Juli 2026 sebesar 2,88% masih ideal. Ia minta Pemda waspada terhadap daerah dengan inflasi tinggi.</t>
+        </is>
+      </c>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G756" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612586/inflasi-juli-2026-capai-2-88-persen-mendagri-sebut-masih-rentang-ideal</t>
+        </is>
+      </c>
+      <c r="H756" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/kemendagri-1786358338269.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I756" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Mendikdasmen soal Temuan 995 Senjata di Sekolah Jaksel: Sedang Dicari Jalan Keluar</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:41:12 +0700</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>Mendikdasmen Abdul Mu'ti menanggapi temuan 995 senjata di sekolah Jaksel. Dia berkomitmen menjadikan sekolah aman sambil mencari solusi bersama pihak terkait.</t>
+        </is>
+      </c>
+      <c r="F757" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G757" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612561/mendikdasmen-soal-temuan-995-senjata-di-sekolah-jaksel-sedang-dicari-jalan-keluar</t>
+        </is>
+      </c>
+      <c r="H757" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/20/mendikdasmen-abdul-muti-1784547333294_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I757" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Bima Arya Minta Pemda Perkuat Sistem Penanganan Kekerasan Perempuan-Anak</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:39:18 +0700</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>Rahmat Khairurizqi</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr">
+        <is>
+          <t>Wamendagri Bima Arya tegaskan dukungan Kemendagri untuk penguatan sistem penanganan kekerasan terhadap perempuan &amp; anak melalui integrasi dan pembiayaan memadai</t>
+        </is>
+      </c>
+      <c r="F758" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612556/bima-arya-minta-pemda-perkuat-sistem-penanganan-kekerasan-perempuan-anak</t>
+        </is>
+      </c>
+      <c r="H758" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/kemendagri-1786358338343_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I758" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Puan Maharani Minta Kebakaran Bromo Segera Ditangani Total</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:39:14 +0700</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>Moch. Prima Fauzi</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr">
+        <is>
+          <t>Ketua DPR Puan Maharani mendesak pemerintah tangani kebakaran hutan di Bromo dan Palangka Raya. Keselamatan masyarakat dan pemulihan ekosistem jadi prioritas.</t>
+        </is>
+      </c>
+      <c r="F759" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G759" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612555/puan-maharani-minta-kebakaran-bromo-segera-ditangani-total</t>
+        </is>
+      </c>
+      <c r="H759" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/20/puan-maharani-dok-youtube-setpres-1779247794648_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I759" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Destry Damayanti Calon Tunggal Gubernur BI, Airlangga Bilang Begini</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:30:46 +0700</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>Retno Ayuningrum</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Perekonomian Airlangga Hartarto mengatakan sosok Destry bukanlah orang baru.</t>
+        </is>
+      </c>
+      <c r="F760" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G760" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8612628/destry-damayanti-calon-tunggal-gubernur-bi-airlangga-bilang-begini</t>
+        </is>
+      </c>
+      <c r="H760" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/13/menko-perekonomian-airlangga-hartarto-1783940653691_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I760" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Art Toys RI Berpeluang Cuan Rp 17 Miliar dari Pasar Korea Selatan</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:01:06 +0700</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>Art toys Indonesia berpotensi meraih Rp 17 miliar dari pasar Korea Selatan. Pameran URBAN BREAK &amp; TOY CON SEOUL 2026 menarik perhatian besar pembeli.</t>
+        </is>
+      </c>
+      <c r="F761" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G761" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8612612/art-toys-ri-berpeluang-cuan-rp-17-miliar-dari-pasar-korea-selatan</t>
+        </is>
+      </c>
+      <c r="H761" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/11/18/pameran-hong-kong-art-toys-2024-jakarta-digelar-di-mall-of-indonesia-jakarta-utara-hingga-24-november-2024-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I761" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Pegadaian Jadi Satu-satunya Bullion Bank Underlying Provider ETF Emas RI</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:58:29 +0700</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>Moch. Prima Fauzi</t>
+        </is>
+      </c>
+      <c r="E762" t="inlineStr">
+        <is>
+          <t>Peluncuran ETF Emas di Indonesia menandai langkah baru dalam investasi emas, memperluas akses masyarakat melalui pasar modal dan sinergi industri bullion.</t>
+        </is>
+      </c>
+      <c r="F762" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G762" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8612607/pegadaian-jadi-satu-satunya-bullion-bank-underlying-provider-etf-emas-ri</t>
+        </is>
+      </c>
+      <c r="H762" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/pegadaian-1786359492880_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I762" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Rumah Kontrakan dan Wacana Pajak 2027</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:58:10 +0700</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>Rifkianto Nugroho</t>
+        </is>
+      </c>
+      <c r="E763" t="inlineStr">
+        <is>
+          <t>DJP memastikan belum ada program pajak khusus bagi pemilik rumah kontrakan pada 2027, meski pemerintah berencana memperluas basis perpajakan.</t>
+        </is>
+      </c>
+      <c r="F763" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G763" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8612474/rumah-kontrakan-dan-wacana-pajak-2027</t>
+        </is>
+      </c>
+      <c r="H763" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/rumah-kontrakan-dalam-wacana-perluasan-basis-pajak-wacana-perluasan-pajak-dan-rumah-kontrakan-1786355268864.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I763" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>Jonathan Frizzy Bentuk Badan demi Penampilan</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:10:24 +0700</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr">
+        <is>
+          <t>Jonathan Frizzy kembali bersinar setelah kasus vape ilegal. Kini, ia aktif sebagai brand ambassador dan affiliator, sambil fokus pada kebugaran tubuhnya.</t>
+        </is>
+      </c>
+      <c r="F764" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G764" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8612260/jonathan-frizzy-bentuk-badan-demi-penampilan</t>
+        </is>
+      </c>
+      <c r="H764" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/03/03/jonathan-frizzy-1772514298397_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I764" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Keseruan Kylie Jenner Rayakan Ultah dengan Pesta Serba Pink</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:07:18 +0700</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E765" t="inlineStr">
+        <is>
+          <t>Selebritas Kylie Jenner baru saja merayakan ulang tahunnya yang ke-29 dengan meriah. Begini keseruannya.</t>
+        </is>
+      </c>
+      <c r="F765" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G765" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8611884/keseruan-kylie-jenner-rayakan-ultah-dengan-pesta-serba-pink</t>
+        </is>
+      </c>
+      <c r="H765" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/kylie-jenner-1786338705752_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I765" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Augie Fantinus Happy Syuting Bapakmu Kiper</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 16:47:27 +0700</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr">
+        <is>
+          <t>Film Bapakmu Kiper tayang 3 September 2026. Augie Fantinus berbagi pengalaman syuting dan kecintaannya pada sepakbola dalam film ini.</t>
+        </is>
+      </c>
+      <c r="F766" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G766" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/movie/d-8612461/augie-fantinus-happy-syuting-bapakmu-kiper</t>
+        </is>
+      </c>
+      <c r="H766" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/augie-fantinus-1786354925017_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I766" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Momen Aldi Taher Peluk Vokalis Jet di Panggung Jadi Sorotan</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 16:12:20 +0700</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>wes</t>
+        </is>
+      </c>
+      <c r="E767" t="inlineStr">
+        <is>
+          <t>Aldi Taher tiba-tiba aja naik ke atas panggung dan memeluk vokalis Jet, Nic Cester. Momen itu menuai sorotan.</t>
+        </is>
+      </c>
+      <c r="F767" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G767" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8612119/momen-aldi-taher-peluk-vokalis-jet-di-panggung-jadi-sorotan</t>
+        </is>
+      </c>
+      <c r="H767" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/aldi-taher-1786345749578_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I767" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Mata Juling Mendadak pada Orang Dewasa, Waspadai Sinyal Diabetes, Hipertensi, hingga Gangguan Saraf</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:24:59 +0700</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E768" t="inlineStr">
+        <is>
+          <t>Penyakit sistemik seperti diabetes dan hipertensi dapat memicu gangguan pada saraf yang mengatur pergerakan mata.</t>
+        </is>
+      </c>
+      <c r="F768" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G768" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866480/mata-juling-mendadak-pada-orang-dewasa-waspadai-sinyal-diabetes-hipertensi-hingga-gangguan-saraf</t>
+        </is>
+      </c>
+      <c r="H768" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/oYC7Eu25ziOyR3hKvcJU_h4-zIA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/bakti-sosial-operasi-mata-juling-jec_20231015_172841.jpg</t>
+        </is>
+      </c>
+      <c r="I768" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Dari Pengintai hingga Eksekutor, Begini Peran Komplotan Begal Bekasi</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:23:29 +0700</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E769" t="inlineStr">
+        <is>
+          <t>Enam pelaku membagi tugas saat mengincar nasabah bank di Bekasi, dari mengamati target hingga mengeksekusi korban.</t>
+        </is>
+      </c>
+      <c r="F769" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G769" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866479/dari-pengintai-hingga-eksekutor-begini-peran-komplotan-begal-bekasi</t>
+        </is>
+      </c>
+      <c r="H769" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0rBKhvLskYx-2WBQEOKl8okIBJo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pengendara-motor-menjadi-korban-perampokan-bersenjata-tajam-di-Tokma-Cibitung-Bekasi.jpg</t>
+        </is>
+      </c>
+      <c r="I769" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Khariq Anhar Tertunduk dan Geleng-geleng Kepala Dituntut 6 Bulan Penjara Tekait Kasus Timpa Teks</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:23:20 +0700</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>Khariq Anhar tertunduk dan menggeleng-gelengkan kepala setelah tuntutan 6 bulan penjara terhadap dirinya dibacakan jaksa penuntut umum</t>
+        </is>
+      </c>
+      <c r="F770" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G770" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866478/khariq-anhar-tertunduk-dan-geleng-geleng-kepala-dituntut-6-bulan-penjara-tekait-kasus-timpa-teks</t>
+        </is>
+      </c>
+      <c r="H770" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/vaPH1NzCY8A7jHYj-ZNhGO_Q3pE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Khariq-Anhar-tertunduk-dan-menggeleng-gelengkan-kepala.jpg</t>
+        </is>
+      </c>
+      <c r="I770" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu Disenchanted - My Chemical Romance: If I'm So Wrong</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:19:53 +0700</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>Berikut ini merupakan terjemahan lirik lagu Disenchanted yang dipopulerkan oleh grup band My Chemical Romance.</t>
+        </is>
+      </c>
+      <c r="F771" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G771" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7866477/terjemahan-lirik-lagu-disenchanted-my-chemical-romance-if-im-so-wrong</t>
+        </is>
+      </c>
+      <c r="H771" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zLN77GXG_MWcQ27NDqNvGgp-QJs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-musik-ilustrasi-lirik-ilustrasi-terjemahan-lirik-lagu.jpg</t>
+        </is>
+      </c>
+      <c r="I771" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>NSHE Jalankan Revegetasi di Pembangunan PLTA Batangtoru Tapanuli Selatan</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:19:16 +0700</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>Pembangunan PLTA Batangtoru dilakukan beriringan dengan revegetasi, pemantauan lingkungan dan pembangunan jembatan arboreal.</t>
+        </is>
+      </c>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G772" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7866476/nshe-jalankan-revegetasi-di-pembangunan-plta-batangtoru-tapanuli-selatan</t>
+        </is>
+      </c>
+      <c r="H772" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/O_v98bwH_ZfAzpTpMfQtuTxJYhc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kegiatan-revegetasi-PT-North-Sumatera-Hydro-Energy-PT-NSHE.jpg</t>
+        </is>
+      </c>
+      <c r="I772" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>Salah Tekstur MPASI Bisa Bikin Anak Sulit Mengunyah dan Menelan, Ini Kata Dokter Gigi Anak</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:19:10 +0700</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>Tekstur MPASI tidak sesuai kemampuan anak dapat membuat anak sulit mengunyah dan menelan, orang tua sebaiknya tidak buru-buru, ini penjelasan dokter.</t>
+        </is>
+      </c>
+      <c r="F773" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G773" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866475/salah-tekstur-mpasi-bisa-bikin-anak-sulit-mengunyah-dan-menelan-ini-kata-dokter-gigi-anak</t>
+        </is>
+      </c>
+      <c r="H773" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/nVKQQ_L9VD82UiYOZ_otjUt-4Mc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-bayi-ilustrasi-mpasi.jpg</t>
+        </is>
+      </c>
+      <c r="I773" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>Bigmo Sowan ke Keluarga Anak yang Terlibat Livestreaming, Minta Maaf ke Orang Tua Mereka</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:18:53 +0700</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>Bigmo mendatangi keluarga anak-anak tersebut sebagai bentuk iktikad baik setelah kejadian live streaming yang menjadi polemik.</t>
+        </is>
+      </c>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G774" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866474/bigmo-sowan-ke-keluarga-anak-yang-terlibat-livestreaming-minta-maaf-ke-orang-tua-mereka</t>
+        </is>
+      </c>
+      <c r="H774" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/MB1ZiNQ6NK2dGnKcwEd1QqaGYkc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bigmo-1-10082026.jpg</t>
+        </is>
+      </c>
+      <c r="I774" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Noda Gigi Belum Tentu Karies, Begini Cara Bedakan dengan Gigi Berlubang</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:16:43 +0700</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>Noda pada gigi belum tentu tanda karies. Kenali perbedaan noda akibat kopi, teh, rokok dengan gigi berlubang menurut dokter gigi.</t>
+        </is>
+      </c>
+      <c r="F775" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G775" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866473/noda-gigi-belum-tentu-karies-begini-cara-bedakan-dengan-gigi-berlubang</t>
+        </is>
+      </c>
+      <c r="H775" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/fHcmJWiZ5D6iDxXn5TaUg_EZ5rc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/siswa-sd-SIKAT-GIGI-1.jpg</t>
+        </is>
+      </c>
+      <c r="I775" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Discover Nusantara: Rayakan Semangat Kemerdekaan melalui Ragam Budaya, Kuliner dan Ekonomi Kreatif</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:15:50 +0700</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>Sebanyak 24 provinsi membawa seni, wastra, kuliner, dan produk UMKM ke Jakarta lewat Discover Nusantara dalam rangkaian HUT ke-81 RI</t>
+        </is>
+      </c>
+      <c r="F776" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G776" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866472/discover-nusantara-rayakan-semangat-kemerdekaan-melalui-ragam-budaya-kuliner-dan-ekonomi-kreatif</t>
+        </is>
+      </c>
+      <c r="H776" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/G_zb50yF9zVZ2vqBtLJLiAs5shE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/diskafer111111.jpg</t>
+        </is>
+      </c>
+      <c r="I776" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>Inflasi Juli 2026 Capai 2,88 Persen, Mendagri Tito: Masih dalam Rentang Ideal</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:14:01 +0700</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>Mendagri Tito mengapresiasi tingkat inflasi secara year on year (yoy) pada Juli 2026 yang tercatat sebesar 2,88 persen.</t>
+        </is>
+      </c>
+      <c r="F777" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G777" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kilas-kementerian/7866471/inflasi-juli-2026-capai-288-persen-mendagri-tito-masih-dalam-rentang-ideal</t>
+        </is>
+      </c>
+      <c r="H777" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/71B_xWOFzKOREG94sS3z4gO4gHw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Mendagri-Tito-Karnavian-Senin-108.jpg</t>
+        </is>
+      </c>
+      <c r="I777" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Buntut Live Streaming Vape Libatkan Anak, Bigmo Diperiksa Polisi dan Akui Kesalahannya</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:12:22 +0700</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>Saat live streaming, Bigmo diduga menyebut salah satu brand liquid vape atau rokok elektrik ketika berinteraksi dengan anak-anak di bawah umur.</t>
+        </is>
+      </c>
+      <c r="F778" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G778" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866470/buntut-live-streaming-vape-libatkan-anak-bigmo-diperiksa-polisi-dan-akui-kesalahannya</t>
+        </is>
+      </c>
+      <c r="H778" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/kVJ1JVg63OmX06VPzX6uBJAdK7g=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/bigmo-apa.jpg</t>
+        </is>
+      </c>
+      <c r="I778" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Jadi Calon Tunggal Gubernur BI, Destry Damayanti Dihadapkan Tantangan Jaga Rupiah dan Independensi</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:11:39 +0700</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>Koordinasi antara BI dan pemerintah memang penting, tetapikoordinasi tersebut tidak boleh menghilangkan independensi bank sentral.</t>
+        </is>
+      </c>
+      <c r="F779" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G779" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7866469/jadi-calon-tunggal-gubernur-bi-destry-damayanti-dihadapkan-tantangan-jaga-rupiah-dan-independensi</t>
+        </is>
+      </c>
+      <c r="H779" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/65Lo5yaCMnnV5UuorcZ5wxSBZwE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Penjabat-Gubernur-Bank-Indonesia-BI-Destry-Damayanti-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I779" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>'NATO Timur Tengah' Bentukan Arab Saudi-Pakistan-Turki Jadi Ancaman atau Sekutu Bagi Iran?</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:07:47 +0700</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>Paradoksnya, salah satu kemungkinan jangka panjang justru adalah Iran masuk ke dalam arsitektur keamanan regional tersebut.</t>
+        </is>
+      </c>
+      <c r="F780" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G780" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866468/nato-timur-tengah-bentukan-arab-saudi-pakistan-turki-jadi-ancaman-atau-sekutu-bagi-iran</t>
+        </is>
+      </c>
+      <c r="H780" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/sKTjW2IWme_tj-rBEFT9DF7gqhA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PAKTA-PERTAHANAN-Bendera-Arab-Saudi-Pakistan-dan-Turki.jpg</t>
+        </is>
+      </c>
+      <c r="I780" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Misteri Kematian Winda Lorenza, Saksi KPK yang Sempat Terima Apartemen dan Jam Tangan Mewah</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:06:36 +0700</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>Winda Lorenza Gowasa, mantan istri polisi yang meninggal dunia di Medan disebut pernah diperiksa KPK terkait kasus suap pejabat Bea Cukai.</t>
+        </is>
+      </c>
+      <c r="F781" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G781" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866467/misteri-kematian-winda-lorenza-saksi-kpk-yang-sempat-terima-apartemen-dan-jam-tangan-mewah</t>
+        </is>
+      </c>
+      <c r="H781" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/qz6cNS9JQnwE8G3U7M2BKGZF1Ng=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/mantan-istri-polisi-di-medan.jpg</t>
+        </is>
+      </c>
+      <c r="I781" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>Tumbang Usia Syuting, Dimas Aditya Ngoyo Gym 6 Hari Sepekan dan Tidur 3 Jam Demi Urang Bunian</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:05:43 +0700</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>Kesehatan Dimas Aditya menurun usai syuting film horor Urang Bunian. Bahkan ia harus menjalani pengobatan ke Malaysia.</t>
+        </is>
+      </c>
+      <c r="F782" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G782" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866466/tumbang-usia-syuting-dimas-aditya-ngoyo-gym-6-hari-sepekan-dan-tidur-3-jam-demi-urang-bunian</t>
+        </is>
+      </c>
+      <c r="H782" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Xyon9h6AXxUCv24WjA1iHGIj3vI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Dimas-Aditya-1-10082026.jpg</t>
+        </is>
+      </c>
+      <c r="I782" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Bima Arya Dorong Penguatan Sistem Penanganan Kekerasan terhadap Perempuan dan Anak di Daerah</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:05:40 +0700</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>Kemendagri berkomitmen mendukung penguatan sistem penanganan kekerasan terhadap perempuan dan anak di daerah melalui integrasi antarsistem.</t>
+        </is>
+      </c>
+      <c r="F783" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G783" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kilas-kementerian/7866465/bima-arya-dorong-penguatan-sistem-penanganan-kekerasan-terhadap-perempuan-dan-anak-di-daerah</t>
+        </is>
+      </c>
+      <c r="H783" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/gsRVQtShNuekIBhrXILzSPyvI8I=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Wamendagri-Bima-Arya-Senin-108.jpg</t>
+        </is>
+      </c>
+      <c r="I783" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Rusa Bawean di Ambang Kepunahan, Habitat Menyusut hingga Ancaman Anjing, DiCaprio-Bezos Turun Tangan</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:01:54 +0700</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>Rusa Bawean hanya hidup di Pulau Bawean dan kini terancam punah. Populasinya terbatas, sementara habitat dan ruang hidupnya terus tertekan</t>
+        </is>
+      </c>
+      <c r="F784" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G784" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866464/rusa-bawean-di-ambang-kepunahan-habitat-menyusut-hingga-ancaman-anjing-dicaprio-bezos-turun-tangan</t>
+        </is>
+      </c>
+      <c r="H784" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/m78o3AHLbf_lw9austaCyXD-NTQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/rusabawean1111111.jpg</t>
+        </is>
+      </c>
+      <c r="I784" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>30 Banner Malam Tirakatan 17 Agustus 2026, Pilihan Desain Kreatif dan Meriah untuk Perayaan HUT RI</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:01:51 +0700</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>Banner malam tirakatan berfungsi sebagai dekorasi acara, dengan desain yang dapat disesuaikan dengan tema dan suasana perayaan.</t>
+        </is>
+      </c>
+      <c r="F785" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G785" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866463/30-banner-malam-tirakatan-17-agustus-2026-pilihan-desain-kreatif-dan-meriah-untuk-perayaan-hut-ri</t>
+        </is>
+      </c>
+      <c r="H785" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/26sTuo-0R_YY-xflIjfKv94m6ak=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/acara-malam-tirakatan-313.jpg</t>
+        </is>
+      </c>
+      <c r="I785" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>Potensi Cuaca di Indonesia Periode 11 – 17 Agustus 2026: Puncak Fenomena El Nino</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:59:17 +0700</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>Simak potensi curah hujan di Indonesia selama periode 11 – 17 Agustus 2026, hujan semakin jarang terjadi namun kini menuju puncak fenomena El Nino.</t>
+        </is>
+      </c>
+      <c r="F786" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G786" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866462/potensi-cuaca-di-indonesia-periode-11-17-agustus-2026-puncak-fenomena-el-nino</t>
+        </is>
+      </c>
+      <c r="H786" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5NsvRAfKVVqlNUGVnYRGovtF7v4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-cerah-berawan-8.jpg</t>
+        </is>
+      </c>
+      <c r="I786" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Menko Polkam: Karhutla Bisa Pengaruhi Karier Pangdam dan Kapolda</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:58:41 +0700</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>Menko Polkam menegaskan keberhasilan mengendalikan karhutla menjadi ukuran kinerja Pangdam dan Kapolda di daerah.</t>
+        </is>
+      </c>
+      <c r="F787" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G787" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866461/menko-polkam-karhutla-bisa-pengaruhi-karier-pangdam-dan-kapolda</t>
+        </is>
+      </c>
+      <c r="H787" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Hd-phEqUAJjjJpVJ0H0S_SSBao8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Menko-Polkam-Djamari-Chaniago-seusai-memimpin-rapat-di-Kemenko-Polkam.jpg</t>
+        </is>
+      </c>
+      <c r="I787" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Investor Pasar Modal Bertambah 9,9 Juta, Tembus 30,27 Juta di 2026</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:36:24 +0700</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>Friska Yolandha</t>
+        </is>
+      </c>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA — PT Bursa Efek Indonesia (BEI) mencatat penambahan sekitar 9,9 juta investor pasar modal dalam 7,5 bulan pada 2026. Dengan penambahan tersebut, jumlah investor pasar modal mencapai...</t>
+        </is>
+      </c>
+      <c r="F788" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G788" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjjxko370/investor-pasar-modal-bertambah-99-juta-tembus-3027-juta-di-2026</t>
+        </is>
+      </c>
+      <c r="H788" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/030039500-1769669495-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Gamer Diajak Belajar Investasi dari Strategi Bermain Esports</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Perkembangan esports membuka ruang baru untuk mengenalkan literasi keuangan kepada generasi muda yang akrab dengan ekosistem digital. Kemampuan membaca situasi, menyusun strategi, dan menjaga disiplin dalam permainan...</t>
+        </is>
+      </c>
+      <c r="F789" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G789" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjjrdu416/gamer-diajak-belajar-investasi-dari-strategi-bermain-esports</t>
+        </is>
+      </c>
+      <c r="H789" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260810162512-347.png</t>
+        </is>
+      </c>
+      <c r="I789" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Kejagung Periksa 7 Saksi Terkait Kasus TPPU Febrie Adriansyah</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:42:50 +0700</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>Penyidik memanggil sebanyak 13 orang untuk dimintai keterangan terkait perkara TPPU Febrie Adriansyah, namun hanya tujuh orang yang memenuhi panggilan.</t>
+        </is>
+      </c>
+      <c r="F790" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G790" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266530/kejagung-periksa-7-saksi-terkait-kasus-tppu-febrie-adriansyah</t>
+        </is>
+      </c>
+      <c r="H790" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/AdibnpaOlQuNR5w3Be37I-wjLuE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320653/original/012439900_1786362162-71890.jpg</t>
+        </is>
+      </c>
+      <c r="I790" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>Paspampres Siapkan Alutsista hingga Anti-Drone untuk HUT Ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:03:37 +0700</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>Apel juga digelar untuk memastikan kesiapan 1.147 personel Paspampres serta alutsista.</t>
+        </is>
+      </c>
+      <c r="F791" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G791" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266503/paspampres-siapkan-alutsista-hingga-anti-drone-untuk-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H791" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/t1n1mNvr-bfeza8C8BfMprtF0SU=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320627/original/023592100_1786359807-IMG-20260810-WA0024.jpg</t>
+        </is>
+      </c>
+      <c r="I791" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Pahitnya Potensi Panen Kopi Petani Purwakarta, Buah Dicuri hingga Pohon Ditebang</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:44:57 +0700</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>Petani kopi Purwakarta menghadapi tahun terberat 2026. Produksi anjlok akibat kemarau, serangan hama, dan pencurian brutal rusak tanaman.</t>
+        </is>
+      </c>
+      <c r="F792" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G792" t="inlineStr">
+        <is>
+          <t>https://bandung.kompas.com/read/2026/08/10/184339678/pahitnya-potensi-panen-kopi-petani-purwakarta-buah-dicuri-hingga-pohon</t>
+        </is>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/Fy21nFSmTLXq0H6vR6y80198Gwg=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/10/6a79a63632afc.jpeg</t>
+        </is>
+      </c>
+      <c r="I792" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Kecewa pada FIFA, 3 Konfederasi Mau Bikin Turnamen Tandingan Piala Dunia</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:44:57 +0700</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>Tiga konfederasi sepak bola mulai membahas pembentukan kompetisi di luar FIFA, menyusul memburuknya hubungan dengan Gianni Infantino.</t>
+        </is>
+      </c>
+      <c r="F793" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G793" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/global/read/2026/08/10/183041970/kecewa-pada-fifa-3-konfederasi-mau-bikin-turnamen-tandingan-piala-dunia</t>
+        </is>
+      </c>
+      <c r="H793" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/IjxOcautHznQ5BXDNwmgTWzUQn0=/0x0:4992x3328/1200x675/filters:watermark(data/photo/2026/01/30/697c81ac46b81.png,0,-0,1)/data/photo/2026/06/16/6a308dcc235ea.jpg</t>
+        </is>
+      </c>
+      <c r="I793" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>PSSI Rencanakan Timnas Indonesia Hadapi Peserta Piala Dunia 2026</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:44:57 +0700</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>Timnas Indonesia berpeluang melawan negara Piala Dunia 2026 di FIFA Matchday.</t>
+        </is>
+      </c>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>https://bola.kompas.com/read/2026/08/10/18080448/pssi-rencanakan-timnas-indonesia-hadapi-peserta-piala-dunia-2026</t>
+        </is>
+      </c>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/HPAIDi_2V8Fg5mjy9PlQyJOLwvw=/113x0:1136x682/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/06/09/6a281a5adcd81.jpeg</t>
+        </is>
+      </c>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I719"/>
+  <autoFilter ref="A1:I794"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 12:44 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$794</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$886</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I794"/>
+  <dimension ref="A1:I886"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -37757,8 +37757,4332 @@
         </is>
       </c>
     </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Pemerintah kerahkan 43 helikopter untuk operasi udara tangani karhutla</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:39:25 +0700</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah kini mewaspadai ancaman El Nino kuat yang diperkirakan melanda Indonesia pada awal September hingga ...</t>
+        </is>
+      </c>
+      <c r="F795" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G795" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5687981/pemerintah-kerahkan-43-helikopter-untuk-operasi-udara-tangani-karhutla</t>
+        </is>
+      </c>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SANS_PEMERINTAH-KERAHKAN-43-HELIKOPTER-UNTUK-OPERASI-UDARA-TANGANI-KARHUTLA.jpg</t>
+        </is>
+      </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Kejati NTB banding atas vonis bebas tiga anggota DPRD</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:38:03 +0700</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>Kejaksaan Tinggi Nusa Tenggara Barat mengajukan banding atas putusan bebas tiga anggota DPRD NTB dalam perkara ...</t>
+        </is>
+      </c>
+      <c r="F796" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688008/kejati-ntb-banding-atas-vonis-bebas-tiga-anggota-dprd</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/gedung-kejati-ntb-2.jpg</t>
+        </is>
+      </c>
+      <c r="I796" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Angka kebangkrutan perusahaan di Jepang pada Juli tembus 1.000</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:36:25 +0700</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>Angka kebangkrutan perusahaan di Jepang pada Juli melampaui 1.000 kasus untuk bulan kedua berturut-turut, seiring ...</t>
+        </is>
+      </c>
+      <c r="F797" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G797" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688007/angka-kebangkrutan-perusahaan-di-jepang-pada-juli-tembus-1000</t>
+        </is>
+      </c>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/CjkinzN000012_20260810_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I797" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Fatmah Nahdi ungkap tantangan peran di film "Bisikan Desa Gringsing"</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:32:11 +0700</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>Aktris Fatmah Nahdi mengungkap tantangan memerankan karakter Fatimah dalam film terbaru berjudul "Bisikan Desa ...</t>
+        </is>
+      </c>
+      <c r="F798" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688005/fatmah-nahdi-ungkap-tantangan-peran-di-film-bisikan-desa-gringsing</t>
+        </is>
+      </c>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_20260810_184226-3.jpg</t>
+        </is>
+      </c>
+      <c r="I798" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Sulsel siapkan forum dan satgas pangan atasi harga pakan ternak ayam</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:30:52 +0700</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Provinsi Sulawesi Selatan menyiapkan sejumlah langkah untuk merespons keluhan peternak ayam petelur ...</t>
+        </is>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G799" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5687951/sulsel-siapkan-forum-dan-satgas-pangan-atasi-harga-pakan-ternak-ayam</t>
+        </is>
+      </c>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SULSEL-SIAPKAN-FORUM-DAN-SATGAS-PANGAN-ATASI-HARGA-PAKAN-TERNAK-AYAM.jpg</t>
+        </is>
+      </c>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Perbasi kembali panggil pemain untuk Asian Games 2026</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:30:31 +0700</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>Dewan Pengurus Pusat Persatuan Bola Basket Seluruh Indonesia (DPP Perbasi) kembali memanggil empat pemain untuk ...</t>
+        </is>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688003/perbasi-kembali-panggil-pemain-untuk-asian-games-2026</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/WhatsApp-Image-2026-07-30-at-19.44.26.jpeg</t>
+        </is>
+      </c>
+      <c r="I800" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Sekelompok anjing "PAW Patrol" bakal ramaikan bioskop pada 14 Agustus</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:27:14 +0700</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>Kru Paw Patrol yang beranggotakan sekelompok anjing akan berlaga dalam film "PAW Patrol:The Dino Movie" yang ...</t>
+        </is>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687999/sekelompok-anjing-paw-patrol-bakal-ramaikan-bioskop-pada-14-agustus</t>
+        </is>
+      </c>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/photo_6325543407836664781_y.jpg</t>
+        </is>
+      </c>
+      <c r="I801" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Pengadilan China selesaikan kasus tabrakan antarkapal di Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:25:04 +0700</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>Pengadilan maritim China berhasil memediasi sengketa yang timbul akibat tabrakan antara dua kapal asing di dekat Selat ...</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687997/pengadilan-china-selesaikan-kasus-tabrakan-antarkapal-di-selat-hormuz</t>
+        </is>
+      </c>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/CjkinzN000009_20260810_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I802" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>BNPB siagakan operasi darat dan OMC di 6 provinsi rawan karhutla</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:24:53 +0700</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>Badan Nasional Penanggulangan Bencana (BNPB) menyiagakan pasukan operasi darat dan operasi modifikasi cuaca (OMC) di ...</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G803" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687993/bnpb-siagakan-operasi-darat-dan-omc-di-6-provinsi-rawan-karhutla</t>
+        </is>
+      </c>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/20260810_151712.jpg</t>
+        </is>
+      </c>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Sebanyak 65 personel damkar padamkan kebakaran toko buah di Priok</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:24:37 +0700</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>Sebanyak 65 personel pemadam kebakaran dikerahkan memadamkan kebakaran toko buah yang berlokasi di Jalan Bisma Raya, ...</t>
+        </is>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687992/sebanyak-65-personel-damkar-padamkan-kebakaran-toko-buah-di-priok</t>
+        </is>
+      </c>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/17/1000938564.jpg</t>
+        </is>
+      </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Konektivitas Menuju Kepulauan Seribu Menguat, Commuter Line Hubungkan Perjalanan dari Daratan Jakarta</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:22:18 +0700</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>Rencana Pemerintah Provinsi DKI Jakarta memperkuat layanan transportasi menuju Kepulauan Seribu mulai 2027 membuka ...</t>
+        </is>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G805" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687989/konektivitas-menuju-kepulauan-seribu-menguat-commuter-line-hubungkan-perjalanan-dari-daratan-jakarta</t>
+        </is>
+      </c>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/Stasiun-Angke-pic.jpg</t>
+        </is>
+      </c>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>KAI: Manggarai disiapkan perkuat konektivitas transportasi Jakarta</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:22:11 +0700</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) menyiapkan Stasiun Manggarai untuk memperkuat konektivitas transportasi Jakarta ...</t>
+        </is>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687988/kai-manggarai-disiapkan-perkuat-konektivitas-transportasi-jakarta</t>
+        </is>
+      </c>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/7E0EA540-666C-42EB-BB88-6C0E1868B9B3.jpeg</t>
+        </is>
+      </c>
+      <c r="I806" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Hotel Borobudur gelar "Discover Nusantara" sambut HUT Kemerdekaan RI</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:22:08 +0700</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>Hotel Borobudur Jakarta menggelar program "Discover Nusantara" sepanjang Agustus 2026 dalam rangka menyambut ...</t>
+        </is>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G807" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687985/hotel-borobudur-gelar-discover-nusantara-sambut-hut-kemerdekaan-ri</t>
+        </is>
+      </c>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG-20260810-WA0016.jpg</t>
+        </is>
+      </c>
+      <c r="I807" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>162 Ribu Pergerakan Pelanggan per Hari, Manggarai Disiapkan Menguatkan Konektivitas Transportasi Jakarta</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:19:30 +0700</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) memandang Stasiun Manggarai memiliki peran strategis dalam perkembangan sistem ...</t>
+        </is>
+      </c>
+      <c r="F808" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G808" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687979/162-ribu-pergerakan-pelanggan-per-hari-manggarai-disiapkan-menguatkan-konektivitas-transportasi-jakarta</t>
+        </is>
+      </c>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/Stasiun-Manggarai-pic.jpg</t>
+        </is>
+      </c>
+      <c r="I808" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Pluang catat investor saham AS tumbuh enam kali lipat dalam tiga tahun</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:17:23 +0700</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>Jakarta (ANTARA) – Pluang mencatat jumlah investor saham Amerika Serikat (AS) yang aktif bertransaksi setiap ...</t>
+        </is>
+      </c>
+      <c r="F809" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G809" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687976/pluang-catat-investor-saham-as-tumbuh-enam-kali-lipat-dalam-tiga-tahun</t>
+        </is>
+      </c>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/Aplikasi-Pluang.jpg</t>
+        </is>
+      </c>
+      <c r="I809" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Polda Bengkulu tangkap pemilik gudang oplosan MinyaKita</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:16:05 +0700</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>Subdit I Indagsi Ditreskrimsus Polda Bengkulu menangkap HS (37), warga Jakarta, yang diduga sebagai pemilik gudang ...</t>
+        </is>
+      </c>
+      <c r="F810" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687972/polda-bengkulu-tangkap-pemilik-gudang-oplosan-minyakita</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_20260810_162750.jpg</t>
+        </is>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Papua Barat pulihkan Rp29 miliar dan serahkan 24 temuan ke APH</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:16:04 +0700</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>Inspektorat Provinsi Papua Barat menyerahkan penanganan 24 temuan terkait pengelolaan anggaran pada 2025 kepada aparat ...</t>
+        </is>
+      </c>
+      <c r="F811" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G811" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687969/papua-barat-pulihkan-rp29-miliar-dan-serahkan-24-temuan-ke-aph</t>
+        </is>
+      </c>
+      <c r="H811" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/25098.jpg</t>
+        </is>
+      </c>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Polisi olah TKP di sekolah temuan senjata dan narkoba di Jaksel</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:14:36 +0700</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>Kepolisian melakukan olah tempat kejadian perkara (TKP) di sekolah temuan 995 airsoft gun dan narkoba di kawasan Pondok ...</t>
+        </is>
+      </c>
+      <c r="F812" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687965/polisi-olah-tkp-di-sekolah-temuan-senjata-dan-narkoba-di-jaksel</t>
+        </is>
+      </c>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1001021514.jpg</t>
+        </is>
+      </c>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Kejati NTB periksa eks dirut bank syariah terkait pinjaman Rp11 miliar</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:11:35 +0700</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>Kejaksaan Tinggi Nusa Tenggara Barat memeriksa mantan Direktur Utama bank syariah milik pemerintah daerah, Kukuh ...</t>
+        </is>
+      </c>
+      <c r="F813" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G813" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687961/kejati-ntb-periksa-eks-dirut-bank-syariah-terkait-pinjaman-rp11-miliar</t>
+        </is>
+      </c>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/jubir-kejati-ntb-harun.jpg</t>
+        </is>
+      </c>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>BKSDA turunkan tim nekropsi bangkai gajah sumatra di Aceh Tamiang</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:08:23 +0700</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>Balai Konservasi Sumber Daya Alam (BKSDA) Aceh menurunkan tim dokter hewan melakukan bedah bangkai atau nekropsi gajah ...</t>
+        </is>
+      </c>
+      <c r="F814" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687957/bksda-turunkan-tim-nekropsi-bangkai-gajah-sumatra-di-aceh-tamiang</t>
+        </is>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/gajah-mati-aceh-tamiang.jpg</t>
+        </is>
+      </c>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Rudenim Tanjungpinang deportasi 25 warga negara Vietnam</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:06:42 +0700</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>Rumah Detensi Imigrasi (Rudenim) Pusat Tanjungpinang, Kepulauan Riau, mendeportasi 25 warga negara Vietnam yang ...</t>
+        </is>
+      </c>
+      <c r="F815" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G815" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687955/rudenim-tanjungpinang-deportasi-25-warga-negara-vietnam</t>
+        </is>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/inbound2795638213678190306.jpg</t>
+        </is>
+      </c>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Menhut pastikan penguatan antisipasi karhutla saat fenomena El Nino</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:06:05 +0700</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>Menteri Kehutanan (Menhut) Raja Juli Antoni mengatakan pemerintah memperkuat antisipasi kebakaran hutan dan lahan ...</t>
+        </is>
+      </c>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687952/menhut-pastikan-penguatan-antisipasi-karhutla-saat-fenomena-el-nino</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_20260810_182710.jpg</t>
+        </is>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Kemenimipas gandeng Kemenkes gelar CKG di Lapas Cipinang sambut HUT RI</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:01:50 +0700</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>ANTARA - Kementerian Imigrasi dan Pemasyarakatan (Imipas) berkolaborasi dengan Kementerian Kesehatan (Kemenkes) ...</t>
+        </is>
+      </c>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5687923/kemenimipas-gandeng-kemenkes-gelar-ckg-di-lapas-cipinang-sambut-hut-ri</t>
+        </is>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KEMENIMIPAS-GANDENG-KEMENKES-GELAR-CKG-DI-LAPAS-CIPINANG-SAMBUT-HUT-RI.jpg</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Sekolah Nasional Terintegrasi IKN beroperasi perdana dengan 82 siswa</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:58:42 +0700</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>ANTARA - Sekolah Nasional Terintegrasi (SNT) di Ibu Kota Nusantara (IKN) memulai kegiatan perdana setelah ...</t>
+        </is>
+      </c>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5687800/sekolah-nasional-terintegrasi-ikn-beroperasi-perdana-dengan-82-siswa</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SEKOLAH-NASIONAL-TERINTEGRASI-IKN-BEROPERASI-PERDANA-DENGAN-82-SISWA.jpg</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo beri dukungan penuh untuk restorasi ekosistem</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:58:10 +0700</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>Menteri Kehutanan Raja Juli Antoni mengungkapkan bahwa Presiden Prabowo Subianto memberikan dukungan penuh terhadap ...</t>
+        </is>
+      </c>
+      <c r="F819" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G819" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687947/presiden-prabowo-beri-dukungan-penuh-untuk-restorasi-ekosistem</t>
+        </is>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/01/01/1000638883.jpg</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Mendagri dan Menteri ATR/BPN percepat layanan BPHTB lewat SEB</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:55:51 +0700</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>Menteri Dalam Negeri Muhammad Tito Karnavian dan Menteri Agraria dan Tata Ruang/Kepala Badan Pertanahan Nasional Nusron ...</t>
+        </is>
+      </c>
+      <c r="F820" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G820" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687943/mendagri-dan-menteri-atr-bpn-percepat-layanan-bphtb-lewat-seb</t>
+        </is>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000583242.jpg</t>
+        </is>
+      </c>
+      <c r="I820" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Kakorbinmas Polri dorong Bhabinkamtibmas perkuat pendekatan warga</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:53:58 +0700</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>Kepala Korps Pembinaan Masyarakat (Kakorbinmas) Baharkam Polri Irjen Pol Mardiyono mendorong Bhabinkamtibmas memperkuat ...</t>
+        </is>
+      </c>
+      <c r="F821" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687940/kakorbinmas-polri-dorong-bhabinkamtibmas-perkuat-pendekatan-warga</t>
+        </is>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/489818.jpg</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Luncuran lava pijar Gunung Karangetang tak jangkau permukiman warga</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:50:56 +0700</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>Penyelidik Bumi Ahli Muda, Balai Pemantauan Gunung Api dan Mitigasi Bencana Gerakan Tanah Sulawesi Maluku, Sandy ...</t>
+        </is>
+      </c>
+      <c r="F822" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687936/luncuran-lava-pijar-gunung-karangetang-tak-jangkau-permukiman-warga</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1001994877.jpg</t>
+        </is>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>PT JIEP dorong transparansi untuk perkuat kepercayaan publik</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:48:49 +0700</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>PT Jakarta Industrial Estate Pulogadung (Perseroda) atau PT JIEP mendorong keterbukaan informasi publik sebagai salah ...</t>
+        </is>
+      </c>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687933/pt-jiep-dorong-transparansi-untuk-perkuat-kepercayaan-publik</t>
+        </is>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/InShot_20260810_180458343.jpg</t>
+        </is>
+      </c>
+      <c r="I823" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>AFC, UEFA dan Concacaf surati FIFA tolak FFE</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:48:02 +0700</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>Konfederasi sepak bola Asia (AFC0, Eropa  (UEFA) dan (Amerika Utara, Amerika Tengah, Karibia (Concacaf) ...</t>
+        </is>
+      </c>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687932/afc-uefa-dan-concacaf-surati-fifa-tolak-ffe</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/06/Peresmian-Kantor-FIFA-Jakarta-101123-hma-08.jpg</t>
+        </is>
+      </c>
+      <c r="I824" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Polresta Palu periksa sembilan saksi kasus pembunuhan satu keluarga</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:48:00 +0700</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>Polresta Palu, Sulawesi Tengah, telah memeriksa sembilan saksi dalam kasus pembunuhan satu keluarga di Jalan PDAM, ...</t>
+        </is>
+      </c>
+      <c r="F825" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687929/polresta-palu-periksa-sembilan-saksi-kasus-pembunuhan-satu-keluarga</t>
+        </is>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG-20260810-WA0007-1.jpg</t>
+        </is>
+      </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>X dikabarkan ubah skema monetisasi untuk kreator tekan orisinal konten</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:47:15 +0700</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>Platform jejaring sosial milik pebisnis Elon Musk, X dikabarkan akan melakukan perubahan skema monetisasi terhadap ...</t>
+        </is>
+      </c>
+      <c r="F826" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687927/x-dikabarkan-ubah-skema-monetisasi-untuk-kreator-tekan-orisinal-konten</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/10/08/Logo-X.jpg</t>
+        </is>
+      </c>
+      <c r="I826" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>HUT pertama Kodam XXII/Tambun Bungai teguhkan pertahanan Kalteng</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:47:14 +0700</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>ANTARA - Peringatan HUT pertama Kodam XXII/Tambun Bungai menjadi momentum memperkuat komitmen menjaga pertahanan dan ...</t>
+        </is>
+      </c>
+      <c r="F827" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G827" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5687836/hut-pertama-kodam-xxii-tambun-bungai-teguhkan-pertahanan-kalteng</t>
+        </is>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/HUT-PERTAMA-KODAM-XXII-TAMBUN-BUNGAI-TEGUHKAN-PERTAHANAN-KALTENG.jpg</t>
+        </is>
+      </c>
+      <c r="I827" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Bulog sebut stok beras 5,25 juta ton tersebar seluruh gudang Indonesia</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:45:14 +0700</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>Perum Bulog menegaskan stok cadangan beras pemerintah (CBP) secara nasional yang dikelola mencapai 5,25 juta ton, ...</t>
+        </is>
+      </c>
+      <c r="F828" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687920/bulog-sebut-stok-beras-525-juta-ton-tersebar-seluruh-gudang-indonesia</t>
+        </is>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/EC556D40-7F50-4F3D-BFA5-0B17C15F0154.jpeg</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Pengadilan Tinggi Surabaya terapkan sidang elektronik tingkat banding</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:44:29 +0700</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>ANTARA - Pengadilan Tinggi Surabaya mulai menerapkan sidang elektronik untuk seluruh perkara tingkat banding, termasuk ...</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5687687/pengadilan-tinggi-surabaya-terapkan-sidang-elektronik-tingkat-banding</t>
+        </is>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PENGADILAN-TINGGI-SURABAYA-TERAPKAN-SIDANG-ELEKTRONIK-TINGKAT-BANDING_1.jpg</t>
+        </is>
+      </c>
+      <c r="I829" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Sekolah anak-anak desa terpencil di Kerinci</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:43:58 +0700</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>Sejumlah murid berjalan meninggalkan sekolah usai mengikuti kegiatan belajar mengajar di SDN 226/III Renah Kasah, ...</t>
+        </is>
+      </c>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5687917/sekolah-anak-anak-desa-terpencil-di-kerinci</t>
+        </is>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/Semangat-sekolah-anak-anak-desa-terpencil-Kerinci-100826-ws-6.jpg</t>
+        </is>
+      </c>
+      <c r="I830" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Mensesneg serahkan surpres terkait Gubernur BI kepada DPR</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:43:04 +0700</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Sekretaris Negara Prasetyo Hadi menyerahkan tiga Surat Presiden (Surpres) kepada DPR RI, di Kompleks ...</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G831" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5687891/mensesneg-serahkan-surpres-terkait-gubernur-bi-kepada-dpr</t>
+        </is>
+      </c>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/MENSESNEG-SERAHKAN-SURPRES-TERKAIT-GUBERNUR-BI-KEPADA-DPR.jpg</t>
+        </is>
+      </c>
+      <c r="I831" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Aghniny Haque jajal syuting di kompleks Iskandar Malaysia Studios</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:42:15 +0700</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>Aktris Indonesia Aghniny Haque dan Hesti Putri membagikan pengalaman menjajal proses syuting film "Bisikan Desa ...</t>
+        </is>
+      </c>
+      <c r="F832" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5687915/aghniny-haque-jajal-syuting-di-kompleks-iskandar-malaysia-studios</t>
+        </is>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_20260810_130330.jpg</t>
+        </is>
+      </c>
+      <c r="I832" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Pencapaian Alikka Kalistha Usai Ultah ke-22: Happy Masuk TV!</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:09:51 +0700</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>Selebgram Alikka Kalistha mengungkapkan salah satu pencapaian. Kebetulan ia baru juga ulang tahun.</t>
+        </is>
+      </c>
+      <c r="F833" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G833" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8612013/pencapaian-alikka-kalistha-usai-ultah-ke-22-happy-masuk-tv</t>
+        </is>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/alikka-kalistha-1786343086146_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I833" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Vietnam Layak Waspada, Kans Malaysia Ciptakan Dejavu Masa Lalu di Semifinal Piala AFF 2026</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:26:43 +0700</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>Timnas Vietnam harus menaruh waspada terhadap Malaysia yang bakal jadi lawan mereka di semifinal Piala AFF 2026.</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866508/vietnam-layak-waspada-kans-malaysia-ciptakan-dejavu-masa-lalu-di-semifinal-piala-aff-2026</t>
+        </is>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0ZYdO2i7sJNRdAvkLPBImQFZQSw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Nguyen-Quang-Hai-Vietnam-Piala-AFF-2024-1612.jpg</t>
+        </is>
+      </c>
+      <c r="I834" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Resmikan Gol Perdana Berbaju Real Madrid, Carlos Espi Terus Jalani Proses</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:24:36 +0700</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>Pemain depan anyar Real Madrid, Carlos Espi, mencetak gol perdananya bagi Los Blancos saat berhadapan dengan Ferencvaros di laga uji coba.</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G835" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866507/resmikan-gol-perdana-berbaju-real-madrid-carlos-espi-terus-jalani-proses</t>
+        </is>
+      </c>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/KSajdTxa1ppoHKZQfARaD3lvLBw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pemain-baru-Real-Madrid-Carlos-Espi.jpg</t>
+        </is>
+      </c>
+      <c r="I835" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Kaisar Naruhito dan Permaisuri Masako Batalkan Liburan, Sumbangkan Dana Bantuan untuk Kumamoto</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:23:59 +0700</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>Kaisar Naruhito dan Permaisuri Masako menyalurkan bantuan bagi korban Gempa Kumamoto 2026. Keluarga Kekaisaran juga membatalkan agenda</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866506/kaisar-naruhito-dan-permaisuri-masako-batalkan-liburan-sumbangkan-dana-bantuan-untuk-kumamoto</t>
+        </is>
+      </c>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/eMRqsPN4yuuhvRDv1V0dYQkWps4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/naruhito111111.jpg</t>
+        </is>
+      </c>
+      <c r="I836" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Khariq Anhar Wisuda di Tengah Tuntutan 6 Bulan: “Semoga Dapat Kerja, Bukan Penjara”</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:23:52 +0700</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>Dituntut enam bulan penjara pada 10 Agustus, Khariq akan wisuda 18 Agustus sebelum kembali ke ruang sidang.</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G837" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866505/khariq-anhar-wisuda-di-tengah-tuntutan-6-bulan-semoga-dapat-kerja-bukan-penjara</t>
+        </is>
+      </c>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8fRftMALcqsKVRKz4f9OCapaRjA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Terdakwa-Khariq-Anhar-kuasa-hukum-usai-sidang-tuntutan-kasus-timpa-teks.jpg</t>
+        </is>
+      </c>
+      <c r="I837" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Jejak Gagasan Destry Damayanti Calon Gubernur BI saat Fit and Proper Test di Komisi XI DPR</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:19:29 +0700</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>Gagasannya mencakup stabilitas rupiah, kebijakan moneter, makroprudensial, sistem pembayaran digital, pasar keuangan, dan UMKM.</t>
+        </is>
+      </c>
+      <c r="F838" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G838" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7866504/jejak-gagasan-destry-damayanti-calon-gubernur-bi-saat-fit-and-proper-test-di-komisi-xi-dpr</t>
+        </is>
+      </c>
+      <c r="H838" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/c1C0qZ4ZTdcn1wQcewDcdVgY3Sk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/destry-damayanti-deputi-gubernur-senior-dgs-bank-indonesia.jpg</t>
+        </is>
+      </c>
+      <c r="I838" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>SUV  T2 i-DM Punya Garansi Kendaraan 6 Tahun Tanpa Batasan Kilometer</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:18:21 +0700</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>Perusahaan menyiapkan pusat distribusi suku cadang seluas 2.000 meter persegi yang mencakup 31.000 item parts.</t>
+        </is>
+      </c>
+      <c r="F839" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G839" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7866503/suv-t2-i-dm-punya-garansi-kendaraan-6-tahun-tanpa-batasan-kilometer</t>
+        </is>
+      </c>
+      <c r="H839" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/XfO4wACdahOFt6ItkTY6iL2cBmE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Paparan-teknologi-SUV-Jetour-T2-i-DM-di-GIIAS-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I839" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Masa Depan Pangkalan Rusia di Suriah Ditentukan dalam 3 Bulan, Ini Perubahannya</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:12:36 +0700</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>Pemerintah Suriah mengumumkan telah mencapai kesepakatan dengan Rusia mengenai masa depan kedua fasilitas tersebut.</t>
+        </is>
+      </c>
+      <c r="F840" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G840" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866502/masa-depan-pangkalan-rusia-di-suriah-ditentukan-dalam-3-bulan-ini-perubahannya</t>
+        </is>
+      </c>
+      <c r="H840" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/cepEmntAKDHO6SS1JIcGlTjHW6c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/selongsong-bom-serangan-udara-Israel-di-Suriah.jpg</t>
+        </is>
+      </c>
+      <c r="I840" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Kebakaran Hutan dan Lahan Meluas, Pemerintah Minta Masyarakat Tingkatkan Kewaspadaan</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:04:34 +0700</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>Pemerintah berharap kewaspadaan masyarakat dapat membantu mencegah munculnya titik api baru.</t>
+        </is>
+      </c>
+      <c r="F841" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G841" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866501/kebakaran-hutan-dan-lahan-meluas-pemerintah-minta-masyarakat-tingkatkan-kewaspadaan</t>
+        </is>
+      </c>
+      <c r="H841" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/j2S7gAqYm6hUyXDc9EsEv3NLcUc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Karhutla-Bromo-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I841" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Jelang HUT ke-81 RI, Pemerintah Siapkan Bantuan Beras Tahap II untuk 33,24 Juta KPM</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:01:17 +0700</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>Pemerintah akan kembali menyalurkan Bantuan Pangan Beras Tahap II kepada 33,24 juta keluarga penerima manfaat (KPM) di seluruh Indonesia.</t>
+        </is>
+      </c>
+      <c r="F842" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G842" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866500/jelang-hut-ke-81-ri-pemerintah-siapkan-bantuan-beras-tahap-ii-untuk-3324-juta-kpm</t>
+        </is>
+      </c>
+      <c r="H842" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Sn2AzBvrauTN9Mxi4xaVbPHeLE8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-beras-di-gudang.jpg</t>
+        </is>
+      </c>
+      <c r="I842" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Transportasi Kepulauan Seribu Beralih ke TransJakarta, Fahira Soroti 6 Hal Ini</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:01:00 +0700</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>Tantangan utama transportasi Kepulauan Seribu adalah memastikan warga memperoleh layanan publik yang setara dengan masyarakat di wilayah lainnya</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866499/transportasi-kepulauan-seribu-beralih-ke-transjakarta-fahira-soroti-6-hal-ini</t>
+        </is>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/VW5HtMPTQmzbHprUzB8VxR5P0a4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/fahiraidris111111.jpg</t>
+        </is>
+      </c>
+      <c r="I843" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Flores Besok Selasa 11 Agustus 2026: Bajawa Diprediksi Kabut Asap</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:00:08 +0700</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>Berikut detail prakiraan cuaca di beberapa kota terkenal di Flores untuk Selasa (11/8/2026) dilansir dari BMKG.</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866498/prakiraan-cuaca-flores-besok-selasa-11-agustus-2026-bajawa-diprediksi-kabut-asap</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/OhzEZi8-TThzoLbcoQWSjHOkPjE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pantai-pink-pulau-komodo-labuan-bajo-manggarai-barat-ntt.jpg</t>
+        </is>
+      </c>
+      <c r="I844" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>43.805 Pekerja Kena PHK Januari-Juli 2026, Terbanyak di Jabar</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:59:44 +0700</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>Sebanyak 43 ribu lebih pekerja di Indonesia harus menghadapi pemutusan hubungan kerja (PHK) sepanjang Januari-Juli 2026.</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866497/43805-pekerja-kena-phk-januari-juli-2026-terbanyak-di-jabar</t>
+        </is>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/fI4dy5xULfqtZz8Z5nhadxzCVNI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/angka-phk-di-jabar232.jpg</t>
+        </is>
+      </c>
+      <c r="I845" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Pulihkan Pasokan Semen di Aceh, SMGR Optimalisasi Produksi dan Distribusi</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:57:07 +0700</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>SMGR tetap berupaya maksimal dalam menjaga ketersediaan produk di berbagai titik penjualan walaupun perusahaan tengah mengalami tekanan</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7866496/pulihkan-pasokan-semen-di-aceh-smgr-optimalisasi-produksi-dan-distribusi</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/twtsLeG6muRZCGg9ncrkUqlVtBA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SMGR-pasokan-semen-Aceh.jpg</t>
+        </is>
+      </c>
+      <c r="I846" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Mengenal Gejala Superflu, Lengkap dengan Penyebab dan Cara Mencegahnya</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:55:13 +0700</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>Superflu merupakan istilah yang dikaitkan dengan influenza, berikut gejala, faktor penyebab, hingga cara mencegahnya berikut ini.</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866495/mengenal-gejala-superflu-lengkap-dengan-penyebab-dan-cara-mencegahnya</t>
+        </is>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/yvYBk7Mj-zTlRR51mwpwa8LWo7E=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Cek-kesehatan-gratis-di-Colomadu-Tohudan.jpg</t>
+        </is>
+      </c>
+      <c r="I847" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Israel Tolak Penarikan Pasukan Sebelum Hamas Dilucuti, Rencana Damai Gaza Terancam</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:54:30 +0700</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>Pemerintah Israel menilai penarikan pasukan sebelum pelucutan senjata selesai dapat menciptakan risiko keamanan baru.</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866494/israel-tolak-penarikan-pasukan-sebelum-hamas-dilucuti-rencana-damai-gaza-terancam</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/67KE1S1-igdGhTGm1JEcCY0c8Uk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ANGGOTA-BRIGADE-AL-QASSAM-wr24324234234.jpg</t>
+        </is>
+      </c>
+      <c r="I848" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>ABK Indonesia Berusia 20 Tahun Hilang, Diduga Jatuh dari Kapal Kontainer di Perairan Ehime Jepang</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:52:19 +0700</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>ABK Indonesia berusia 20 tahun hilang diduga jatuh ke laut dari kapal kontainer di lepas pantai Ehime, Jepang. Tim SAR masih mencari</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866493/abk-indonesia-berusia-20-tahun-hilang-diduga-jatuh-dari-kapal-kontainer-di-perairan-ehime-jepang</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/GYWEhOLACcBdVWWBSG7xROAPsa4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/tkptenggelam1111.jpg</t>
+        </is>
+      </c>
+      <c r="I849" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Nasib Tian Ngantung Pembalap Drag Race Tabrak Penonton hingga 8 Orang Tewas, Wajah Dipenuhi Perban</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:52:09 +0700</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>Drag race di Kotamobagu berujung maut, mobil pembalap menabrak penonton hingga 8 orang tewas dan 9 lainnya terluka.</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866492/nasib-tian-ngantung-pembalap-drag-race-tabrak-penonton-hingga-8-orang-tewas-wajah-dipenuhi-perban</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/AXdgAr9Iw3PgL4auFlOtiwlS1HI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kecelakaan-Drag-Race-dan-Drag-Bike-di-kotamobagu.jpg</t>
+        </is>
+      </c>
+      <c r="I850" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Malang-Batu Besok, Selasa 11 Agustus 2026: Batu Lebih Dingin, Malang 30 Derajat</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:47:23 +0700</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>Cuaca Malang dan Batu besok diprakirakan cerah berkabut hingga udara kabur, suhu Malang mencapai 30 derajat Celsius.</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G851" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866491/prakiraan-cuaca-malang-batu-besok-selasa-11-agustus-2026-batu-lebih-dingin-malang-30-derajat</t>
+        </is>
+      </c>
+      <c r="H851" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/eu4A6cMigDB3AsrpfAl0TfCYo68=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/alun-alun-kota-malang-april-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I851" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Jelang HUT ke-81 RI, Istana Pastikan Aman, TNI Wanti-wanti Hoaks</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:45:51 +0700</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>Jelang HUT ke-81 RI, Istana memastikan pengamanan siap. Panglima TNI mengingatkan warga mewaspadai hoaks dan isu provokatif.</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866490/jelang-hut-ke-81-ri-istana-pastikan-aman-tni-wanti-wanti-hoaks</t>
+        </is>
+      </c>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/b9Hcqv7iS4vvK6LuL2i9t4rjFXQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Presiden-Prabowo-Subianto-Gibran-Rakabuming-Prasetyo-Hadi-Muhaimin-Iskandar-di-Halim.jpg</t>
+        </is>
+      </c>
+      <c r="I852" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Kuasa Hukum Febrie Adriansyah Minta Kejagung RI Tak Hindari Sidang Gugatan Praperadilan</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:44:39 +0700</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>Kejagung RI selaku salah satu termohon dalam gugatan praperadilan Febrie Adriansyah diminta untuk bersedia hadir di persidangan.</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866489/kuasa-hukum-febrie-adriansyah-minta-kejagung-ri-tak-hindari-sidang-gugatan-praperadilan</t>
+        </is>
+      </c>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/eQh7NUBPd1a5LZJ7hmRGe9FD4wA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Febrie-Adriansyah-Jalani-Pemeriksaan-Lanjutan-Kasus-TPPU_20260807_134205.jpg</t>
+        </is>
+      </c>
+      <c r="I853" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Destry Calon Tunggal Gubernur BI, Airlangga Beri Komentar Tak Terduga</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:25:54 +0700</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>Airlangga Hartanto buka suara soal Destry Damayanti menjadi calon tunggal Gubernur definitif Bank Indonesia (BI).</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810181654-17-758058/destry-calon-tunggal-gubernur-bi-airlangga-beri-komentar-tak-terduga</t>
+        </is>
+      </c>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/06/aimenteri-koordinator-bidang-perekonomian-airlangga-hartarto-pada-konferensi-pers-di-jakarta-rabu-582026-1785971442706_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I854" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Jelang Review MSCI Agustus 2026, OJK Bilang Gini</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>OJK berharap MSCI mencabut pembekuan saham Indonesia dalam tinjauan 12 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G855" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810170312-17-758042/jelang-review-msci-agustus-2026-ojk-bilang-gini</t>
+        </is>
+      </c>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2022/07/15/ilustrasi-bursa-cnbc-indonesiaandrean-kristianto-4_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I855" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Efek 'Sulap' Prabowo, Valuasi Emiten BUMN Ini Melonjak Drastis</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:52:46 +0700</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>PT Timah Tbk (TINS) mencatat laba usaha Rp3,48 triliun di Semester I 2026, meningkat signifikan. Target produksi logam hingga 25.000 ton diharapkan tercapai.</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810183732-17-758071/efek-sulap-prabowo-valuasi-emiten-bumn-ini-melonjak-drastis</t>
+        </is>
+      </c>
+      <c r="H856" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/08/25/timah-balok-siap-jual-cnbc-indonesiafirda-dwi-muliawati-1756098257458_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I856" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Danantara Bisa Jadi Pemegang Saham BEI, OJK Masih Godok Aturan</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:10:00 +0700</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>OJK mengungkap rencana demutualisasi BEI dan keterlibatan BPI Danantara sebagai pemegang saham.</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810145436-17-757986/danantara-bisa-jadi-pemegang-saham-bei-ojk-masih-godok-aturan</t>
+        </is>
+      </c>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/03/26/ilustrasi-ojk-cnbc-indonesiafaisal-rahman-1_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I857" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Bukan Cuma Uang, Wakaf di Istiqlal Bisa Berupa Saham</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:55:10 +0700</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>Bursa Efek Indonesia memperkenalkan program wakaf dan sedekah melalui pasar modal, termasuk saham dan reksa dana, untuk mendukung filantropi Islam.</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810142935-17-757976/bukan-cuma-uang-wakaf-di-istiqlal-bisa-berupa-saham</t>
+        </is>
+      </c>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/30/layar-menampilkan-pergerakan-indeks-harga-saham-gabungan-ihsg-di-bursa-efek-indonesia-bei-jakarta-selasa-3062026-1782797019885_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I858" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Tantangan Besar Destry-Calon Gubernur BI di Tengah Gejolak Global</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:25:06 +0700</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>Destry Damayanti menjadi calon tunggal Gubernur Bank Indonesia (BI) pilihan Presiden Prabowo Subianto.</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810143206-17-757969/tantangan-besar-destry-calon-gubernur-bi-di-tengah-gejolak-global</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2019/08/07/5771d0f6-119c-445f-808c-6c2f636386f8_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I859" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Video: Calon Tunggal Gubernur BI hingga IHSG Anjlok Lagi ke 6.300-an</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:22:24 +0700</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>Calon Tunggal Gubernur BI hingga IHSG Anjlok Lagi ke Level 6.300-an</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810165854-19-758037/video-calon-tunggal-gubernur-bi-hingga-ihsg-anjlok-lagi-ke-6300-an</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/10/calon-tunggal-gubernur-bi-hingga-ihsg-anjlok-lagi-ke-level-6300-an-1786357244157_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I860" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Video: Sinyal Suku Bunga Tinggi BI dan The Fed, Bos MI Ungkap Efeknya</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 16:58:12 +0700</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>Sinyal Suku Bunga Tinggi BI dan The Fed, Bos MI Ungkap Efeknya IHSG hingga SBN</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810155822-19-758002/video-sinyal-suku-bunga-tinggi-bi-the-fed-bos-mi-ungkap-efeknya</t>
+        </is>
+      </c>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/10/sinyal-suku-bunga-tinggi-bi-the-fed-bos-mi-ungkap-efeknya-ihsg-hingga-sbn-1786352623714_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I861" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>IHSG Ambruk 0,69%, Dua Saham Ini Jadi Beban</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 16:35:17 +0700</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>IHSG ditutup melemah di level 6.365,37 pada hari ini, Senin (10/8/2026).</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810161653-17-758017/ihsg-ambruk-069-dua-saham-ini-jadi-beban</t>
+        </is>
+      </c>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/05/19/ilustrasi-orang-berdoa-dengan-latar-belakang-bursa-saham-indonesia-di-bursa-efek-indonesia-jakarta-selasa-1952026-1779182674119_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I862" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Video: Prabowo Usul Destry Jadi Gubernur BI, Pasar Respons Begini</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 16:14:57 +0700</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>Prabowo Usulkan Destry Damayanti Jadi Gubernur BI, Pasar Respon Positif</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G863" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810160015-19-758003/video-prabowo-usul-destry-jadi-gubernur-bi-pasar-respons-begini</t>
+        </is>
+      </c>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/10/prabowo-usulkan-destry-damayanti-jadi-gubernur-bi-pasar-respon-positif-1786352735826_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I863" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Universitas Tempatkan Dana di Sukuk Negara: Hasilkan Beasiswa-Riset</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 15:50:10 +0700</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>Kementerian Keuangan (Kemenkeu) mengungkapkan manfaat dari surat berharga syariah negara (SBSN) atau Sukuk Negara</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810132119-17-757937/universitas-tempatkan-dana-di-sukuk-negara-hasilkan-beasiswa-riset</t>
+        </is>
+      </c>
+      <c r="H864" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/05/22/direktur-pembiayaan-syariah-djppr-kementerian-keuangan-deni-ridwan-saat-menyampaikan-pemaparan-dalam-sesi-educational-class-di-1779456376570_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I864" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Duit Investor Menguap, SpaceX Bakar Rp288 T Cuma buat AI</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 15:45:32 +0700</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>Elon Musk mengalami momen tak terduga saat roket SpaceX menghantam Bulan. Pendapatan SpaceX melonjak, namun kerugian tetap membayangi.</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G865" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810153232-17-757992/duit-investor-menguap-spacex-bakar-rp288-t-cuma-buat-ai</t>
+        </is>
+      </c>
+      <c r="H865" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/02/13/roket-spacex-falcon-9-dan-pesawat-ruang-angkasa-dragon-lepas-landas-dalam-misi-crew-12-nasa-ke-stasiun-luar-angkasa-internasio-1770990649346_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I865" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Danantara Mau Bawa BUMN Melantai di BEI, Pandu: Buat Tambah Likuiditas</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 15:43:28 +0700</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>BPI Danantara rencanakan IPO sejumlah BUMN di BEI untuk meningkatkan likuiditas pasar. Perusahaan seperti Pelindo dan Angkasa Pura akan dilibatkan.</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G866" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810154057-17-757995/danantara-mau-bawa-bumn-melantai-di-bei-pandu-buat-tambah-likuiditas</t>
+        </is>
+      </c>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/12/19/chief-investment-officer-cio-danantara-pandu-sjahrir-menyampaikan-paparan-dalam-acara-big-alpha-business-summit-2025-di-jakart-1766116798744_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I866" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>OJK Bakal Punya Bos Baru, Prabowo Hari Ini Kirim Surpres ke DPR</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 15:30:03 +0700</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>Pemerintah memperluas kewenangan OJK untuk mengawasi Bursa Mineral dan Komoditas Strategis mulai 2027.</t>
+        </is>
+      </c>
+      <c r="F867" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G867" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810140608-17-757952/ojk-bakal-punya-bos-baru-prabowo-hari-ini-kirim-surpres-ke-dpr</t>
+        </is>
+      </c>
+      <c r="H867" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/03/26/ilustrasi-ojk-cnbc-indonesiafaisal-rahman-2_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I867" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>BRI Perkuat Pembiayaan Perumahan dalam Danantara Housing Expo 2026</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 15:14:15 +0700</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>Danantara Housing Expo 2026 hadir untuk mendukung Program 3 Juta Rumah, menawarkan 200.000 unit hunian dan solusi pembiayaan</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G868" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810150534-17-757988/bri-perkuat-pembiayaan-perumahan-dalam-danantara-housing-expo-2026</t>
+        </is>
+      </c>
+      <c r="H868" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/10/danantara-housing-expo-1786349470824_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I868" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Rupiah Menguat 4 Hari Beruntun, Dolar AS Turun ke Rp17.750</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 15:06:00 +0700</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>Nilai tukar rupiah berhasil menutup perdagangan awal pekan dengan penguatan tajam melawan dolar Amerika Serikat (AS).</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G869" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810144853-17-757977/rupiah-menguat-4-hari-beruntun-dolar-as-turun-ke-rp17750</t>
+        </is>
+      </c>
+      <c r="H869" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/09/25/petugas-menjunjukkan-mata-uang-dolar-amerika-serikat-as-dan-rupiah-di-vip-money-changer-jakarta-kamis-2592025-1758794525604_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I869" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Video: Transaksi Bursa Berjangka Diramal Masih Bisa Naik 60% di 2026</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 14:53:55 +0700</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>Volatilitas Masih Tinggi, Transaksi Bursa Berjangka 2026 Diramal Masih Bisa Naik 60%</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G870" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810141600-19-757957/video-transaksi-bursa-berjangka-diramal-masih-bisa-naik-60-di-2026</t>
+        </is>
+      </c>
+      <c r="H870" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/10/perdagangan-perak-saham-as-di-bursa-berjangka-kian-marak-di-2026-apa-pendorongnya-1786347672100_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I870" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Airlangga dan Bos Pajak Pertimbangkan Potensi Pajak ETF Emas Direvisi</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 14:45:35 +0700</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>Menko Airlangga Hartarto koordinasi dengan Kemenkeu terkait revisi pajak untuk Electronic Gold Receipt. Harapannya, transaksi ETF emas meningkat.</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G871" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810122756-17-757914/airlangga-bos-pajak-pertimbangkan-potensi-pajak-etf-emas-direvisi</t>
+        </is>
+      </c>
+      <c r="H871" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/10/menko-pereknomian-airlangga-hartarto-saat-acara-peringatan-hut-ke-49-pasar-modal-indonesia-dan-peluncuran-produk-etf-emas-seni-1786330817178_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I871" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Awas! Michael Burry Wanti-wanti Crash 1987 Terulang Lagi</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 14:35:03 +0700</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>Investor legendaris Michael Burry tetap bertahan dengan posisi jual meski SdanP 500 mencetak rekor. Ia peringatkan potensi kejatuhan pasar seperti 1987.</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G872" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810131347-17-757934/awas-michael-burry-wanti-wanti-crash-1987-terulang-lagi</t>
+        </is>
+      </c>
+      <c r="H872" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/05/11/michael-burry-dimitrios-kambouris-getty-images-north-america-getty-images-via-afp-1778480233916_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I872" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Video: Rupiah Makin Perkasa dan Menguat ke Rp 17.700-an per Dolar AS</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 14:34:49 +0700</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>Rupiah Makin Perkasa dan Menguat ke Rp 17.700-an per Dolar AS</t>
+        </is>
+      </c>
+      <c r="F873" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G873" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810142639-19-757965/video-rupiah-makin-perkasa-menguat-ke-rp-17700-an-per-dolar-as</t>
+        </is>
+      </c>
+      <c r="H873" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/10/rupiah-makin-perkasa-menguat-ke-rp-17700-an-per-dolar-as-1786347234430_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I873" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Airlangga Soroti Pajak 'PPN dan PPh' dari Transaksi EGR</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 14:15:47 +0700</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>Menko Airlangga Hartarto dorong perlakuan pajak untuk transaksi Electronic Gold Receipt (EGR) guna pengembangan ETF emas di Indonesia.</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G874" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810135234-17-757950/airlangga-soroti-pajak-ppn-dan-pph-dari-transaksi-egr</t>
+        </is>
+      </c>
+      <c r="H874" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/10/menko-pereknomian-airlangga-hartarto-saat-acara-peringatan-hut-ke-49-pasar-modal-indonesia-dan-peluncuran-produk-etf-emas-seni-1786330817178_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I874" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Video: ETF Emas Resmi Diluncurkan, Wamenkeu Titip Tiga Pesan</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 14:15:03 +0700</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>ETF Emas Resmi Diluncurkan, Wamenkeu Titip Tiga Pesan</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G875" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810124636-19-757918/video-etf-emas-resmi-diluncurkan-wamenkeu-titip-tiga-pesan</t>
+        </is>
+      </c>
+      <c r="H875" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/10/etf-emas-resmi-diluncurkan-wamenkeu-titip-tiga-pesan-1786344716395_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I875" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Perubahan Teknologi Makin Cepat, Perusahaan IT Genjot Adaptasi AI</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:31:39 +0700</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Perkembangan teknologi yang semakin cepat mendorong perusahaan teknologi informasi (IT) memperkuat kemampuan adaptasi, terutama dalam menghadapi perkembangan artificial intelligence (AI). Perubahan yang sebelumnya berlangsung dalam hitungan tahun...</t>
+        </is>
+      </c>
+      <c r="F876" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G876" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjk04r416/perubahan-teknologi-makin-cepat-perusahaan-it-genjot-adaptasi-ai</t>
+        </is>
+      </c>
+      <c r="H876" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/kecerdasan-buatan-atau-ai-ilustrasi-lebih-dari-200-tokoh_250924111739-212.jpg</t>
+        </is>
+      </c>
+      <c r="I876" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Pembangunan Tol Layang Ancol Timur-Pluit Capai 44,12 Persen, Ditargetkan Beroperasi 2028</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Pembangunan Jalan Tol Harbour Road II (HBR II) terus berjalan dengan progres konstruksi mencapai 44,12 persen per awal Agustus 2026. Ruas tol layang Ancol Timur-Pluit tersebut ditargetkan...</t>
+        </is>
+      </c>
+      <c r="F877" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G877" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjjsfd416/pembangunan-tol-layang-ancol-timurpluit-capai-4412-persen-ditargetkan-beroperasi-2028</t>
+        </is>
+      </c>
+      <c r="H877" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260810164713-634.png</t>
+        </is>
+      </c>
+      <c r="I877" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Bigmo Dicecar 40 Pertanyaan, Akui Salah Promosi Vape Ajak Anak</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:28:14 +0700</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>Bigmo menjalani pemeriksaan selama sekitar empat jam.</t>
+        </is>
+      </c>
+      <c r="F878" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G878" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266554/bigmo-dicecar-40-pertanyaan-akui-salah-promosi-vape-ajak-anak</t>
+        </is>
+      </c>
+      <c r="H878" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/fU5Qq94_Eb5gSrPjGZ_wg7oj-oc=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320661/original/015938000_1786364749-71853.jpg</t>
+        </is>
+      </c>
+      <c r="I878" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Menko Polkam ke Pangdam dan Kapolda: Karhutla Tentukan Karier Anda</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:17:33 +0700</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>Menurut Djamari, keberhasilan penanganan karhutla diukur dari kemampuan aparat mengendalikan titik api.</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G879" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266551/menko-polkam-ke-pangdam-dan-kapolda-karhutla-tentukan-karier-anda</t>
+        </is>
+      </c>
+      <c r="H879" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/v65nxNPh494cmWMnnl7ST70epHM=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320658/original/015286800_1786364252-IMG_8200.jpeg</t>
+        </is>
+      </c>
+      <c r="I879" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Strategi Pemerintah Cegah Asap Karhutla Menyebar ke Negara Tetangga</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:09:25 +0700</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>Pemerintah pun menanti kemunculan awan hujan untuk menjalankan Operasi Modifikasi Cuaca (OMC).</t>
+        </is>
+      </c>
+      <c r="F880" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G880" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266548/strategi-pemerintah-cegah-asap-karhutla-menyebar-ke-negara-tetangga</t>
+        </is>
+      </c>
+      <c r="H880" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/drley7BU6pBcGwJIxbChDJ5cnqM=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320657/original/072138100_1786363761-IMG_8202.jpeg</t>
+        </is>
+      </c>
+      <c r="I880" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>BPA Gelar Lelang Serentak: Limit Terendah Rp 3 Ribu, Tertinggi Rp 9,1 Miliar</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:05:26 +0700</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>Setiap rupiah yang berhasil dipulihkan BPA Kejaksaan merupakan hak negara dan masyarakat yang wajib dikembalikan.</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G881" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266544/bpa-gelar-lelang-serentak-limit-terendah-rp-3-ribu-tertinggi-rp-91-miliar</t>
+        </is>
+      </c>
+      <c r="H881" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/95nxxVphs6VNs9nq8KsRTLg5sE0=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320656/original/022231000_1786363519-WhatsApp_Image_2026-08-10_at_16.13.38.jpeg</t>
+        </is>
+      </c>
+      <c r="I881" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Karhutla Meluas, 107.000 Hektare Lahan di Indonesia Terbakar</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:39:27 +0700</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>Fenomena El Nino atau kemarau yang melanda Indonesia saat ini mempercepat terjadinya kebakaran hutan dan lahan (karhutla).</t>
+        </is>
+      </c>
+      <c r="F882" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G882" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266493/karhutla-meluas-107000-hektare-lahan-di-indonesia-terbakar</t>
+        </is>
+      </c>
+      <c r="H882" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/52ERORkc0kbwgpNk-Zs71NbkIyk=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320558/original/015050400_1786355841-men6.jpg</t>
+        </is>
+      </c>
+      <c r="I882" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Panglima TNI Minta Warga Tak Terprovokasi Isu Medsos</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:19:15 +0700</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>Panglima TNI Jenderal Agus Subiyanto menegaskan keamanan nasional tetap terjaga pasca rapat dengan pimpinan DPR.</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G883" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266124/panglima-tni-minta-warga-tak-terprovokasi-isu-medsos</t>
+        </is>
+      </c>
+      <c r="H883" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/rD3ueMTqt3nI5n9Y9DV2HbCXMo0=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320239/original/070492200_1786341140-c57a18a3-9595-4171-9ddf-5e5fedc25804.jpg</t>
+        </is>
+      </c>
+      <c r="I883" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>KPK Tahan 4 Tersangka Kasus Pengadaan Iklan Bank BJB</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:44:32 +0700</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>KPK menahan 4 tersangka kasus korupsi pengadaan iklan fiktif di Bank BJB yang merugikan negara Rp 222 miliar, satu tersangka lain belum ditahan.</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G884" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/10/19435331/kpk-tahan-4-tersangka-kasus-pengadaan-iklan-bank-bjb</t>
+        </is>
+      </c>
+      <c r="H884" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/469bCMWHgGRvW4sa8pM0mm9-QYY=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/10/6a79c41e45066.jpeg</t>
+        </is>
+      </c>
+      <c r="I884" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Dua JPO Tak Terintegrasi di Rasuna, Ketika Kepentingan Berbeda Bertemu di Satu Kawasan</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:44:32 +0700</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>Dua JPO di Rasuna tak terintegrasi meski berdiri berdekatan. Pengamat menilai perbedaan aset dan kepentingan jadi tantangan.</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G885" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/10/19231931/dua-jpo-tak-terintegrasi-di-rasuna-ketika-kepentingan-berbeda-bertemu-di</t>
+        </is>
+      </c>
+      <c r="H885" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/P807KvISkgYTpCrYkWD_L6vlU6M=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/04/6a716628f297a.jpg</t>
+        </is>
+      </c>
+      <c r="I885" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>China-Rusia Langsung "Melek" Saat Amunisi AS Terkuras di Perang Iran</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:44:32 +0700</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>Rangkaian pengeboman dan operasi pertahanan Amerika selama lebih dari 5 bulan melawan Iran menguras ribuan rudal presisi bernilai jutaan dollar AS.</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G886" t="inlineStr">
+        <is>
+          <t>https://internasional.kompas.com/read/2026/08/10/190000870/china-rusia-langsung-melek-saat-amunisi-as-terkuras-di-perang-iran</t>
+        </is>
+      </c>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/lYO_7LPMZNLZPppdjChIiVnV0pI=/0x0:2000x1333/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/10/6a7972125450a.jpg</t>
+        </is>
+      </c>
+      <c r="I886" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I794"/>
+  <autoFilter ref="A1:I886"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 15:51 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1067</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1140</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1067"/>
+  <dimension ref="A1:I1140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -50588,8 +50588,3439 @@
         </is>
       </c>
     </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>Bupati sebut Transjakarta permudah mobilitas warga kepulauan</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:43:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1068" t="inlineStr">
+        <is>
+          <t>Bupati Kepulauan Seribu Muhammad Fadjar Churniawan mengatakan kehadiran PT Transjakarta yang menggantikan Dinas ...</t>
+        </is>
+      </c>
+      <c r="F1068" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1068" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688273/bupati-sebut-transjakarta-permudah-mobilitas-warga-kepulauan</t>
+        </is>
+      </c>
+      <c r="H1068" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/12/1000303145.jpg</t>
+        </is>
+      </c>
+      <c r="I1068" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>Kemenimipas usulkan pemberian amensti HUT RI ke Presiden</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:40:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1069" t="inlineStr">
+        <is>
+          <t>Kementerian Imigrasi dan Pemasyarakatan (Kemenimipas) mengusulkan pemberian amnesti bagi warga binaan pemasyarakatan ...</t>
+        </is>
+      </c>
+      <c r="F1069" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1069" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688269/kemenimipas-usulkan-pemberian-amensti-hut-ri-ke-presiden</t>
+        </is>
+      </c>
+      <c r="H1069" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000013001.jpg</t>
+        </is>
+      </c>
+      <c r="I1069" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>Kepuasan jamaah haji naik Qodari sebut bukti perbaikan layanan</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:37:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1070" t="inlineStr">
+        <is>
+          <t>Kepala Badan Komunikasi Pemerintah (Bakom) RI Muhammad Qodari menilai peningkatan kepuasan jamaah haji Indonesia pada ...</t>
+        </is>
+      </c>
+      <c r="F1070" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1070" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688265/kepuasan-jamaah-haji-naik-qodari-sebut-bukti-perbaikan-layanan</t>
+        </is>
+      </c>
+      <c r="H1070" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/02/kedatangan-jamaah-haji-kloter-pertama-debarkasi-medan-2797785.jpg</t>
+        </is>
+      </c>
+      <c r="I1070" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>Nusron: Percepatan layanan dan integrasi data tutup celah mafia tanah</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:35:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1071" t="inlineStr">
+        <is>
+          <t>Menteri Agraria dan Tata Ruang/Kepala Badan Pertanahan Nasional (ATR/BPN) Nusron Wahid mengatakan percepatan pelayanan ...</t>
+        </is>
+      </c>
+      <c r="F1071" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1071" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688261/nusron-percepatan-layanan-dan-integrasi-data-tutup-celah-mafia-tanah</t>
+        </is>
+      </c>
+      <c r="H1071" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000583340.jpg</t>
+        </is>
+      </c>
+      <c r="I1071" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>Dompet dhuafa bantu air bersih untuk 370 warga Boyolali dan Grobogan</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:34:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1072" t="inlineStr">
+        <is>
+          <t>Dompet Dhuafa Jawa Tengah melakukan distribusi air bersih kepada 370 warga di Kabupaten Boyolali dan Grobogan, Jawa ...</t>
+        </is>
+      </c>
+      <c r="F1072" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1072" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688260/dompet-dhuafa-bantu-air-bersih-untuk-370-warga-boyolali-dan-grobogan</t>
+        </is>
+      </c>
+      <c r="H1072" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/dhompet-dhuafa.jpg</t>
+        </is>
+      </c>
+      <c r="I1072" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>Bupati: Peringatan HUT RI mementum percepat pembangunan</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:31:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1073" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1073" t="inlineStr">
+        <is>
+          <t>Bupati Kepulauan Seribu, Muhammad Fadjar Churniawan mengatakan peringatan HUT ke-81 Republik Indonesia merupakan ...</t>
+        </is>
+      </c>
+      <c r="F1073" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1073" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688256/bupati-peringatan-hut-ri-mementum-percepat-pembangunan</t>
+        </is>
+      </c>
+      <c r="H1073" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_4804.jpeg</t>
+        </is>
+      </c>
+      <c r="I1073" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>Gempa bumi di Kolombia runtuhkan 19 bangunan di Kota Cali</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:27:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1074" t="inlineStr">
+        <is>
+          <t>Gempa bumi di Kolombia bagian barat pada Senin menyebabkan runtuhnya 19 bangunan di Kota Cali, di negara itu, menurut ...</t>
+        </is>
+      </c>
+      <c r="F1074" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1074" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688255/gempa-bumi-di-kolombia-runtuhkan-19-bangunan-di-kota-cali</t>
+        </is>
+      </c>
+      <c r="H1074" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/ilustrasi-gempa-3.jpg</t>
+        </is>
+      </c>
+      <c r="I1074" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>LPDB tegaskan pengajuan dana bergulir koperasi gratis bisa dipantau</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:26:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1075" t="inlineStr">
+        <is>
+          <t>Lembaga Pengelola Dana Bergulir (LPDB) Koperasi menegaskan pengajuan pembiayaan dana bergulir bagi koperasi tidak ...</t>
+        </is>
+      </c>
+      <c r="F1075" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1075" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688252/lpdb-tegaskan-pengajuan-dana-bergulir-koperasi-gratis-bisa-dipantau</t>
+        </is>
+      </c>
+      <c r="H1075" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/WhatsApp-Image-2026-08-10-at-14.23.33.jpeg</t>
+        </is>
+      </c>
+      <c r="I1075" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>IPB rakit 4 varietas habanero, tingkat kepedasan tembus 1,3 juta SHU</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:25:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1076" t="inlineStr">
+        <is>
+          <t>ANTARA - Institut Pertanian Bogor (IPB) University merakit empat varietas cabai habanero lokal pertama di ...</t>
+        </is>
+      </c>
+      <c r="F1076" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1076" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5688228/ipb-rakit-4-varietas-habanero-tingkat-kepedasan-tembus-13-juta-shu</t>
+        </is>
+      </c>
+      <c r="H1076" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_39_59_08.Still485.jpg</t>
+        </is>
+      </c>
+      <c r="I1076" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>Wali kota minta Kwarcab Medan jadikan Jamnas sarana membangun karakter</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:22:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1077" t="inlineStr">
+        <is>
+          <t>Wali Kota Rico Tri Putra Waas meminta kontingen Kwartir Cabang (Kwarcab) Gerakan Pramuka Kota Medan memanfaatkan ...</t>
+        </is>
+      </c>
+      <c r="F1077" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1077" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688251/wali-kota-minta-kwarcab-medan-jadikan-jamnas-sarana-membangun-karakter</t>
+        </is>
+      </c>
+      <c r="H1077" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000108483.jpg</t>
+        </is>
+      </c>
+      <c r="I1077" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>Modal asing 5,9 miliar dolar AS, Indonesia masih jadi tujuan investasi</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:22:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1078" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1078" t="inlineStr">
+        <is>
+          <t>Permata Institute for Economic Research (PIER) mencatat arus modal asing ke Indonesia sepanjang Januari hingga awal ...</t>
+        </is>
+      </c>
+      <c r="F1078" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1078" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688248/modal-asing-59-miliar-dolar-as-indonesia-masih-jadi-tujuan-investasi</t>
+        </is>
+      </c>
+      <c r="H1078" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/10/27/realisasi-investasi-triwulan-iii-di-sumut-2654605.jpg</t>
+        </is>
+      </c>
+      <c r="I1078" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>Pemkab Kulon Progo komitmen tidak ada pemecatan PPPK di tengah kontrak</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:17:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1079" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1079" t="inlineStr">
+        <is>
+          <t>Pemerintah Kabupaten Kulon Progo, Daerah Istimewa Yogyakarta, menegaskan komitmennya untuk tidak melakukan pemutusan ...</t>
+        </is>
+      </c>
+      <c r="F1079" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1079" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688245/pemkab-kulon-progo-komitmen-tidak-ada-pemecatan-pppk-di-tengah-kontrak</t>
+        </is>
+      </c>
+      <c r="H1079" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000047421.jpg</t>
+        </is>
+      </c>
+      <c r="I1079" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>KPK tahan tersangka korupsi pengadaan iklan Bank BJB</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:12:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1080" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1080" t="inlineStr">
+        <is>
+          <t>Pemimpin Divisi Change Management Office Bank BJB sekaligus eks Pemimpin Divisi Corporate Secretary Bank BJB ...</t>
+        </is>
+      </c>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1080" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5688244/kpk-tahan-tersangka-korupsi-pengadaan-iklan-bank-bjb</t>
+        </is>
+      </c>
+      <c r="H1080" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/KPK-tahan-tersangka-kasus-korupsi-pengadaan-iklan-Bank-BJB-100826-fzn-6.jpg</t>
+        </is>
+      </c>
+      <c r="I1080" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>Ahli sebut kerugian negara tak cukup buktikan seseorang korupsi</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:12:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1081" t="inlineStr">
+        <is>
+          <t>Ahli hukum pidana Universitas Kristen Indonesia Prof. Mompang Panggabean mengatakan unsur kesalahan (mens rea) harus ...</t>
+        </is>
+      </c>
+      <c r="F1081" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1081" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688243/ahli-sebut-kerugian-negara-tak-cukup-buktikan-seseorang-korupsi</t>
+        </is>
+      </c>
+      <c r="H1081" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000479795.jpg</t>
+        </is>
+      </c>
+      <c r="I1081" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>Komisi VII soroti infrastruktur pariwisata berkelanjutan Gili Lombok</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:11:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1082" t="inlineStr">
+        <is>
+          <t>ANTARA -Komisi VII DPR RI menyoroti aspek infrastruktur di kawasan pariwisata Gili Meno, Lombok Utara, NTB. Dalam ...</t>
+        </is>
+      </c>
+      <c r="F1082" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1082" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5688213/komisi-vii-soroti-infrastruktur-pariwisata-berkelanjutan-gili-lombok</t>
+        </is>
+      </c>
+      <c r="H1082" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KOMISI-VII-SOROTI-INFRASTRUKTUR-PARIWISATA-BERKELANJUTAN-GILI-LOMBOK.jpg</t>
+        </is>
+      </c>
+      <c r="I1082" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>Melihat ritual cuci pusaka, tradisi adat di Kerajaan Mempawah</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:10:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1083" t="inlineStr">
+        <is>
+          <t>ANTARA - Kerajaan Mempawah menggelar ritual cuci pusaka di selasar Istana Amantubillah, Desa Pulau Pedalaman, Kecamatan ...</t>
+        </is>
+      </c>
+      <c r="F1083" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1083" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5688192/melihat-ritual-cuci-pusaka-tradisi-adat-di-kerajaan-mempawah</t>
+        </is>
+      </c>
+      <c r="H1083" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_35_32_25.Still483.jpg</t>
+        </is>
+      </c>
+      <c r="I1083" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>Perpres transportasi digital ditargetkan rampung pekan ini</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:10:08 +0700</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1084" t="inlineStr">
+        <is>
+          <t>Menteri Usaha Mikro, Kecil, dan Menengah (UMKM) Maman Abdurrahman mengatakan Peraturan Presiden (Perpres) tentang ...</t>
+        </is>
+      </c>
+      <c r="F1084" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1084" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688240/perpres-transportasi-digital-ditargetkan-rampung-pekan-ini</t>
+        </is>
+      </c>
+      <c r="H1084" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/15/raker-komisi-vii-dpr-dengan-menteri-umkm-2821908.jpg</t>
+        </is>
+      </c>
+      <c r="I1084" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>Polisi dalami kasus pria diduga tabrakkan diri ke kereta api di Jakut</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:09:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1085" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1085" t="inlineStr">
+        <is>
+          <t>Polsek Tanjung Priok mendalami kasus yang membuat pria berinisial A (36) nekat menabrakkan diri ke kereta api yang ...</t>
+        </is>
+      </c>
+      <c r="F1085" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1085" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688236/polisi-dalami-kasus-pria-diduga-tabrakkan-diri-ke-kereta-api-di-jakut</t>
+        </is>
+      </c>
+      <c r="H1085" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_4803.jpeg</t>
+        </is>
+      </c>
+      <c r="I1085" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>PIER: Konsumsi domestik perkuat ekonomi RI di tengah tekanan global</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:08:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1086" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1086" t="inlineStr">
+        <is>
+          <t>Permata Institute for Economic Research (PIER) menilai ekonomi Indonesia perlu semakin mengandalkan kekuatan domestik, ...</t>
+        </is>
+      </c>
+      <c r="F1086" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1086" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688233/pier-konsumsi-domestik-perkuat-ekonomi-ri-di-tengah-tekanan-global</t>
+        </is>
+      </c>
+      <c r="H1086" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000456822.jpg</t>
+        </is>
+      </c>
+      <c r="I1086" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>Kemensos berdayakan penerima bansos di Madura jadi petani ekspor cabai</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:07:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1087" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1087" t="inlineStr">
+        <is>
+          <t>Kementerian Sosial (Kemensos) melalui Direktorat Jenderal Pemberdayaan Sosial memberdayakan penerima bantuan sosial ...</t>
+        </is>
+      </c>
+      <c r="F1087" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1087" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688232/kemensos-berdayakan-penerima-bansos-di-madura-jadi-petani-ekspor-cabai</t>
+        </is>
+      </c>
+      <c r="H1087" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/203452.jpg</t>
+        </is>
+      </c>
+      <c r="I1087" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>Empat korban hilang dalam kecelakaan kapal di perairan Bintan</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:05:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1088" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1088" t="inlineStr">
+        <is>
+          <t>Kepala Kantor Pencarian dan Pertolongan (SAR) Tanjungpinang Fazzli menyebutkan empat korban dinyatakan hilang dalam ...</t>
+        </is>
+      </c>
+      <c r="F1088" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1088" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688229/empat-korban-hilang-dalam-kecelakaan-kapal-di-perairan-bintan</t>
+        </is>
+      </c>
+      <c r="H1088" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/inbound887734786127890032.jpg</t>
+        </is>
+      </c>
+      <c r="I1088" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>BPKP: Lingkungan pengendalian fondasi utama penyelenggaraan SPIP</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:00:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1089" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1089" t="inlineStr">
+        <is>
+          <t>Deputi Bidang Pengawasan Instansi Pemerintah Bidang Perekonomian, Infrastruktur, dan Pembangunan Kewilayahan (PIPK) ...</t>
+        </is>
+      </c>
+      <c r="F1089" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1089" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688224/bpkp-lingkungan-pengendalian-fondasi-utama-penyelenggaraan-spip</t>
+        </is>
+      </c>
+      <c r="H1089" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/BPKP-PPKD.jpg</t>
+        </is>
+      </c>
+      <c r="I1089" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>Jukir di Tambora diringkus polisi usai paksa pengendara bayar Rp5 ribu</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:58:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1090" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1090" t="inlineStr">
+        <is>
+          <t>Polisi meringkus seorang juru parkir berinisial MS di kawasan parkir Pasar Mitra, Jalan KH M Mansyur, Kelurahan ...</t>
+        </is>
+      </c>
+      <c r="F1090" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1090" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688221/jukir-di-tambora-diringkus-polisi-usai-paksa-pengendara-bayar-rp5-ribu</t>
+        </is>
+      </c>
+      <c r="H1090" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/25/Ilustrassi-penangkapan-pelaku.jpg</t>
+        </is>
+      </c>
+      <c r="I1090" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>Mantan pemain Indiana Pacers ditunjuk sebagai GM tim universitas</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:53:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1091" t="inlineStr">
+        <is>
+          <t>Mantan pemain Indiana Pacers, Monta Ellis, memulai babak baru kariernya sebagai general manager (GM) tim bola basket ...</t>
+        </is>
+      </c>
+      <c r="F1091" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1091" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688212/mantan-pemain-indiana-pacers-ditunjuk-sebagai-gm-tim-universitas</t>
+        </is>
+      </c>
+      <c r="H1091" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000478622.jpg</t>
+        </is>
+      </c>
+      <c r="I1091" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>Kereta Y404 jadi sarana widyawisata dan ruang lelas bergerak di China</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:52:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1092" t="inlineStr">
+        <is>
+          <t>Kereta khusus Y404 untuk widyawisata (study tour) yang mengangkut 598 guru dan murid pada Minggu (9/8) berangkat dari ...</t>
+        </is>
+      </c>
+      <c r="F1092" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1092" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688208/kereta-y404-jadi-sarana-widyawisata-dan-ruang-lelas-bergerak-di-china</t>
+        </is>
+      </c>
+      <c r="H1092" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/CjkinzN000016_20260810_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1092" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>Menhub menegaskan cabut izin operator KMP Mutiara bila terbukti lalai</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:49:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1093" t="inlineStr">
+        <is>
+          <t>Menteri Perhubungan (Menhub) Dudy Purwagandhi menegaskan pemerintah akan mencabut izin operator KMP Mutiara Sentosa ...</t>
+        </is>
+      </c>
+      <c r="F1093" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1093" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688205/menhub-menegaskan-cabut-izin-operator-kmp-mutiara-bila-terbukti-lalai</t>
+        </is>
+      </c>
+      <c r="H1093" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/C8926C3A-5632-417E-9635-309C4AAA82A6.jpeg</t>
+        </is>
+      </c>
+      <c r="I1093" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>Morgan jaga peluang ke Kejuaraan Dunia Karting setelah juarai MiniRok</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:49:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1094" t="inlineStr">
+        <is>
+          <t>Atlet gokart muda Morgan Holindo Sonmoahi menjaga peluang meraih tiket Kejuaraan Dunia Karting di Italia setelah ...</t>
+        </is>
+      </c>
+      <c r="F1094" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1094" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688204/morgan-jaga-peluang-ke-kejuaraan-dunia-karting-setelah-juarai-minirok</t>
+        </is>
+      </c>
+      <c r="H1094" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1001101085.jpg</t>
+        </is>
+      </c>
+      <c r="I1094" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>Survei IPO tempatkan Bahlil dan Golkar sama-sama di posisi ketiga</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:45:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1095" t="inlineStr">
+        <is>
+          <t>Survei Indonesia Political Opinion (IPO) menempatkan Menteri Energi dan Sumber Daya Mineral sekaligus Ketua Umum Partai ...</t>
+        </is>
+      </c>
+      <c r="F1095" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1095" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688201/survei-ipo-tempatkan-bahlil-dan-golkar-sama-sama-di-posisi-ketiga</t>
+        </is>
+      </c>
+      <c r="H1095" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_7687.jpg</t>
+        </is>
+      </c>
+      <c r="I1095" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>Pebasket lokal Indonesia makin berkualitas</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:44:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1096" t="inlineStr">
+        <is>
+          <t>Pelatih kepala tim nasional bola basket putra Indonesia David Singleton menilai kualitas pemain lokal semakin bagus ...</t>
+        </is>
+      </c>
+      <c r="F1096" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1096" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688200/pebasket-lokal-indonesia-makin-berkualitas</t>
+        </is>
+      </c>
+      <c r="H1096" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000476680.jpg</t>
+        </is>
+      </c>
+      <c r="I1096" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>Ichsan Pratama gabung Deltras FC siap arungi musim baru</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:38:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1097" t="inlineStr">
+        <is>
+          <t>Gelandang senior Ichsan Pratama resmi bergabung dengan Deltras FC setelah musim lalu membela PSS Sleman, dengan target ...</t>
+        </is>
+      </c>
+      <c r="F1097" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1097" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688196/ichsan-pratama-gabung-deltras-fc-siap-arungi-musim-baru</t>
+        </is>
+      </c>
+      <c r="H1097" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG-20260810-WA0072.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I1097" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>Komisi IX ajak semua pihak ambil peran dalam program 'Genting'</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:38:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1098" t="inlineStr">
+        <is>
+          <t>Ketua Komisi IX DPR-RI, Felly E. Runtuwene mengajak semua pihak ikut mengambil peran dalam program 'Gerakan ...</t>
+        </is>
+      </c>
+      <c r="F1098" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1098" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688193/komisi-ix-ajak-semua-pihak-ambil-peran-dalam-program-genting</t>
+        </is>
+      </c>
+      <c r="H1098" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1001993888.jpg</t>
+        </is>
+      </c>
+      <c r="I1098" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>BTN bermitra dengan Pemkot Padang memperluas layanan KPR hingga UMKM</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:32:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1099" t="inlineStr">
+        <is>
+          <t>PT Bank Tabungan Negara (Persero) Tbk (BTN) bermitra dengan Pemerintah Kota (Pemkot) Padang, Sumatera Barat (Sumbar), ...</t>
+        </is>
+      </c>
+      <c r="F1099" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1099" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688189/btn-bermitra-dengan-pemkot-padang-memperluas-layanan-kpr-hingga-umkm</t>
+        </is>
+      </c>
+      <c r="H1099" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/WhatsApp-Image-2026-08-10-at-18.34.39.jpeg</t>
+        </is>
+      </c>
+      <c r="I1099" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>Puslabfor ambil 30 item dari olah TKP di sekolah temuan senjata di Jaksel</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:31:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1100" t="inlineStr">
+        <is>
+          <t>Tim Pusat Laboratorium Forensik (Puslabfor) Bareskrim Polri mengambil sebanyak 30 item dari olah tempat kejadian ...</t>
+        </is>
+      </c>
+      <c r="F1100" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1100" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688185/puslabfor-ambil-30-item-dari-olah-tkp-di-sekolah-temuan-senjata-di-jaksel</t>
+        </is>
+      </c>
+      <c r="H1100" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1001021779.jpg</t>
+        </is>
+      </c>
+      <c r="I1100" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>DPRD Sulteng minta empat persoalan tambang emas CPM dievaluasi</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:22:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1101" t="inlineStr">
+        <is>
+          <t>Komisi III DPRD Sulawesi Tengah menyoroti empat persoalan terkait operasional tambang emas PT Citra Palu Minerals (CPM) ...</t>
+        </is>
+      </c>
+      <c r="F1101" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1101" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688181/dprd-sulteng-minta-empat-persoalan-tambang-emas-cpm-dievaluasi</t>
+        </is>
+      </c>
+      <c r="H1101" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/13/IMG_20260213_061140.jpg</t>
+        </is>
+      </c>
+      <c r="I1101" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>Polisi segera ekshumasi makam Sutrimo, penjaga kediaman eks Jampidsus</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:21:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1102" t="inlineStr">
+        <is>
+          <t>ANTARA - Menjelang proses pembongkaran makam untuk keperluan penyelidikan kasus atau ekshumasi terhadap makam Sutrimo, ...</t>
+        </is>
+      </c>
+      <c r="F1102" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1102" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5688132/polisi-segera-ekshumasi-makam-sutrimo-penjaga-kediaman-eks-jampidsus</t>
+        </is>
+      </c>
+      <c r="H1102" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SANS_POLISI-SEGERA-EKSHUMASI-MAKAM-SUTRIMO-PENJAGA-KEDIAMAN-EKS-JAMPIDSUS.jpg</t>
+        </is>
+      </c>
+      <c r="I1102" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>Misbakhun ingatkan pemda tertib kelola dan pertanggungjawabkan anggaran</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:18:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1103" t="inlineStr">
+        <is>
+          <t>Ketua Komisi XI DPR RI Mukhamad Misbakhun mengingatkan pemerintah daerah, termasuk pengelola BUMD dan BLUD, agar tertib ...</t>
+        </is>
+      </c>
+      <c r="F1103" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1103" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688179/misbakhun-ingatkan-pemda-tertib-kelola-dan-pertanggungjawabkan-anggaran</t>
+        </is>
+      </c>
+      <c r="H1103" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1001229509.jpg</t>
+        </is>
+      </c>
+      <c r="I1103" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>BNPB desak kepala daerah di Kalbar-Kalteng cabut izin pembukaan lahan</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:16:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1104" t="inlineStr">
+        <is>
+          <t>ANTARA - BNPB mendesak kepala daerah di Kalimantan Barat dan Tengah segera mencabut izin pembukaan lahan untuk ...</t>
+        </is>
+      </c>
+      <c r="F1104" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1104" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5688117/bnpb-desak-kepala-daerah-di-kalbar-kalteng-cabut-izin-pembukaan-lahan</t>
+        </is>
+      </c>
+      <c r="H1104" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/BNPB-DESAK-KEPALA-DAERAH-DI-KALBAR-KALTENG-CABUT-IZIN-PEMBUKAAN-LAHAN.jpg</t>
+        </is>
+      </c>
+      <c r="I1104" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>Kemensos-Komnas HAM sinergi tangani pengungsi konflik Papua Tengah</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:14:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1105" t="inlineStr">
+        <is>
+          <t>Kementerian Sosial (Kemensos) bersinergi dengan Komisi Nasional Hak Asasi Manusia (Komnas HAM) untuk menangani para ...</t>
+        </is>
+      </c>
+      <c r="F1105" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1105" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688173/kemensos-komnas-ham-sinergi-tangani-pengungsi-konflik-papua-tengah</t>
+        </is>
+      </c>
+      <c r="H1105" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/203343.jpg</t>
+        </is>
+      </c>
+      <c r="I1105" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>Kemenhub sebut ETLE Hub tersebar di 51 titik pantau demi tekan ODOL</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:14:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1106" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1106" t="inlineStr">
+        <is>
+          <t>Kementerian Perhubungan (Kemenhub) menyebut sistem Electronic Traffic Law Enforcement Hub (ETLE Hub) telah tersebar di ...</t>
+        </is>
+      </c>
+      <c r="F1106" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1106" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688171/kemenhub-sebut-etle-hub-tersebar-di-51-titik-pantau-demi-tekan-odol</t>
+        </is>
+      </c>
+      <c r="H1106" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/DFECB780-5C05-4D9B-9E7E-BC4E12249CE6.jpeg</t>
+        </is>
+      </c>
+      <c r="I1106" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>Bos Aprilia bertekad juara di kandang Marc Marquez</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:12:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1107" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1107" t="inlineStr">
+        <is>
+          <t>Bos Aprilia Racing Massimo Rivola membidik kemenangan di MotoGP Aragon yang menjadi kandang pembalap Ducati Lenovo Marc ...</t>
+        </is>
+      </c>
+      <c r="F1107" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1107" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688167/bos-aprilia-bertekad-juara-di-kandang-marc-marquez</t>
+        </is>
+      </c>
+      <c r="H1107" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/01/XxjpbeE000208_20260601_PEPFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1107" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>Iran Tuntut AS Penuhi 5 Syarat Agar Selat Hormuz Dibuka Lagi</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:14:53 +0700</t>
+        </is>
+      </c>
+      <c r="D1108" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E1108" t="inlineStr">
+        <is>
+          <t>Iran menegaskan, Amerika Serikat harus memenuhi sejumlah syarat, memberikan kompensasi, mengakhiri sanksi dan ancaman militer sebelum Selat Hormuz dibuka.</t>
+        </is>
+      </c>
+      <c r="F1108" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1108" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8612918/iran-tuntut-as-penuhi-5-syarat-agar-selat-hormuz-dibuka-lagi</t>
+        </is>
+      </c>
+      <c r="H1108" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/18/perang-as-iran-berakhir-selat-hormuz-segera-dibuka-1781798442899_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1108" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>LRT Jakarta Velodrome-Manggarai Rp 4,1 Triliun Bakal Diresmikan Bulan Ini</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:41:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1109" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E1109" t="inlineStr">
+        <is>
+          <t>Penyelesaian konstruksi Light Rail Transit (LRT) Jakarta Fase 1B rute Velodrome-Manggarai terus dipercepat.</t>
+        </is>
+      </c>
+      <c r="F1109" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1109" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8612901/lrt-jakarta-velodrome-manggarai-rp-4-1-triliun-bakal-diresmikan-bulan-ini</t>
+        </is>
+      </c>
+      <c r="H1109" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/12/progres-pembangunan-lrt-jakarta-fase-1-b-1781249050504_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1109" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>Gak Mewah Tapi Hangat! Momo Eks Geisha Beri Kejutan di Ultah Suami</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:02:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1110" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E1110" t="inlineStr">
+        <is>
+          <t>Momo eks Geisha merayakan ulang tahun ke-37 suaminya Nicola Reza Samudra. Dia mempersiapkan kejutan meriah lengkap dengan kehangatan keluarga.</t>
+        </is>
+      </c>
+      <c r="F1110" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1110" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8612215/gak-mewah-tapi-hangat-momo-eks-geisha-beri-kejutan-di-ultah-suami</t>
+        </is>
+      </c>
+      <c r="H1110" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/momo-eks-geisha-1786348658920_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1110" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>Bigmo Serahkan Rekaman Live Utuh ke Polisi: Spontan, Tak Ada Skenario</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:47:08 +0700</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E1111" t="inlineStr">
+        <is>
+          <t>Bigmo menyerahkan rekaman siaran langsung ke Polda Metro Jaya untuk membuktikan interaksi spontan dengan anak-anak, terkait dugaan eksploitasi vape.</t>
+        </is>
+      </c>
+      <c r="F1111" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1111" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8612904/bigmo-serahkan-rekaman-live-utuh-ke-polisi-spontan-tak-ada-skenario</t>
+        </is>
+      </c>
+      <c r="H1111" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/youtuber-bigmo-dicecar-40-pertanyaan-soal-konten-promosi-vape-ajak-anak-1786361146873_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1111" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>Jonathan Frizzy Batasi Main Padel karena Berat Badan Ikut Turun</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:01:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E1112" t="inlineStr">
+        <is>
+          <t>Jonathan Frizzy keranjingan padel setelah 6 bulan berlatih. Ia mengurangi frekuensi latihan untuk menjaga berat badan karena menganggap sudah terlalu kurus.</t>
+        </is>
+      </c>
+      <c r="F1112" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1112" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8612520/jonathan-frizzy-batasi-main-padel-karena-berat-badan-ikut-turun</t>
+        </is>
+      </c>
+      <c r="H1112" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/jonathan-frizzy-1786357077078_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1112" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>Raffi Ahmad Ungkap Dampak Kolaborasi RANS &amp;amp; Mayora di Dunia Entertainment</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 20:32:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E1113" t="inlineStr">
+        <is>
+          <t>PT RANS Entertainment menjalin kemitraan strategis dengan Mayora dan LINK Group. Kolaborasi ini bertujuan memberikan dampak sosial bagi UMKM di Indonesia.</t>
+        </is>
+      </c>
+      <c r="F1113" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1113" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8612819/raffi-ahmad-ungkap-dampak-kolaborasi-rans-mayora-di-dunia-entertainment</t>
+        </is>
+      </c>
+      <c r="H1113" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/rans-1786368608984_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1113" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>Setahun Nikah, Faishal Tanjung-Nadin Amizah Kunjungi Tempat Sakral Ini</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 20:02:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E1114" t="inlineStr">
+        <is>
+          <t>Pasangan musisi Faishal Tanjung dan Nadin Amizah sudah setahun menikah. Begini cara mereka merayakannya.</t>
+        </is>
+      </c>
+      <c r="F1114" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1114" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8612075/setahun-nikah-faishal-tanjung-nadin-amizah-kunjungi-tempat-sakral-ini</t>
+        </is>
+      </c>
+      <c r="H1114" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/nadin-amizah-1786345279328_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1114" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>Effort Leony Saat Pacar dari Selandia Baru Ultah</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:39:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E1115" t="inlineStr">
+        <is>
+          <t>Artis Leony melakukan upaya besar untuk memberi kejutan ulang tahun ke pacarnya, Charles Seaman. Seperti apa?</t>
+        </is>
+      </c>
+      <c r="F1115" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1115" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8612730/effort-leony-saat-pacar-dari-selandia-baru-ultah</t>
+        </is>
+      </c>
+      <c r="H1115" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/leony-1786363964103_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1115" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>Kronologi Polisi Jadi Korban Begal Saat Nyambi Ngojek di Palembang, Pelakunya Sepasang Kekasih</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:41:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1116" t="inlineStr">
+        <is>
+          <t>Aiptu Januardo Eko Satria, seorang anggota Polri menjadi korban begal saat nyambi jadi tukang ojek di Palembang, Sumatera Selatan</t>
+        </is>
+      </c>
+      <c r="F1116" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1116" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866572/kronologi-polisi-jadi-korban-begal-saat-nyambi-ngojek-di-palembang-pelakunya-sepasang-kekasih</t>
+        </is>
+      </c>
+      <c r="H1116" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/XfV5WTRcxonxe_AAIRL1RRXJanY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pelaku-begal-polisi-di-palembang.jpg</t>
+        </is>
+      </c>
+      <c r="I1116" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>7 Langkah Memilih Camilan yang Aman dan Sehat untuk Anak Menurut BPOM RI</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:38:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1117" t="inlineStr">
+        <is>
+          <t>BPOM membagikan tips memilih camilan anak, mulai dari memperhatikan gizi, keamanan bahan, label kemasan, hingga izin edar produk</t>
+        </is>
+      </c>
+      <c r="F1117" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1117" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866571/7-langkah-memilih-camilan-yang-aman-dan-sehat-untuk-anak-menurut-bpom-ri</t>
+        </is>
+      </c>
+      <c r="H1117" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/RJHIYu077TDo8eNWqk2tkJivOvU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/festival-camilan.jpg</t>
+        </is>
+      </c>
+      <c r="I1117" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>Kunci Gitar Lagu Luka Dipelupuk Mata - Dongker: Sayang, Tampar Mukaku Lihat Sekitar</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:30:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1118" t="inlineStr">
+        <is>
+          <t>Kunci gitar lagu Luka di Pelupuk Mata - Dongker feat Binar chord dasar mudah dimainkan: sayang, tampar mukaku lihat sekitar semua yang tak pernah.</t>
+        </is>
+      </c>
+      <c r="F1118" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1118" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7866570/kunci-gitar-lagu-luka-dipelupuk-mata-dongker-sayang-tampar-mukakulihat-sekitar</t>
+        </is>
+      </c>
+      <c r="H1118" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/E33dbHm7VtGLAEgLsyP9Ie4szxc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Dongker-1-27042026.jpg</t>
+        </is>
+      </c>
+      <c r="I1118" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>Kunci Gitar Lagu Moonlight - Nadin Amizah: And We'll Dance Huu, And We'll Dance Huu</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:29:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1119" t="inlineStr">
+        <is>
+          <t>Kunci gitar lagu Moonlight - Nadin Amizah chord dasar yang mudah dimainkan: and we'll dance hu..u..u..uu.. and we'll dance hu..u..u..uu..</t>
+        </is>
+      </c>
+      <c r="F1119" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1119" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7866569/kunci-gitar-lagu-moonlight-nadin-amizah-and-well-dance-huu-and-well-dance-huu</t>
+        </is>
+      </c>
+      <c r="H1119" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/4WAU_R_lDbvx8WfDEi6lDCUI8QA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Nadin-Amizah-1-23012026.jpg</t>
+        </is>
+      </c>
+      <c r="I1119" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>Topan No. 15 Bergerak ke Honshu, Jepang Waspadai Hujan Lebat dan Angin Kencang</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:19:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1120" t="inlineStr">
+        <is>
+          <t>Topan No. 15 bergerak dengan jalur tak biasa dan diperkirakan menghantam Honshu. JMA waspadai hujan lebat, angin kencang, dan gelombang tinggi</t>
+        </is>
+      </c>
+      <c r="F1120" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1120" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866568/topan-no-15-bergerak-ke-honshu-jepang-waspadai-hujan-lebat-dan-angin-kencang</t>
+        </is>
+      </c>
+      <c r="H1120" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zf37Zz_CtYsJh6z7y3PV1F2kY9Q=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/anginjepang212222.jpg</t>
+        </is>
+      </c>
+      <c r="I1120" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>Bulan Imunisasi Anak Sekolah Dimulai, Siswa SD Darunnajah Jaksel Terima Imunisasi Rubella hingga HPV</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:19:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1121" t="inlineStr">
+        <is>
+          <t>Sekolah Dasar Islam (SDI) Darunnajah Ulujami melaksanakan program Bulan Imunisasi Anak Sekolah (BIAS) pada bulan Agustus 2026 ini.</t>
+        </is>
+      </c>
+      <c r="F1121" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1121" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866567/bulan-imunisasi-anak-sekolah-dimulai-siswa-sd-darunnajah-jaksel-terima-imunisasi-rubella-hingga-hpv</t>
+        </is>
+      </c>
+      <c r="H1121" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0NSb0BTHJjMBDMjTtkou8_0d6IM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/imnsasibias2026.jpg</t>
+        </is>
+      </c>
+      <c r="I1121" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban Bahasa Indonesia Kawan Seiring Kelas 3 Halaman 21 Kurikulum Merdeka: Aktivitas 5</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:06:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1122" t="inlineStr">
+        <is>
+          <t>Soal ini terdapat pada buku Bahasa Indonesia Kawan Seiring Kelas 3 Halaman 21 Kurikulum Merdeka, tepatnya pada Aktivitas 5.</t>
+        </is>
+      </c>
+      <c r="F1122" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1122" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7866566/kunci-jawaban-bahasa-indonesia-kawan-seiring-kelas-3-halaman-21-kurikulum-merdeka-aktivitas-5</t>
+        </is>
+      </c>
+      <c r="H1122" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/fLjsurmR-3RdbbUMtGvfTJlnZfs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/siswa-SD-belajar-di-sekolah-2.jpg</t>
+        </is>
+      </c>
+      <c r="I1122" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>Pelajar SMA Meninggal Tertemper KRL di Stasiun Jurangmangu, Polisi Selidiki Penyebabnya</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:04:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1123" t="inlineStr">
+        <is>
+          <t>Pelajar SMA tewas tertemper KRL di Stasiun Jurangmangu. Polisi masih menyelidiki kronologi dan penyebab korban berada di jalur kereta.</t>
+        </is>
+      </c>
+      <c r="F1123" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1123" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866565/pelajar-sma-meninggal-tertemper-krl-di-stasiun-jurangmangu-polisi-selidiki-penyebabnya</t>
+        </is>
+      </c>
+      <c r="H1123" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/vnN8t7-_sNFl5avv0zV2pk7I0Tk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/tertemperKRL1.jpg</t>
+        </is>
+      </c>
+      <c r="I1123" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu I Think God Can Explain - Splender: There's A Lot of Things I Understand</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:03:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1124" t="inlineStr">
+        <is>
+          <t>Simak terjemahan lirik lagu "I Think God Can Explain" yang dipopulerkan oleh grup musik rock alternatif asal Amerika Serikat (AS), Splender.</t>
+        </is>
+      </c>
+      <c r="F1124" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1124" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7866564/terjemahan-lirik-lagu-i-think-god-can-explain-splender-theres-a-lot-of-things-i-understand</t>
+        </is>
+      </c>
+      <c r="H1124" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/U-BX1ieF2y0vnLJFGFlYSjiTfIc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/headphones-desk-black-laid.jpg</t>
+        </is>
+      </c>
+      <c r="I1124" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>Dorong Hilirisasi Mineral, Pakar Unand: Indonesia Harus Kuasai Rantai Teknologi hingga Manufaktur</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:54:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1125" t="inlineStr">
+        <is>
+          <t>Dekan Fakultas Teknik Unand ini menjelaskan bahwa material merupakan fondasi utama bagi hampir seluruh industri berbasis teknologi modern</t>
+        </is>
+      </c>
+      <c r="F1125" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1125" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7866563/dorong-hilirisasi-mineral-pakar-unand-indonesia-harus-kuasai-rantai-teknologi-hingga-manufaktur</t>
+        </is>
+      </c>
+      <c r="H1125" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/D7PvT6d8l9VJtjzMAKtL6oXp7c8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pertambangan-hilirisasi-898.jpg</t>
+        </is>
+      </c>
+      <c r="I1125" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>Hadapi Perubahan Teknologi, Perusahaan IT Perkuat Pengembangan AI</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:48:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1126" t="inlineStr">
+        <is>
+          <t>Perkembangan artificial intelligence (AI), cloud, data, hingga teknologi quantum perlu terus dipahami karena berpotensi mengubah proses bisnis</t>
+        </is>
+      </c>
+      <c r="F1126" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1126" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/techno/7866562/hadapi-perubahan-teknologi-perusahaan-it-perkuat-pengembangan-ai</t>
+        </is>
+      </c>
+      <c r="H1126" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/IrGaDFDwqU1c7vZPabKq0pBNfR4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/lari2222222.jpg</t>
+        </is>
+      </c>
+      <c r="I1126" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>Mengenal Taktik Hellscape: Cara Taiwan Mengubah Keunggulan China Jadi Beban di Medan Perang</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:42:42 +0700</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1127" t="inlineStr">
+        <is>
+          <t>hellscape adalah strategi yang dirancang untuk mengubah Selat Taiwan menjadi medan perang yang penuh hambatan bagi pasukan penyerang China.</t>
+        </is>
+      </c>
+      <c r="F1127" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1127" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866561/mengenal-taktik-hellscape-cara-taiwan-mengubah-keunggulan-china-jadi-beban-di-medan-perang</t>
+        </is>
+      </c>
+      <c r="H1127" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/z4Tm0IS7mQdIa40zymiZZ-LAvAg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Tentara-Taiwan-dalam-latihan-tembak.jpg</t>
+        </is>
+      </c>
+      <c r="I1127" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>Personel Manchester United Makin Lengkap, 9 Pemain Boyongan ke Irlandia</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:41:42 +0700</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1128" t="inlineStr">
+        <is>
+          <t>9 pemain Manchester United akan bergabung dengan pemusatan latihan klub yang kini berada di Irlandia untuk persiapan melawan Leeds United.</t>
+        </is>
+      </c>
+      <c r="F1128" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1128" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866560/personel-manchester-united-makin-lengkap-9-pemain-boyongan-ke-irlandia</t>
+        </is>
+      </c>
+      <c r="H1128" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rUPG4n-YQc8DyP71l6MuTLUdAoA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Logo-klub-Manchester-United.jpg</t>
+        </is>
+      </c>
+      <c r="I1128" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>Konsumen Makin Selektif Memilih Skincare, Tak Sekadar Ikuti Tren</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:41:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1129" t="inlineStr">
+        <is>
+          <t>Hasil survei menunjukkan 75 persen responden menilai rutinitas kecantikan yang konsisten berkontribusi terhadap kesejahteraan dan kepercayaan diri.</t>
+        </is>
+      </c>
+      <c r="F1129" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1129" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/lifestyle/7866559/konsumen-makin-selektif-memilih-skincare-tak-sekadar-ikuti-tren</t>
+        </is>
+      </c>
+      <c r="H1129" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/a3B5NvDnzgBQn-90xCwln5CAeuY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/MEMLIH-SKINCARE-teknologi-AI.jpg</t>
+        </is>
+      </c>
+      <c r="I1129" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>Dede Yusuf Dorong Tugas Wakil Kepala Daerah Diperjelas Agar Tak Hanya Jadi 'Ban Serep'</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:39:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1130" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Komisi II DPR RI Dede Yusuf, menanggapi wacana wakil kepala daerah tidak lagi dipilih secara langsung melalui Pilkada.</t>
+        </is>
+      </c>
+      <c r="F1130" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1130" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866558/dede-yusuf-dorong-tugas-wakil-kepala-daerah-diperjelas-agar-tak-hanya-jadi-ban-serep</t>
+        </is>
+      </c>
+      <c r="H1130" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/-T52nXX_9IXg4te5nAc2zjS-18k=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Wakil-Ketua-Umum-Partai-Demokrat-Dede-Yusuf-3219.jpg</t>
+        </is>
+      </c>
+      <c r="I1130" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>Morgan Holindo Menangi MiniRok Round 5, Tiket Kejuaraan Dunia Italia Makin Panas</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:37:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1131" t="inlineStr">
+        <is>
+          <t>Presisi dalam melewati setiap tikungan menjadi salah satu kunci Morgan mempertahankan keunggulannya.</t>
+        </is>
+      </c>
+      <c r="F1131" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1131" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866557/morgan-holindo-menangi-minirok-round-5-tiket-kejuaraan-dunia-italia-makin-panas</t>
+        </is>
+      </c>
+      <c r="H1131" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/duPs0oHISYocgK343koqJuRgcBw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PACU-GOKART-Morgan-Holindo-Sonmoahi-memacu-gokartnya.jpg</t>
+        </is>
+      </c>
+      <c r="I1131" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>Perwira Menengah TNI AL Didakwa Edarkan Sabu, Pelaku Libatkan Istri</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:34:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1132" t="inlineStr">
+        <is>
+          <t>Mayor Laut Faisal mengaku sudah sudah mengonsumsi sabu bersama Kapten Laut I Made Surya sejak tahun 2024</t>
+        </is>
+      </c>
+      <c r="F1132" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1132" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866556/perwira-menengah-tni-al-didakwa-edarkan-sabu-pelaku-libatkan-istri</t>
+        </is>
+      </c>
+      <c r="H1132" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/NNQ5R-oY_sv9elawTryf6vOvk-U=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Suasana-Mayor-Laut-Faisal-Mulia.jpg</t>
+        </is>
+      </c>
+      <c r="I1132" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>Rutin Olahraga Senam Bantu Jaga Kelenturan Otot dan Keseimbangan Tubuh hingga Usia Lanjut</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:33:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1133" t="inlineStr">
+        <is>
+          <t>Senam salah satu olahraga yang dianjurkan, karena kelenturan otot dan mobilitas sendi cenderung mengalami penurunan seiring bertambahnya usia.</t>
+        </is>
+      </c>
+      <c r="F1133" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1133" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866555/rutin-olahraga-senam-bantu-jaga-kelenturan-otot-dan-keseimbangan-tubuh-hingga-usia-lanjut</t>
+        </is>
+      </c>
+      <c r="H1133" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/qni-z7ElwzZkJZT7rK3b72XOaaI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Senam-1-10082026.jpg</t>
+        </is>
+      </c>
+      <c r="I1133" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>Metode 3R dan Pentingnya Pendekatan Menyeluruh dalam Pengelolaan Diabetes</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:31:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1134" t="inlineStr">
+        <is>
+          <t>Banyak penderita DMT2 kesulitan konsisten ubah gaya hidup. Metode 3R hadir sebagai solusi menyeluruh cegah komplikasi.</t>
+        </is>
+      </c>
+      <c r="F1134" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1134" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/tribunners/7866554/metode-3r-dan-pentingnya-pendekatan-menyeluruh-dalam-pengelolaan-diabetes</t>
+        </is>
+      </c>
+      <c r="H1134" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WHGJgJjnf79jZ8IvUeiyxZf9Mq8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-diabetes.jpg</t>
+        </is>
+      </c>
+      <c r="I1134" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>Singapura vs Thailand di 4 Besar Piala AFF 2026: Kisah Heroik The Lions Lanjut atau Berakhir?</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:30:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1135" t="inlineStr">
+        <is>
+          <t>Dongeng indah yang sejauh ini diciptakan Timnas Singapura di Piala AFF 2026 akan berlanjut pada babak semifinal.</t>
+        </is>
+      </c>
+      <c r="F1135" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1135" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866553/singapura-vs-thailand-di-4-besar-piala-aff-2026-kisah-heroik-the-lions-lanjut-atau-berakhir</t>
+        </is>
+      </c>
+      <c r="H1135" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iboht6amQhsYVg3hY7SU_axQqZo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Aksi-kiper-Timnas-Indonesia-Cahya-Supriadi-dan-Beckham-Putra-berusaha-meredam-pemain-Singapura.jpg</t>
+        </is>
+      </c>
+      <c r="I1135" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>Jelang HUT ke-42, KBI Raih Tiga Penghargaan dalam Dua Ajang</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr">
+        <is>
+          <t>Ichsan Emrald Alamsyah</t>
+        </is>
+      </c>
+      <c r="E1136" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- PT Kliring Berjangka Indonesia (PT KBI) meraih tiga penghargaan dari dua ajang berbeda dalam satu hari. Capaian tersebut diraih menjelang peringatan HUT ke-42 PT KBI yang jatuh...</t>
+        </is>
+      </c>
+      <c r="F1136" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1136" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjk0lg349/jelang-hut-ke42-kbi-raih-tiga-penghargaan-dalam-dua-ajang</t>
+        </is>
+      </c>
+      <c r="H1136" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/pt-kliring-berjangka-indonesia-pt-kbi-meraih-tiga-penghargaan_260810194049-761.jpg</t>
+        </is>
+      </c>
+      <c r="I1136" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>Polisi Dalami Penyebab Siswi SMA Tertemper KRL di Jurangmangu</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:36:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1137" t="inlineStr">
+        <is>
+          <t>Petugas melakukan identifikasi dan pemeriksaan di lokasi kejadian.</t>
+        </is>
+      </c>
+      <c r="F1137" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1137" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266627/polisi-dalami-penyebab-siswi-sma-tertemper-krl-di-jurangmangu</t>
+        </is>
+      </c>
+      <c r="H1137" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/cXOlyfDT2PZaYxlfJ_SLh9dJWwY=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/3583727/original/039256500_1632655961-2021026-FOTO---KRL-Herman-8.jpg</t>
+        </is>
+      </c>
+      <c r="I1137" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>Berkas Lengkap, KPK Limpahkan Ajudan Gubernur Riau Abdul Wahid ke JPU</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:21:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1138" t="inlineStr">
+        <is>
+          <t>Pelimpahan tahap dua tersebut dilakukan terkait kasus pemerasan di lingkungan Pemprov Riau tahun anggaran 2025.</t>
+        </is>
+      </c>
+      <c r="F1138" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1138" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266623/berkas-lengkap-kpk-limpahkan-ajudan-gubernur-riau-abdul-wahid-ke-jpu</t>
+        </is>
+      </c>
+      <c r="H1138" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/ShIfkKlF2x04R1g_FIea0Cswkb4=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5554637/original/039376600_1776082734-IMG_0315.jpg</t>
+        </is>
+      </c>
+      <c r="I1138" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>KPK Bongkar Skema Korupsi Iklan Bank BJB, Negara Rugi Rp 223,6 Miliar</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:41:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1139" t="inlineStr">
+        <is>
+          <t>Dari anggaran tersebut, sekitar Rp 410 miliar disetujui untuk penempatan iklan di media televisi, cetak, dan daring melalui pengadaan jasa agensi.</t>
+        </is>
+      </c>
+      <c r="F1139" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1139" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266619/kpk-bongkar-skema-korupsi-iklan-bank-bjb-negara-rugi-rp-2236-miliar</t>
+        </is>
+      </c>
+      <c r="H1139" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/cYgvVSSkr1LAnPTCETtvLPa8NRw=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/4065432/original/001612500_1656325087-WhatsApp_Image_2022-06-27_at_5.08.03_PM.jpeg</t>
+        </is>
+      </c>
+      <c r="I1139" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>Siswi SMA Tertemper KRL di Jurangmangu</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:55:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1140" t="inlineStr">
+        <is>
+          <t>Polisi masih melakukan identifikasi dan penyelidikan untuk mengetahui penyebab kejadian.</t>
+        </is>
+      </c>
+      <c r="F1140" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1140" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266613/siswi-sma-tertemper-krl-di-jurangmangu</t>
+        </is>
+      </c>
+      <c r="H1140" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/U_qlSYUdcatyMU2uoGrWoeWdKM0=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9309837/original/095095900_1785290323-faisal-hanafi-zmr4ypKgTyg-unsplash.jpg</t>
+        </is>
+      </c>
+      <c r="I1140" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1067"/>
+  <autoFilter ref="A1:I1140"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 16:45 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1186</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1140"/>
+  <dimension ref="A1:I1186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -54019,8 +54019,2170 @@
         </is>
       </c>
     </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>IDM ajak masyarakat maknai kemerdekaan dengan mencintai warisan budaya</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:34:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1141" t="inlineStr">
+        <is>
+          <t>InJourney Destination Management (IDM) mengajak masyarakat memaknai kemerdekaan tidak hanya sebagai perayaan seremonial ...</t>
+        </is>
+      </c>
+      <c r="F1141" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1141" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688344/idm-ajak-masyarakat-maknai-kemerdekaan-dengan-mencintai-warisan-budaya</t>
+        </is>
+      </c>
+      <c r="H1141" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000481689.jpg</t>
+        </is>
+      </c>
+      <c r="I1141" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>PIER: Sektor jasa penopang pertumbuhan ekonomi kuartal II 2026</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:34:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1142" t="inlineStr">
+        <is>
+          <t>Permata Institute for Economic Research (PIER) mencatat sektor jasa menjadi salah satu penopang penting pertumbuhan ...</t>
+        </is>
+      </c>
+      <c r="F1142" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1142" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688340/pier-sektor-jasa-penopang-pertumbuhan-ekonomi-kuartal-ii-2026</t>
+        </is>
+      </c>
+      <c r="H1142" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000456874.jpg</t>
+        </is>
+      </c>
+      <c r="I1142" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>Kelompok IRT Jember ubah tutup botol jadi gantungan bernilai ekonomi</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:33:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1143" t="inlineStr">
+        <is>
+          <t>ANTARA - Sekelompok ibu-ibu rumah tangga di di Desa Suci, Kecamatan Panti, Jember, Jawa Timur mengubah limbah tutup ...</t>
+        </is>
+      </c>
+      <c r="F1143" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1143" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5688320/kelompok-irt-jember-ubah-tutup-botol-jadi-gantungan-bernilai-ekonomi</t>
+        </is>
+      </c>
+      <c r="H1143" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KELOMPOK-IRT-JEMBER-UBAH-TUTUP-BOTOL-JADI-GANTUNGAN-BERNILAI-EKONOMI.jpg</t>
+        </is>
+      </c>
+      <c r="I1143" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>Dua kelurahan di Makassar jadi percontohan Sadar HAM</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:23:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1144" t="inlineStr">
+        <is>
+          <t>Kementerian Hak Asasi Manusia memilih Kelurahan Mattoanging, Kecamatan Mariso, dan Kelurahan Kaluku Bodoa, Kecamatan ...</t>
+        </is>
+      </c>
+      <c r="F1144" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1144" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688339/dua-kelurahan-di-makassar-jadi-percontohan-sadar-ham</t>
+        </is>
+      </c>
+      <c r="H1144" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/ImgResizer_IMG-20260810-WA0029.jpg</t>
+        </is>
+      </c>
+      <c r="I1144" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>Antisipasi kebakaran, Pemkot Jakbar bangun pos Damkar-hidran mandiri</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:21:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1145" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota (Pemkot) Jakarta Barat (Jakbar) membangun Pos Pemadam Kebakaran (Damkar) dan hidran mandiri di lokasi ...</t>
+        </is>
+      </c>
+      <c r="F1145" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1145" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688337/antisipasi-kebakaran-pemkot-jakbar-bangun-pos-damkar-hidran-mandiri</t>
+        </is>
+      </c>
+      <c r="H1145" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_20260810_213619.jpg</t>
+        </is>
+      </c>
+      <c r="I1145" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>Pemprov Sumut: Pembangunan di Kepulauan Nias berjalan sesuai rencana</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:20:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) Sumatera Utara (Sumut) memastikan berbagai program prioritas pembangunan ...</t>
+        </is>
+      </c>
+      <c r="F1146" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1146" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688336/pemprov-sumut-pembangunan-di-kepulauan-nias-berjalan-sesuai-rencana</t>
+        </is>
+      </c>
+      <c r="H1146" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1001039869.jpg</t>
+        </is>
+      </c>
+      <c r="I1146" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>OJK: Indeks literasi dan inklusi keuangan 2026 melampaui target RPJMN</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:18:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>Otoritas Jasa Keuangan (OJK) menyampaikan, pencapaian indeks literasi dan inklusi keuangan pada 2026 telah melampaui ...</t>
+        </is>
+      </c>
+      <c r="F1147" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688332/ojk-indeks-literasi-dan-inklusi-keuangan-2026-melampaui-target-rpjmn</t>
+        </is>
+      </c>
+      <c r="H1147" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/9ee27bf0-fbd4-4cf3-8968-5054d21b681d.jpeg</t>
+        </is>
+      </c>
+      <c r="I1147" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>Ekonomi RI diproyeksikan tumbuh di kisaran 5 persen hingga akhir tahun</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:17:39 +0700</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>Chief Economist Permata Bank, Josua Pardede mengatakan perekonomian Indonesia diproyeksikan tetap tumbuh solid di ...</t>
+        </is>
+      </c>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1148" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688331/ekonomi-ri-diproyeksikan-tumbuh-di-kisaran-5-persen-hingga-akhir-tahun</t>
+        </is>
+      </c>
+      <c r="H1148" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000456822.jpg</t>
+        </is>
+      </c>
+      <c r="I1148" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>Dewa United Esports umumkan jadwal laga tim untuk MPL ID musim ke-18</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:17:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>Dewa United Esports mengumumkan jadwal pertandingan tim dalam babak reguler Mobile Legends: Bang Bang Professional ...</t>
+        </is>
+      </c>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1149" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688328/dewa-united-esports-umumkan-jadwal-laga-tim-untuk-mpl-id-musim-ke-18</t>
+        </is>
+      </c>
+      <c r="H1149" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000474548.jpg</t>
+        </is>
+      </c>
+      <c r="I1149" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Polda Jateng siap bantu ekshumasi jenazah Sutrimo</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:16:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>Polda Jawa Tengah siap membantu pelaksanaan ekshumasi jenazah kepala rumah tangga mantan Jaksa Agung Muda Bidang Pidana ...</t>
+        </is>
+      </c>
+      <c r="F1150" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1150" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688324/polda-jateng-siap-bantu-ekshumasi-jenazah-sutrimo</t>
+        </is>
+      </c>
+      <c r="H1150" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_20260810_172957.jpg</t>
+        </is>
+      </c>
+      <c r="I1150" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>Empat dari lima tersangka kasus Bank BJB resmi ditahan KPK</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:13:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>ANTARA - Komisi Pemberantasan Korupsi (KPK) resmi menahan empat dari lima tersangka kasus dugaan korupsi pengadaan ...</t>
+        </is>
+      </c>
+      <c r="F1151" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1151" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5688296/empat-dari-lima-tersangka-kasus-bank-bjb-resmi-ditahan-kpk</t>
+        </is>
+      </c>
+      <c r="H1151" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/EMPAT-DARI-LIMA-TERSANGKA-KASUS-BANK-BJB-RESMI-DITAHAN-KPK.jpg</t>
+        </is>
+      </c>
+      <c r="I1151" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>Menhut dorong gerakan pemulihan hutan dan ekosistem dalam HKAN 2026</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:12:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>Menteri Kehutanan (Menhut) Raja Juli Antoni mendorong gerakan pemulihan hutan dan ekosistem yang mengalami kerusakan ...</t>
+        </is>
+      </c>
+      <c r="F1152" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1152" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688323/menhut-dorong-gerakan-pemulihan-hutan-dan-ekosistem-dalam-hkan-2026</t>
+        </is>
+      </c>
+      <c r="H1152" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/9827e61f-9b6b-4379-8eb9-3a7b1f977a1b.jpeg</t>
+        </is>
+      </c>
+      <c r="I1152" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>BPS menilai cakupan survei pengaruhi penurunan indeks keuangan syariah</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:09:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>Kepala Badan Pusat Statistik (BPS) Amalia Adininggar Widyasanti menilai perubahan cakupan data survei menjadi ...</t>
+        </is>
+      </c>
+      <c r="F1153" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1153" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688319/bps-menilai-cakupan-survei-pengaruhi-penurunan-indeks-keuangan-syariah</t>
+        </is>
+      </c>
+      <c r="H1153" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/c52f08ca-ef66-4b88-9ffb-343422a35fd4.jpeg</t>
+        </is>
+      </c>
+      <c r="I1153" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Enam bandara ditutup akibat gempa magnitudo 7,4 guncang Kolombia</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:09:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>Enam bandara di Kolombia bagian barat mengalami kerusakan dan harus ditutup menyusul gempa bumi dahsyat yang ...</t>
+        </is>
+      </c>
+      <c r="F1154" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1154" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688315/enam-bandara-ditutup-akibat-gempa-magnitudo-74-guncang-kolombia</t>
+        </is>
+      </c>
+      <c r="H1154" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/ilustrasi-gempa-2_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1154" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>Motor wartawan hilang usai liputan di Kantor Kemenko Polkam</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:09:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>Sepeda motor milik pewarta iNews Media Group, Danandaya Arya Putra hilang saat bertugas meliput di Kantor Kemenko ...</t>
+        </is>
+      </c>
+      <c r="F1155" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1155" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688311/motor-wartawan-hilang-usai-liputan-di-kantor-kemenko-polkam</t>
+        </is>
+      </c>
+      <c r="H1155" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/02/25/IMG_20230225_132120.jpg</t>
+        </is>
+      </c>
+      <c r="I1155" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>Puan minta dampak ekonomi penutupan wisata Bromo mulai dihitung</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:07:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>Ketua DPR RI Puan Maharani meminta pemerintah mulai menghitung dampak ekonomi kebakaran di kawasan Taman Nasional Bromo ...</t>
+        </is>
+      </c>
+      <c r="F1156" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1156" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688307/puan-minta-dampak-ekonomi-penutupan-wisata-bromo-mulai-dihitung</t>
+        </is>
+      </c>
+      <c r="H1156" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/titik-api-baru-kebakaran-hutan-kawasan-tnbts-2838619.jpg</t>
+        </is>
+      </c>
+      <c r="I1156" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>Gempa bumi telan korban jiwa di sejumlah daerah Kolombia</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:06:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>Empat orang, termasuk tiga anak, meninggal dunia akibat gempa bumi dahsyat di departemen Valle del Cauca di barat daya ...</t>
+        </is>
+      </c>
+      <c r="F1157" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1157" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688303/gempa-bumi-telan-korban-jiwa-di-sejumlah-daerah-kolombia</t>
+        </is>
+      </c>
+      <c r="H1157" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/02/Bendera-Kolombia.jpg</t>
+        </is>
+      </c>
+      <c r="I1157" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>Presiden Abelardo tangani langsung gempa Kolombia</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:05:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>Presiden Kolombia Abelardo de la Espriella pada Senin menuju Bogota untuk memimpin langsung koordinasi bantuan bagi ...</t>
+        </is>
+      </c>
+      <c r="F1158" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688300/presiden-abelardo-tangani-langsung-gempa-kolombia</t>
+        </is>
+      </c>
+      <c r="H1158" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/thumbs_b_c_6e143678c2cb56b3ec9b82b9a1ee2450.jpg</t>
+        </is>
+      </c>
+      <c r="I1158" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>Kasus temuan senjata di sekolah, polisi identifikasi pelaku lewat DNA</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:04:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1159" t="inlineStr">
+        <is>
+          <t>Kepolisian mengidentifikasi pelaku yang masuk atau pernah berkontak dengan ruangan yang diduga menjadi tempat ...</t>
+        </is>
+      </c>
+      <c r="F1159" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1159" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688297/kasus-temuan-senjata-di-sekolah-polisi-identifikasi-pelaku-lewat-dna</t>
+        </is>
+      </c>
+      <c r="H1159" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1001021852.jpg</t>
+        </is>
+      </c>
+      <c r="I1159" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>Tukang parkir yang viral karena paksa bayar Rp5 ribu ternyata positif narkoba</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:02:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1160" t="inlineStr">
+        <is>
+          <t>Juru parkir (jukir) liar berinisial MS yang ditangkap usai memaksa pengendara membayar Rp5.000 di minimarket wilayah ...</t>
+        </is>
+      </c>
+      <c r="F1160" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1160" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688293/tukang-parkir-yang-viral-karena-paksa-bayar-rp5-ribu-ternyata-positif-narkoba</t>
+        </is>
+      </c>
+      <c r="H1160" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2015/09/20150919juru_parkir-fanny_octavianus.jpg</t>
+        </is>
+      </c>
+      <c r="I1160" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>Menteri ATR sebut Verifikasi BPHTB kini dipercepat jadi tiga hari</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:01:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1161" t="inlineStr">
+        <is>
+          <t>Menteri Agraria dan Tata Ruang (ATR)/Kepala Badan Pertanahan Nasional (BPN) Nusron Wahid mengatakan Surat Edaran ...</t>
+        </is>
+      </c>
+      <c r="F1161" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1161" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688291/menteri-atr-sebut-verifikasi-bphtb-kini-dipercepat-jadi-tiga-hari</t>
+        </is>
+      </c>
+      <c r="H1161" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_20260810_223530.jpg</t>
+        </is>
+      </c>
+      <c r="I1161" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>Kreator Indonesia temukan pesona budaya dalam kunjungannya ke China</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:58:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>Dalam perjalanan keduanya ke China, seorang pemudi Indonesia bernama Najwa Nur Awalia (24) memperoleh sudut pandang ...</t>
+        </is>
+      </c>
+      <c r="F1162" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1162" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688288/kreator-indonesia-temukan-pesona-budaya-dalam-kunjungannya-ke-china</t>
+        </is>
+      </c>
+      <c r="H1162" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/CjkinzN000007_20260810_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1162" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>Pemkab Sigi targetkan SRMP 22 tampung 2.160 siswa pada tahun 2027</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:57:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1163" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kabupaten Sigi menargetkan Sekolah Rakyat setingkat SMP di wilayah tersebut dapat menampung hingga ...</t>
+        </is>
+      </c>
+      <c r="F1163" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1163" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5688267/pemkab-sigi-targetkan-srmp-22-tampung-2160-siswa-pada-tahun-2027</t>
+        </is>
+      </c>
+      <c r="H1163" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PEMKAB-SIGI-TARGETKAN-SRMP-22-TAMPUNG-2.160-SISWA-PADA-TAHUN-2027.jpg</t>
+        </is>
+      </c>
+      <c r="I1163" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>Bupati tekankan pentingnya edukasi perdamaian Aceh bagi generasi muda</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:54:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1164" t="inlineStr">
+        <is>
+          <t>Bupati Aceh Besar, Muharram Idris menekankan pentingnya edukasi sejarah perdamaian Aceh yang sudah berumur 21 tahun ...</t>
+        </is>
+      </c>
+      <c r="F1164" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1164" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688284/bupati-tekankan-pentingnya-edukasi-perdamaian-aceh-bagi-generasi-muda</t>
+        </is>
+      </c>
+      <c r="H1164" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1002104834.jpg</t>
+        </is>
+      </c>
+      <c r="I1164" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>Wanita di Jakbar diduga jadi korban pelecehan oleh sopir taksi online</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:54:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1165" t="inlineStr">
+        <is>
+          <t>Seorang perempuan berinisial SN diduga menjadi korban pelecehan oleh sopir taksi online di wilayah Jakarta Barat ...</t>
+        </is>
+      </c>
+      <c r="F1165" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1165" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688283/wanita-di-jakbar-diduga-jadi-korban-pelecehan-oleh-sopir-taksi-online</t>
+        </is>
+      </c>
+      <c r="H1165" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/22/1000267701.jpg</t>
+        </is>
+      </c>
+      <c r="I1165" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>KKP sebut produk olahan lele marinasi Indonesia tembus pasar Taiwan</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:50:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1166" t="inlineStr">
+        <is>
+          <t>Produk olahan lele marinasi produksi usaha mikro kecil dan menengah (UMKM) asal Bandung, Jawa Barat, menembus pasar ...</t>
+        </is>
+      </c>
+      <c r="F1166" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1166" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688279/kkp-sebut-produk-olahan-lele-marinasi-indonesia-tembus-pasar-taiwan</t>
+        </is>
+      </c>
+      <c r="H1166" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/WhatsApp-Image-2026-08-10-at-22.27.38.jpeg</t>
+        </is>
+      </c>
+      <c r="I1166" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>Komisi XI minta mitra SPPG dukung pembenahan tata kelola MBG</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:48:39 +0700</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1167" t="inlineStr">
+        <is>
+          <t>Ketua Komisi XI DPR RI Mukhamad Misbakhun meminta mitra Satuan Pelayanan Pemenuhan Gizi (SPPG) untuk mendukung ...</t>
+        </is>
+      </c>
+      <c r="F1167" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1167" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688277/komisi-xi-minta-mitra-sppg-dukung-pembenahan-tata-kelola-mbg</t>
+        </is>
+      </c>
+      <c r="H1167" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/dapur-mbg-wajib-memiliki-sertifikat-laik-higiene-sanitasi-2835365.jpg</t>
+        </is>
+      </c>
+      <c r="I1167" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>Kemenimipas usulkan amnesti warga binaan usia produktif</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:40:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1168" t="inlineStr">
+        <is>
+          <t>Kementerian Imigrasi dan Pemasyarakatan (Kemenimipas) mengusulkan pemberian amnesti bagi warga binaan pemasyarakatan ...</t>
+        </is>
+      </c>
+      <c r="F1168" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1168" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688269/kemenimipas-usulkan-amnesti-warga-binaan-usia-produktif</t>
+        </is>
+      </c>
+      <c r="H1168" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000013001.jpg</t>
+        </is>
+      </c>
+      <c r="I1168" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>2 Tahun Hilang, Wanita di Sulsel Ternyata Dibunuh Sopir Travel-Dibuang ke Jurang</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:25:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1169" t="inlineStr">
+        <is>
+          <t>Agung Pramono</t>
+        </is>
+      </c>
+      <c r="E1169" t="inlineStr">
+        <is>
+          <t>Kasus hilangnya Paramita Titania Angelica terungkap. Mita dibunuh sopir travel, Alber, yang membuang jasadnya ke jurang.</t>
+        </is>
+      </c>
+      <c r="F1169" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1169" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612969/2-tahun-hilang-wanita-di-sulsel-ternyata-dibunuh-sopir-travel-dibuang-ke-jurang</t>
+        </is>
+      </c>
+      <c r="H1169" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/11/24/gadis-asal-wajo-paramitha-titania-anggelica-alias-mita-26-sudah-4-bulan-hilang_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1169" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>Area Pondok Cabe Udik Tangsel Mati Listrik Sejak Sore, PLN Ungkap Penyebabnya</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:51:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1170" t="inlineStr">
+        <is>
+          <t>Matius Alfons Hutajulu</t>
+        </is>
+      </c>
+      <c r="E1170" t="inlineStr">
+        <is>
+          <t>Kelurahan Pondok Cabe Udik mengalami mati listrik sejak sore. PLN sedang perbaikan jaringan dan berupaya mengembalikan pasokan listrik secepatnya.</t>
+        </is>
+      </c>
+      <c r="F1170" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1170" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612951/area-pondok-cabe-udik-tangsel-mati-listrik-sejak-sore-pln-ungkap-penyebabnya</t>
+        </is>
+      </c>
+      <c r="H1170" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2019/08/05/13d53a89-ea1b-48d3-8905-0df8d290609a_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1170" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>Periksa Istri Bos BlueRay, KPK Dalami Bukti Transfer ke Pejabat Bea Cukai</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:22:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1171" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1171" t="inlineStr">
+        <is>
+          <t>KPK memeriksa Vina Purnamasari, istri bos PT BlueRay Cargo, terkait kasus korupsi di Ditjen Bea Cukai. Penyidikan melibatkan tersangka baru Gatot Heroe.</t>
+        </is>
+      </c>
+      <c r="F1171" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1171" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612922/periksa-istri-bos-blueray-kpk-dalami-bukti-transfer-ke-pejabat-bea-cukai</t>
+        </is>
+      </c>
+      <c r="H1171" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/30/plt-direktur-penyidikan-kpk-achmad-taufik-husein-di-gedung-kpk-kuningan-jakarta-kamis-3072026-1785396044650_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1171" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>Gunung Picung Cianjur Kebakaran, Warga Duga karena Pembakaran Sampah</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:08:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr">
+        <is>
+          <t>Ikbal Slamet</t>
+        </is>
+      </c>
+      <c r="E1172" t="inlineStr">
+        <is>
+          <t>Kebakaran lahan di Gunung Picung, Cianjur, diduga akibat pembakaran sampah. Petugas kesulitan memadamkan api karena akses yang sulit.</t>
+        </is>
+      </c>
+      <c r="F1172" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1172" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612914/gunung-picung-cianjur-kebakaran-warga-duga-karena-pembakaran-sampah</t>
+        </is>
+      </c>
+      <c r="H1172" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/kebakaran-lahan-di-gunung-picung-cianjur-1786372838563_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1172" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>Kelakuan Sopir Taksi Cabuli Penumpang Berujung Mohon Ampunan</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:07:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E1173" t="inlineStr">
+        <is>
+          <t>Sopir taksi online ARA (54) ditangkap setelah mencabuli penumpang wanita di Jakarta Barat. Dia meminta ampun saat diserahkan ke polisi. Kasus ditangani PPA-PPO.</t>
+        </is>
+      </c>
+      <c r="F1173" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1173" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612913/kelakuan-sopir-taksi-cabuli-penumpang-berujung-mohon-ampunan</t>
+        </is>
+      </c>
+      <c r="H1173" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/12/17/ilustrasi-rawan-pelecehan-seksual-taksi-online_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1173" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>Kebakaran Dekat Stasiun Kampung Bandan yang Ganggu Arus KRL Dipicu Bara Rokok</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:33:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr">
+        <is>
+          <t>Jabbar Ramdhani</t>
+        </is>
+      </c>
+      <c r="E1174" t="inlineStr">
+        <is>
+          <t>Kebakaran di dekat Stasiun Kampung Bandan, Jakarta Utara, diduga akibat puntung rokok. Proses pemadaman selesai dalam 3 jam, arus KRL kini normal.</t>
+        </is>
+      </c>
+      <c r="F1174" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1174" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612898/kebakaran-dekat-stasiun-kampung-bandan-yang-ganggu-arus-krl-dipicu-bara-rokok</t>
+        </is>
+      </c>
+      <c r="H1174" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/kebakaran-alang-alang-terjadi-di-dekat-stasiun-kampung-bandan-jakarta-utara-jakut-perjalanan-kereta-rel-listrik-krl-sempat-ter-1786354296171_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1174" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>Kenneth DPRD DKI Bantu Siswa SMK Al-Irsyad Agar Kembali Belajar Tanpa Beban Biaya</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:28:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr">
+        <is>
+          <t>Mega Putra Ratya</t>
+        </is>
+      </c>
+      <c r="E1175" t="inlineStr">
+        <is>
+          <t>Anggota DPRD DKI Jakarta, Hardiyanto Kenneth, bantu lunasi tunggakan administrasi dan seragam siswa SMK Al-Irsyad. Ia dorong masyarakat peduli pendidikan.</t>
+        </is>
+      </c>
+      <c r="F1175" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1175" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612893/kenneth-dprd-dki-bantu-siswa-smk-al-irsyad-agar-kembali-belajar-tanpa-beban-biaya</t>
+        </is>
+      </c>
+      <c r="H1175" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/kenneth-dprd-dki-bantu-siswa-smk-al-irsyad-agar-kembali-belajar-tanpa-beban-biaya-1786372089822.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1175" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>K3 MPR RI Beri Rekomendasi Evaluasi Implementasi Konstitusi-Tata Kelola SDA</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:20:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1176" t="inlineStr">
+        <is>
+          <t>Moch. Prima Fauzi</t>
+        </is>
+      </c>
+      <c r="E1176" t="inlineStr">
+        <is>
+          <t>K3 MPR RI menyusun rekomendasi strategis untuk evaluasi implementasi konstitusi di bidang otonomi daerah, demokrasi ekonomi, dan pengelolaan sumber daya alam.</t>
+        </is>
+      </c>
+      <c r="F1176" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1176" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612886/k3-mpr-ri-beri-rekomendasi-evaluasi-implementasi-konstitusi-tata-kelola-sda</t>
+        </is>
+      </c>
+      <c r="H1176" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/mpr-ri-1786371584505_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1176" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>Lestari Moerdijat Dorong Reformasi Budaya Sekolah dan Kesejahteraan Guru</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:18:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1177" t="inlineStr">
+        <is>
+          <t>Akfa Nasrulhak</t>
+        </is>
+      </c>
+      <c r="E1177" t="inlineStr">
+        <is>
+          <t>Wakil Ketua MPR Lestari Moerdijat menekankan pentingnya kesejahteraan guru dan tata kelola pendidikan untuk menciptakan sekolah yang aman dan nyaman bagi siswa.</t>
+        </is>
+      </c>
+      <c r="F1177" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1177" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612883/lestari-moerdijat-dorong-reformasi-budaya-sekolah-dan-kesejahteraan-guru</t>
+        </is>
+      </c>
+      <c r="H1177" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/10/28/wakil-ketua-mpr-ri-lestari-moerdijat-1761654592023_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1177" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>ASN Bandung Barat Terancam Kena PHK gegara Live TikTok Bahas Fee Proyek</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:12:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1178" t="inlineStr">
+        <is>
+          <t>Whisnu Pradana</t>
+        </is>
+      </c>
+      <c r="E1178" t="inlineStr">
+        <is>
+          <t>Indah Yusuvia, ASN di Bandung Barat, mendapat kecaman setelah live TikTok saat jam kerja. Ia terancam PHK setelah pemeriksaan oleh Inspektorat KBB.</t>
+        </is>
+      </c>
+      <c r="F1178" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1178" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612879/asn-bandung-barat-terancam-kena-phk-gegara-live-tiktok-bahas-fee-proyek</t>
+        </is>
+      </c>
+      <c r="H1178" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/asn-kbb-yang-melakukan-live-tiktok-saat-jam-kerja-minta-maaf-1786272528570_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1178" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>Intel Cari Modal Rp 266 Triliun demi Genjot Bisnis AI</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:43:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E1179" t="inlineStr">
+        <is>
+          <t>Intel mengumumkan penawaran saham senilai US$ 15 miliar atau Rp 266,76 triliun (kurs Rp 17.784).</t>
+        </is>
+      </c>
+      <c r="F1179" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1179" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8612936/intel-cari-modal-rp-266-triliun-demi-genjot-bisnis-ai</t>
+        </is>
+      </c>
+      <c r="H1179" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/09/04/intel-core-ultra-lunar-lake_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1179" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>Menko Polkam Pastikan Asap Kebakaran Hutan di Indonesia Belum Ganggu Negara Tetangga</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:26:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1180" t="inlineStr">
+        <is>
+          <t>TribunNews.com menyajikan berita dan video terkini dari regional, nasional dan internasional dengan sudut pandang dan nilai-nilai lokal</t>
+        </is>
+      </c>
+      <c r="F1180" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1180" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/</t>
+        </is>
+      </c>
+      <c r="H1180" t="inlineStr">
+        <is>
+          <t>https://asset-2.tribunnews.com/tribunnews/foto/bank/images/logo-tribunnews1_20160901_101844.jpg</t>
+        </is>
+      </c>
+      <c r="I1180" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>Poslabfor Cek DNA hingga Barang Terkait Senjata di Yayasan Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:34:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1181" t="inlineStr">
+        <is>
+          <t>Dalam pemeriksaan tersebut, petugas menemukan 30 item.</t>
+        </is>
+      </c>
+      <c r="F1181" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1181" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266639/poslabfor-cek-dna-hingga-barang-terkait-senjata-di-yayasan-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H1181" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/ETTDU2qEXOzAfRQOJ_Mo1H87TaE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9317518/original/012310700_1786017988-Bungker.webp</t>
+        </is>
+      </c>
+      <c r="I1181" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>Kebakaran Dekat Stasiun Kampung Bandan Diduga Akibat Rokok, KRL Terganggu</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:25:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1182" t="inlineStr">
+        <is>
+          <t>Kebakaran tersebut sempat mengganggu perjalanan Commuter Line relasi Tanjung Priok-Jakarta Kota.</t>
+        </is>
+      </c>
+      <c r="F1182" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1182" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266638/kebakaran-dekat-stasiun-kampung-bandan-diduga-akibat-rokok-krl-terganggu</t>
+        </is>
+      </c>
+      <c r="H1182" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/YWJtbokY5rHQCWY7GjDLRGPOUjo=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320737/original/079815200_1786378545-IMG_4802.jpeg</t>
+        </is>
+      </c>
+      <c r="I1182" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>Bigmo Usai Dicecar 40 Pertanyaan: Sangat Kapok</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:07:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1183" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1183" t="inlineStr">
+        <is>
+          <t>Bigmo juga meminta maaf atas kegaduhan yang ditimbulkan akibat livestreamingnya.</t>
+        </is>
+      </c>
+      <c r="F1183" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1183" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266634/bigmo-usai-dicecar-40-pertanyaan-sangat-kapok</t>
+        </is>
+      </c>
+      <c r="H1183" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/yMyvLcWzAHymwzftNQDkQrdSxmo=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320662/original/029781800_1786364749-71851.jpg</t>
+        </is>
+      </c>
+      <c r="I1183" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>Ruangan Bekas Simpan 995 Airsoft Gun di Sekolah Swasta Jaksel Akan Dipakai Kegiatan Belajar</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:45:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1184" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1184" t="inlineStr">
+        <is>
+          <t>Ruangan bekas penyimpanan ratusan senjata api dan airsoft gun di sekolah swasta Kebayoran Lama sterilized. Akan dibersihkan dan dipakai KBM.</t>
+        </is>
+      </c>
+      <c r="F1184" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1184" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/10/23431041/ruangan-bekas-simpan-995-airsoft-gun-di-sekolah-swasta-jaksel-akan</t>
+        </is>
+      </c>
+      <c r="H1184" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/sMNCYEQLxPOgZz8Tu7fMxsETD_E=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/10/6a79cb0478fef.jpeg</t>
+        </is>
+      </c>
+      <c r="I1184" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>Transjakarta Akan Layani Rute Kepulauan Seribu, Apakah Pakai Bus? Ini Penjelasannya</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:45:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1185" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1185" t="inlineStr">
+        <is>
+          <t>Transjakarta akan kelola transportasi ke Kepulauan Seribu mulai 2027. Modanya bukan bus, melainkan kapal atau angkutan perairan.</t>
+        </is>
+      </c>
+      <c r="F1185" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1185" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/10/22151481/transjakarta-akan-layani-rute-kepulauan-seribu-apakah-pakai-bus-ini</t>
+        </is>
+      </c>
+      <c r="H1185" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/WIiKfpR36LdiI1OwHvC6_fBUfb8=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/02/06/6985ab6f6b80e.jpeg</t>
+        </is>
+      </c>
+      <c r="I1185" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>Hype</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>Bigmo Mengaku Tak Ada Niat Eksploitasi Anak untuk Promosikan Vape</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:45:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1186" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1186" t="inlineStr">
+        <is>
+          <t>Kreator Bigmo diperiksa polisi atas dugaan eksploitasi anak untuk promosi vape. Ia mengakui salah dan berjanji lebih bijak. Kanal YouTube-nya dicabut monetisasinya.</t>
+        </is>
+      </c>
+      <c r="F1186" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1186" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/hype/read/2026/08/10/214122666/bigmo-mengaku-tak-ada-niat-eksploitasi-anak-untuk-promosikan-vape</t>
+        </is>
+      </c>
+      <c r="H1186" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/OI31En78bK8vEsBJTiUbTaGfeEg=/0x0:4000x2667/1200x675/filters:watermark(data/photo/2026/01/30/697c8191ee571.png,0,-0,1)/data/photo/2026/04/13/69dcc68baa116.jpg</t>
+        </is>
+      </c>
+      <c r="I1186" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1140"/>
+  <autoFilter ref="A1:I1186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 17:46 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1186</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1196</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1186"/>
+  <dimension ref="A1:I1196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -56181,8 +56181,478 @@
         </is>
       </c>
     </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>Legislator DKI minta Pemda perkuat perlindungan siswa kurang mampu</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:58:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1187" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1187" t="inlineStr">
+        <is>
+          <t>Anggota DPRD DKI Jakarta Hardiyanto Kenneth meminta agar pemerintah daerah (Pemda) memperkuat kebijakan ...</t>
+        </is>
+      </c>
+      <c r="F1187" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1187" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688359/legislator-dki-minta-pemda-perkuat-perlindungan-siswa-kurang-mampu</t>
+        </is>
+      </c>
+      <c r="H1187" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/IMG_20260810_233505.jpg</t>
+        </is>
+      </c>
+      <c r="I1187" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>KBRI Tunis soroti pentingnya nilai historis, revolusioner, jelang HUT</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:57:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1188" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1188" t="inlineStr">
+        <is>
+          <t>Kedutaan Besar Republik Indonesia di Tunis, Tunisia, menyoroti pentingnya nilai historis dan revolusioner saat memulai ...</t>
+        </is>
+      </c>
+      <c r="F1188" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1188" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688355/kbri-tunis-soroti-pentingnya-nilai-historis-revolusioner-jelang-hut</t>
+        </is>
+      </c>
+      <c r="H1188" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000683003.jpg</t>
+        </is>
+      </c>
+      <c r="I1188" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>DPRD Sulteng desak hak 1.900 pekerja GNI terdampak PHK dipenuhi</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:56:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1189" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1189" t="inlineStr">
+        <is>
+          <t>DPRD Sulawesi Tengah meminta PT Gunbuster Nickel Industry (GNI) untuk memastikan pemenuhan hak sekitar 1.900 pekerja ...</t>
+        </is>
+      </c>
+      <c r="F1189" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1189" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688351/dprd-sulteng-desak-hak-1900-pekerja-gni-terdampak-phk-dipenuhi</t>
+        </is>
+      </c>
+      <c r="H1189" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/02/08/IMG_20230208_155148.jpg</t>
+        </is>
+      </c>
+      <c r="I1189" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>MK dengarkan keterangan Polri dan KPK terkait uji materiil KUHP</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:48:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1190" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1190" t="inlineStr">
+        <is>
+          <t>Sembilan hakim Mahkamah Konstitusi (MK) melanjutkan sidang uji materiil Undang-Undang Nomor 1 Tahun 2023 tentang KUHP ...</t>
+        </is>
+      </c>
+      <c r="F1190" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1190" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688345/mk-dengarkan-keterangan-polri-dan-kpk-terkait-uji-materiil-kuhp</t>
+        </is>
+      </c>
+      <c r="H1190" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000013002.jpg</t>
+        </is>
+      </c>
+      <c r="I1190" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>KPK Temukan Kasus Pemerasan Lain Dilakukan Eks Staf KPK yang Peras Bupati</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:46:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1191" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1191" t="inlineStr">
+        <is>
+          <t>KPK menemukan berkas terkait dugaan pemerasan oleh mantan stafnya, Setya Budi Dias, dan ayahnya. Penyidikan berlanjut untuk mengungkap kasus lebih dalam.</t>
+        </is>
+      </c>
+      <c r="F1191" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1191" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8612977/kpk-temukan-kasus-pemerasan-lain-dilakukan-eks-staf-kpk-yang-peras-bupati</t>
+        </is>
+      </c>
+      <c r="H1191" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/03/02/gedung-baru-kpk-2_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1191" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>2 Pria Ditangkap Buntut Unggahan Pidato Prabowo Soal Nuklir Iran, Gun Romli: Pemerintah Represif</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:44:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1192" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1192" t="inlineStr">
+        <is>
+          <t>Gun Romli menegaskan, penangkapan AYP dan AF terkait unggahan pidato Prabowo soal nuklir Iran justru mencederai kebebasan berpendapat.</t>
+        </is>
+      </c>
+      <c r="F1192" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1192" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866577/2-pria-ditangkap-buntut-unggahan-pidato-prabowo-soal-nuklir-iran-gun-romli-pemerintah-represif</t>
+        </is>
+      </c>
+      <c r="H1192" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0iL7xMX-_zskwBZCe2XRTCl1Bzs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/prabowo-kadin-dks.jpg</t>
+        </is>
+      </c>
+      <c r="I1192" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>10 Provinsi dengan PHK Terbanyak dan Terendah Januari-Juli 2026</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:14:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1193" t="inlineStr">
+        <is>
+          <t>Sejak Januari-Juli 2026, sekitar 43.805 pekerja terkena PHK, terbanyak di Jabar, terendah di Gorontalo.</t>
+        </is>
+      </c>
+      <c r="F1193" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1193" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866576/10-provinsi-dengan-phk-terbanyak-dan-terendah-januari-juli-2026</t>
+        </is>
+      </c>
+      <c r="H1193" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/C4q8OaWhwWglosa5Ry9IFpBZvdM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PHK-di-Jatim565.jpg</t>
+        </is>
+      </c>
+      <c r="I1193" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>Pengacara Khariq Anhar: Tuntutan “Timpa Teks” Bisa Batasi Hak Sipil di Medsos</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:05:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1194" t="inlineStr">
+        <is>
+          <t>Tuntutan enam bulan penjara terhadap Khariq dinilai berpotensi membatasi hak sipil dalam bermedia sosial dan menyampaikan kritik.</t>
+        </is>
+      </c>
+      <c r="F1194" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1194" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866575/pengacara-khariq-anhar-tuntutan-timpa-teks-bisa-batasi-hak-sipil-di-medsos</t>
+        </is>
+      </c>
+      <c r="H1194" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8fRftMALcqsKVRKz4f9OCapaRjA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Terdakwa-Khariq-Anhar-kuasa-hukum-usai-sidang-tuntutan-kasus-timpa-teks.jpg</t>
+        </is>
+      </c>
+      <c r="I1194" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>Dokter Ungkap Syarat Donor hingga Tantangan Transplantasi Ginjal di Indonesia</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:02:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1195" t="inlineStr">
+        <is>
+          <t>Transplantasi ginjal bukan sekadar mengganti organ yang mengalami kerusakan. Prosedur ini membutuhkan rangkaian  panjang.</t>
+        </is>
+      </c>
+      <c r="F1195" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1195" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866574/dokter-ungkap-syarat-donor-hingga-tantangantransplantasi-ginjal-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H1195" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/7hnsWcKbwnmteHzQ26LP4-GB7CA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/psien-gagal-ginjal.jpg</t>
+        </is>
+      </c>
+      <c r="I1195" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>KPK Panggil Ulang Rudy Tanoesoedibjo Selasa Besok Terkait Kasus Korupsi Bansos</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:51:53 +0700</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1196" t="inlineStr">
+        <is>
+          <t>KPK menjadwalkan ulang pemeriksaan terhadap Komisaris Utama PT DNR Logistik, Bambang Rudijanto Tanoesoedibjo alias Rudy Tanoe pada Selasa besok.</t>
+        </is>
+      </c>
+      <c r="F1196" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1196" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866573/kpk-panggil-ulang-rudy-tanoesoedibjo-selasa-besok-terkait-kasus-korupsi-bansos</t>
+        </is>
+      </c>
+      <c r="H1196" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/NiicxNmUufN85Wh9ihQ-pd6jyww=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Juru-Bicara-KPK-Budi-Prasetyo-302901.jpg</t>
+        </is>
+      </c>
+      <c r="I1196" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1186"/>
+  <autoFilter ref="A1:I1196"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 19:52 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1319</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1337</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1319"/>
+  <dimension ref="A1:I1337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -62432,8 +62432,854 @@
         </is>
       </c>
     </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>FOTO: Taiwan Gelar Latihan Perang Akbar Siap-siap Hadapi China</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>REUTERS</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>Taiwan kembali menggelar latihan militer besar-besaran demi menghadapi ancaman China yang masih berupaya menjegal keinginan Taipei untuk merdeka.</t>
+        </is>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1320" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810141039-115-1390585/foto-taiwan-gelar-latihan-perang-akbar-siap-siap-hadapi-china</t>
+        </is>
+      </c>
+      <c r="H1320" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/10/china-mengancam-taiwan-gelar-latihan-perang-akbar-1786345630376_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1320" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>Calon Senat Muslim AS Ejek Trump usai Disebut Tukang Bual</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>Calon senator Muslim Amerika Serikat dari Partai Demokrat Abdul El Sayed mengejek balik Presiden Donald Trump usai disebut tukang bual.</t>
+        </is>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1321" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810203049-134-1390779/calon-senat-muslim-as-ejek-trump-usai-disebut-tukang-bual</t>
+        </is>
+      </c>
+      <c r="H1321" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/politikus-demokrat-abdul-el-sayed-1785992947567_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1321" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>FOTO: TKP Penembakan Pejabat Daerah Thailand Gegara Utang</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:10:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>Seorang mantan anggota parlemen Thailand menembak mati seorang pejabat pemerintah daerah pada Senin (10/8) siang bolong akibat masalah utang.</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1322" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810183129-108-1390732/foto-tkp-penembakan-pejabat-daerah-thailand-gegara-utang</t>
+        </is>
+      </c>
+      <c r="H1322" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/10/eks-anggota-parlemen-diduga-tembak-mati-pejabat-thai-1786361386492_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1322" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>2 Penembakan dalam Sepekan, Bagaimana Aturan Senjata di Thailand?</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 20:35:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>Penembakan kembali terjadi di Bangkok, Thailand, saat eks anggota parlemen Chalong Riewran menembak mati seorang pejabat pemerintah daerah di siang bolong.</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1323" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810191131-106-1390747/2-penembakan-dalam-sepekan-bagaimana-aturan-senjata-di-thailand</t>
+        </is>
+      </c>
+      <c r="H1323" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/07/28/penembakan-massal-di-chatuchak-bangkok-thailand-1753694963803_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1323" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>Gempa M 7,4 Guncang Kolombia</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 20:01:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>Gempa berkekuatan magnitude 7,4 mengguncang Kolombia pada Senin (10/8).</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1324" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810194244-134-1390765/gempa-m-74-guncang-kolombia</t>
+        </is>
+      </c>
+      <c r="H1324" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2019/11/16/1a6c82e7-a220-416f-89ca-d0bf27b2dd6b_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1324" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>Malaysia Ungkap Penyebab PM Anwar Ibrahim Masuk RS</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 20:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>Perdana Menteri Malaysia Anwar Ibrahim menjalani operasi di rumah sakit pada Senin (10/8).</t>
+        </is>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1325" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810192837-106-1390755/malaysia-ungkap-penyebab-pm-anwar-ibrahim-masuk-rs</t>
+        </is>
+      </c>
+      <c r="H1325" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/11/05/anwar-ibrahim-1762331055170_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1325" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>Terbongkar Istri Netanyahu Digugat Gegara Sering Kasar dan Hina Staf ART</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>Istri PM Israel Benjamin Netanyahu, Sara Netanyahu, telah menghadapi tuduhan kekerasan terhadap staf rumah tangga, jelang pemilu pada Oktober mendatang.</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1326" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810184252-120-1390744/terbongkar-istri-netanyahu-digugat-gegara-sering-kasar-hina-staf-art</t>
+        </is>
+      </c>
+      <c r="H1326" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/10/sara-netanyahu-istri-dari-pm-israel-benjamin-netanyahu-1786359982783_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1326" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>Kata-kata Menohok Iran soal Pakta Baru Saudi, Pakistan, Turki Bak NATO</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>Iran buka suara usai Turki, Arab Saudi, dan Pakistan menandatangani perjanjian serupa NATO, Pakta Pertahanan Makkah, pada pekan lalu.</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1327" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810181327-120-1390731/kata-kata-menohok-iran-soal-pakta-baru-saudi-pakistan-turki-bak-nato</t>
+        </is>
+      </c>
+      <c r="H1327" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/04/06/iran-israel-conflict-1775454871064_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1327" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>Ratusan Warga di Ceuta Demo Tuntut Solusi Krisis Migrasi</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 18:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>REUTERS/RadioTelevision Ceuta</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>Ratusan warga Ceuta menggelar aksi demonstrasi menuntut solusi atas krisis migrasi pada Minggu (9/8).</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1328" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810074934-139-1390420/ratusan-warga-di-ceuta-demo-tuntut-solusi-krisis-migrasi</t>
+        </is>
+      </c>
+      <c r="H1328" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/10/ratusan-warga-di-ceuta-demo-tuntut-solusi-krisis-migrasi-1786325135454_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1328" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>Israel Larang Turis dan Peziarah Kunjungi Desa Kristen Palestina</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>Militer Israel semakin keji dengan menutup Desa Taybeh yang mayoritas penduduknya beragama Kristen di Tepi Barat, Palestina.</t>
+        </is>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1329" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810164254-120-1390696/israel-larang-turis-peziarah-kunjungi-desa-kristen-palestina</t>
+        </is>
+      </c>
+      <c r="H1329" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/10/desa-taybeh-yerusalem-palestina-1786355805645_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1329" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>Eks Anggota DPR Thailand Tembak Mati Pejabat Gegara Utang</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:21:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>Seorang mantan anggota parlemen Thailand menembak mati seorang pejabat pemerintah daerah pada Senin (10/8) siang bolong akibat masalah utang.</t>
+        </is>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1330" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810170010-106-1390707/eks-anggota-dpr-thailand-tembak-mati-pejabat-gegara-utang</t>
+        </is>
+      </c>
+      <c r="H1330" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/09/04/ilustrasi-penembakan-1756966587846_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1330" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>Houthi Klaim Serang Kilang Minyak Aramco Saudi, Picu Kebakaran</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 17:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1331" t="inlineStr">
+        <is>
+          <t>Kelompok milisi Yaman Houthi mengeklaim telah melancarkan serangan ke pusat kilang minyak Aramco di Kota Jizan, pada Minggu (9/10).</t>
+        </is>
+      </c>
+      <c r="F1331" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1331" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810145606-120-1390637/houthi-klaim-serang-kilang-minyak-aramco-saudi-picu-kebakaran</t>
+        </is>
+      </c>
+      <c r="H1331" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/10/iran-crisissaudi-1786349731672_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1331" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>Pilot Bawa Ekstasi ke RI, Malaysia Akui Screening Bandara Banyak Celah</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 16:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>Menteri Dalam Negeri Malaysia mengakui pemeriksaan barang di Bandara Internasional Kuala Lumpur (KLIA) tidak fokus mendeteksi barang selundupan seperti narkoba.</t>
+        </is>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1332" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810152025-106-1390685/pilot-bawa-ekstasi-ke-ri-malaysia-akui-screening-bandara-banyak-celah</t>
+        </is>
+      </c>
+      <c r="H1332" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/08/21/bandara-internasional-kuala-lumpur-1755751783753_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1332" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>Senator AS: Trump Sudah Kalah di Perang Iran</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 16:25:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>Senator Amerika Serikat asal Partai Demokrat, Chris Murphy, menyebut bahwa Presiden Donald Trump sudah 'kalah' dalam perang melawan Iran.</t>
+        </is>
+      </c>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1333" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810144221-134-1390634/senator-as-trump-sudah-kalah-di-perang-iran</t>
+        </is>
+      </c>
+      <c r="H1333" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/23/trump-kesulitan-lindungi-50-ribu-tentara-as-dari-serangan-iran-1784792922025_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1333" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>China Mulai Lirik Aliansi Baru Bak NATO antara Turki, Saudi, Pakistan</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 15:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>China disebut mulai melirik Pakta Pertahanan Makkah, aliansi pertahanan bak NATO, yang baru disepakati Turki, Arab Saudi, dan Pakistan.</t>
+        </is>
+      </c>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1334" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810141606-113-1390594/china-mulai-lirik-aliansi-baru-bak-nato-antara-turki-saudi-pakistan</t>
+        </is>
+      </c>
+      <c r="H1334" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/05/14/menteri-luar-negeri-china-wang-yi-1778750923688_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1334" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>Mojtaba Khamenei Muncul dalam Video Terbaru yang Dirilis Media Iran</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 15:20:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>Kantor berita semi-resmi Iran, Mehr, pada Sabtu (8/8) merilis video Pemimpin Tertinggi Iran Mojtaba Khamenei sedang berdiskusi dengan sejumlah orang.</t>
+        </is>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1335" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810143516-124-1390612/mojtaba-khamenei-muncul-dalam-video-terbaru-yang-dirilis-media-iran</t>
+        </is>
+      </c>
+      <c r="H1335" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/10/thumbnail-video-1786347574732_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1335" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>Mojtaba Khamenei Muncul ke Publik Lewat Video Bertemu Presiden Iran</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 15:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>Pertemuan Mojtaba Khamenei dan Presiden Masoud Pezeshkian pada Minggu (9/8) menjadi pertama kalinya sang Pemimpin Tertinggi Iran muncul ke publik.</t>
+        </is>
+      </c>
+      <c r="F1336" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1336" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810131527-120-1390557/mojtaba-khamenei-muncul-ke-publik-lewat-video-bertemu-presiden-iran</t>
+        </is>
+      </c>
+      <c r="H1336" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/03/11/mojtaba-khamenei-1773222923893_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1336" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>Menteri Malaysia: Scanner Bandara Kami Canggih, Bisa Deteksi Narkoba</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 14:25:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>Mendagri Malaysia, Saifuddin Nasution Ismail, memastikan mesin scanner yang berada di Bandara KLIA sepenuhnya mampu mendeteksi barang terlarang seperti narkoba.</t>
+        </is>
+      </c>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1337" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810121542-106-1390525/menteri-malaysia-scanner-bandara-kami-canggih-bisa-deteksi-narkoba</t>
+        </is>
+      </c>
+      <c r="H1337" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/08/21/bandara-internasional-kuala-lumpur-1755751783753_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1337" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1319"/>
+  <autoFilter ref="A1:I1337"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 21:35 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1337</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1341</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1337"/>
+  <dimension ref="A1:I1341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -63278,8 +63278,196 @@
         </is>
       </c>
     </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>Penertiban Tambang Ilegal Jadi Katalis Produksi dan Kinerja TINS</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:18:03 +0700</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>Penertiban tambang ilegal dapat meningkatkan produksi PT Timah Tbk (TINS). Kinerja keuangan TINS membaik dengan laba bersih melonjak 805% pada semester I 2026.</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1338" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810211236-17-758105/penertiban-tambang-ilegal-jadi-katalis-produksi-dan-kinerja-tins</t>
+        </is>
+      </c>
+      <c r="H1338" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/08/25/timah-balok-siap-jual-cnbc-indonesiafirda-dwi-muliawati-1756098257383_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1338" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>Literasi dan Inklusi Keuangan Syariah Nasional Turun, Ini Penyebabnya</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 21:05:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>Zefanya Aprilia</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>Survei Nasional Literasi dan Inklusi Keuangan (SNLIK) 2026 mencatat adanya penurunan tingkat literasi dan inklusi keuangan syariah.</t>
+        </is>
+      </c>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1339" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810204935-17-758096/literasi-dan-inklusi-keuangan-syariah-nasional-turun-ini-penyebabnya</t>
+        </is>
+      </c>
+      <c r="H1339" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/02/09/kepala-bps-amalia-a-widyasanti-dalam-rapat-konsultasi-dengan-pimpinan-komisi-dpr-ri-di-komplek-parlemen-jakarta-senin-922026-1770606395422_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1339" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>Destry Damayanti Jadi Calon Tunggal Gubernur BI, Ini Kata Bos LPS</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 20:45:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1340" t="inlineStr">
+        <is>
+          <t>Lembaga Penjamin Simpanan (LPS) buka suara mengenai pencalonan tunggal Destry Damayanti sebagai Gubernur Bank Indonesia (BI).</t>
+        </is>
+      </c>
+      <c r="F1340" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1340" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810203918-17-758095/destry-damayanti-jadi-calon-tunggal-gubernur-bi-ini-kata-bos-lps</t>
+        </is>
+      </c>
+      <c r="H1340" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/03/ketua-dewan-komisioner-lps-anggito-abimanyu-saat-konferensi-pers-hasil-rapat-berskla-kssk-iii-tahun-2016-di-jakarta-senin-3820-1785749402657_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1340" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>OJK Buka Suara Soal Wakaf Saham di Istiqlal</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 19:50:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1341" t="inlineStr">
+        <is>
+          <t>OJK membahas integrasi Masjid Istiqlal dalam ekosistem BEI melalui wakaf saham.</t>
+        </is>
+      </c>
+      <c r="F1341" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1341" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260810153342-17-757997/ojk-buka-suara-soal-wakaf-saham-di-istiqlal</t>
+        </is>
+      </c>
+      <c r="H1341" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/03/26/ilustrasi-ojk-cnbc-indonesiafaisal-rahman_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1341" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1337"/>
+  <autoFilter ref="A1:I1341"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 00:49 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1341</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1342</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1341"/>
+  <dimension ref="A1:I1342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -63466,8 +63466,55 @@
         </is>
       </c>
     </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>BSMR: Bank Tak Cukup Hanya Canggih, Ketahanan Hadapi Risiko Jadi Kunci</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>Budi Raharjo</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Dunia perbankan kini menghadapi tantangan yang tidak lagi hanya datang dari naik-turunnya ekonomi. Kemajuan kecerdasan buatan (AI), ancaman kejahatan siber, hingga hadirnya layanan bullion banking atau bank...</t>
+        </is>
+      </c>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1342" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjkx32415/bsmr-bank-tak-cukup-hanya-canggih-ketahanan-hadapi-risiko-jadi-kunci</t>
+        </is>
+      </c>
+      <c r="H1342" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/the-jakarta-risk-management-convention-jrmc-2026-di-jakarta_260811072251-521.jpeg</t>
+        </is>
+      </c>
+      <c r="I1342" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1341"/>
+  <autoFilter ref="A1:I1342"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 06:49 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-10.xlsx
+++ b/data/berita_2026-08-10.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1342</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1346</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1342"/>
+  <dimension ref="A1:I1346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -63513,8 +63513,196 @@
         </is>
       </c>
     </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>Olah TKP Sekolah Jaksel, Polisi Kembali Temukan Senjata hingga Amunisi</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:45:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>Polres Metro Jakarta Selatan melakukan olah TKP di sekolah swasta Pondok Pinang, menemukan ratusan senjata dan narkoba. Penyelidikan berlanjut.</t>
+        </is>
+      </c>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1343" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260810222520-12-1390810/olah-tkp-sekolah-jaksel-polisi-kembali-temukan-senjata-hingga-amunisi</t>
+        </is>
+      </c>
+      <c r="H1343" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/ratusan-senjata-di-yayasan-sekolah-jaksel-1786100090384_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1343" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>KPK Sebut Dedi Congor Sudah Jadi Tersangka di Kortas Tipidkor Polri</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 23:15:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr">
+        <is>
+          <t>KPK menetapkan Ahmad Dedi, mantan Kepala KPPBC Marunda, sebagai tersangka dalam kasus dugaan korupsi. Ia diduga menerima Rp30 miliar dari Blueray Cargo.</t>
+        </is>
+      </c>
+      <c r="F1344" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1344" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260810222135-12-1390809/kpk-sebut-dedi-congor-sudah-jadi-tersangka-di-kortas-tipidkor-polri</t>
+        </is>
+      </c>
+      <c r="H1344" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/06/12/pengungkapan-suap-audit-laporan-keuangan-di-kabupaten-muara-enim-1781244746815_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1344" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>Karhutla Kepung RI, Menko Polkam hingga Istana Keluarkan Imbauan</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:30:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1345" t="inlineStr">
+        <is>
+          <t>Menko Polkam hingga Istana mengeluarkan sejumlah imbauan terkait kebakaran hutan dan lahan (Karhutla) yang terus meluas.</t>
+        </is>
+      </c>
+      <c r="F1345" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1345" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260810184104-20-1390740/karhutla-kepung-ri-menko-polkam-hingga-istana-keluarkan-imbauan</t>
+        </is>
+      </c>
+      <c r="H1345" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/pemadaman-kebakaran-kawasan-hutan-di-boyolali-1785974493169_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1345" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>Kuasa Hukum Bigmo: Konten Promosi Vape Libatkan Anak Terjadi Spontan</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>Mon, 10 Aug 2026 22:15:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1346" t="inlineStr">
+        <is>
+          <t>Youtuber Bigmo diperiksa terkait dugaan promosi liquid vape kepada anak-anak. Ia meminta maaf dan berkomitmen untuk membuat konten yang lebih positif.</t>
+        </is>
+      </c>
+      <c r="F1346" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1346" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260810201549-12-1390776/kuasa-hukum-bigmo-konten-promosi-vape-libatkan-anak-terjadi-spontan</t>
+        </is>
+      </c>
+      <c r="H1346" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/10/bigmo-memenuhi-panggilan-polda-metro-jaya-1786345392788_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1346" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1342"/>
+  <autoFilter ref="A1:I1346"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>